<commit_message>
H.8 page: Deposit Pricing section (FDIC national rates via FRED, betas, spreads, quarter-end table)
</commit_message>
<xml_diff>
--- a/data/h8-growth5y.xlsx
+++ b/data/h8-growth5y.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="EOP" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Average" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="EOP" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Average" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>

</xml_diff>

<commit_message>
H.8 tile: add full Fed SLOOS detail (standards, demand, willingness; charts, latest table, CSV)
</commit_message>
<xml_diff>
--- a/data/h8-growth5y.xlsx
+++ b/data/h8-growth5y.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="EOP" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Average" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="EOP" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Average" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>

</xml_diff>

<commit_message>
data: refresh 2026-10-14 15:49 UTC
</commit_message>
<xml_diff>
--- a/data/h8-growth5y.xlsx
+++ b/data/h8-growth5y.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="EOP" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Average" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="EOP" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Average" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>

</xml_diff>

<commit_message>
data: refresh 2026-10-16 23:42 UTC
</commit_message>
<xml_diff>
--- a/data/h8-growth5y.xlsx
+++ b/data/h8-growth5y.xlsx
@@ -418,7 +418,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:CG60"/>
+  <dimension ref="A1:CK60"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -847,6 +847,26 @@
           <t>Q3 2026 EOP week</t>
         </is>
       </c>
+      <c r="CH1" s="1" t="inlineStr">
+        <is>
+          <t>Q4 2026 QTD level ($bn)</t>
+        </is>
+      </c>
+      <c r="CI1" s="1" t="inlineStr">
+        <is>
+          <t>Q4 2026 QTD YoY %</t>
+        </is>
+      </c>
+      <c r="CJ1" s="1" t="inlineStr">
+        <is>
+          <t>Q4 2026 QTD LQA %</t>
+        </is>
+      </c>
+      <c r="CK1" s="1" t="inlineStr">
+        <is>
+          <t>Q4 2026 QTD EOP week</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -1141,17 +1161,31 @@
         </is>
       </c>
       <c r="CD2" t="n">
-        <v>12696.91</v>
+        <v>12707.3</v>
       </c>
       <c r="CE2" t="n">
-        <v>6.84</v>
+        <v>6.93</v>
       </c>
       <c r="CF2" t="n">
-        <v>6.62</v>
+        <v>6.97</v>
       </c>
       <c r="CG2" t="inlineStr">
         <is>
           <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="CH2" t="n">
+        <v>12751.96</v>
+      </c>
+      <c r="CI2" t="n">
+        <v>5.74</v>
+      </c>
+      <c r="CJ2" t="n">
+        <v>1.41</v>
+      </c>
+      <c r="CK2" t="inlineStr">
+        <is>
+          <t>2026-10-07</t>
         </is>
       </c>
     </row>
@@ -1448,17 +1482,31 @@
         </is>
       </c>
       <c r="CD3" t="n">
-        <v>2336.53</v>
+        <v>2337.26</v>
       </c>
       <c r="CE3" t="n">
-        <v>8.19</v>
+        <v>8.23</v>
       </c>
       <c r="CF3" t="n">
-        <v>8.66</v>
+        <v>8.800000000000001</v>
       </c>
       <c r="CG3" t="inlineStr">
         <is>
           <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="CH3" t="n">
+        <v>2359.03</v>
+      </c>
+      <c r="CI3" t="n">
+        <v>9.369999999999999</v>
+      </c>
+      <c r="CJ3" t="n">
+        <v>3.78</v>
+      </c>
+      <c r="CK3" t="inlineStr">
+        <is>
+          <t>2026-10-07</t>
         </is>
       </c>
     </row>
@@ -1755,17 +1803,31 @@
         </is>
       </c>
       <c r="CD4" t="n">
-        <v>3018.12</v>
+        <v>3024.68</v>
       </c>
       <c r="CE4" t="n">
-        <v>3.57</v>
+        <v>3.8</v>
       </c>
       <c r="CF4" t="n">
-        <v>3.89</v>
+        <v>4.8</v>
       </c>
       <c r="CG4" t="inlineStr">
         <is>
           <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="CH4" t="n">
+        <v>3031.84</v>
+      </c>
+      <c r="CI4" t="n">
+        <v>3</v>
+      </c>
+      <c r="CJ4" t="n">
+        <v>0.95</v>
+      </c>
+      <c r="CK4" t="inlineStr">
+        <is>
+          <t>2026-10-07</t>
         </is>
       </c>
     </row>
@@ -2062,17 +2124,31 @@
         </is>
       </c>
       <c r="CD5" t="n">
-        <v>432.92</v>
+        <v>434.08</v>
       </c>
       <c r="CE5" t="n">
-        <v>-1.42</v>
+        <v>-1.15</v>
       </c>
       <c r="CF5" t="n">
-        <v>7.29</v>
+        <v>8.449999999999999</v>
       </c>
       <c r="CG5" t="inlineStr">
         <is>
           <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="CH5" t="n">
+        <v>436.16</v>
+      </c>
+      <c r="CI5" t="n">
+        <v>0.61</v>
+      </c>
+      <c r="CJ5" t="n">
+        <v>1.93</v>
+      </c>
+      <c r="CK5" t="inlineStr">
+        <is>
+          <t>2026-10-07</t>
         </is>
       </c>
     </row>
@@ -2369,17 +2445,31 @@
         </is>
       </c>
       <c r="CD6" t="n">
-        <v>122.85</v>
+        <v>123.39</v>
       </c>
       <c r="CE6" t="n">
-        <v>4.59</v>
+        <v>5.06</v>
       </c>
       <c r="CF6" t="n">
-        <v>4.31</v>
+        <v>6.17</v>
       </c>
       <c r="CG6" t="inlineStr">
         <is>
           <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="CH6" t="n">
+        <v>123.51</v>
+      </c>
+      <c r="CI6" t="n">
+        <v>3.82</v>
+      </c>
+      <c r="CJ6" t="n">
+        <v>0.37</v>
+      </c>
+      <c r="CK6" t="inlineStr">
+        <is>
+          <t>2026-10-07</t>
         </is>
       </c>
     </row>
@@ -2676,17 +2766,31 @@
         </is>
       </c>
       <c r="CD7" t="n">
-        <v>619.89</v>
+        <v>621.4400000000001</v>
       </c>
       <c r="CE7" t="n">
-        <v>4.34</v>
+        <v>4.6</v>
       </c>
       <c r="CF7" t="n">
-        <v>1.81</v>
+        <v>2.83</v>
       </c>
       <c r="CG7" t="inlineStr">
         <is>
           <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="CH7" t="n">
+        <v>624.29</v>
+      </c>
+      <c r="CI7" t="n">
+        <v>3.12</v>
+      </c>
+      <c r="CJ7" t="n">
+        <v>1.85</v>
+      </c>
+      <c r="CK7" t="inlineStr">
+        <is>
+          <t>2026-10-07</t>
         </is>
       </c>
     </row>
@@ -2983,17 +3087,31 @@
         </is>
       </c>
       <c r="CD8" t="n">
-        <v>1842.46</v>
+        <v>1845.77</v>
       </c>
       <c r="CE8" t="n">
-        <v>4.49</v>
+        <v>4.67</v>
       </c>
       <c r="CF8" t="n">
-        <v>3.79</v>
+        <v>4.54</v>
       </c>
       <c r="CG8" t="inlineStr">
         <is>
           <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="CH8" t="n">
+        <v>1847.88</v>
+      </c>
+      <c r="CI8" t="n">
+        <v>3.49</v>
+      </c>
+      <c r="CJ8" t="n">
+        <v>0.46</v>
+      </c>
+      <c r="CK8" t="inlineStr">
+        <is>
+          <t>2026-10-07</t>
         </is>
       </c>
     </row>
@@ -3290,17 +3408,31 @@
         </is>
       </c>
       <c r="CD9" t="n">
-        <v>2694.35</v>
+        <v>2697.46</v>
       </c>
       <c r="CE9" t="n">
-        <v>1.38</v>
+        <v>1.49</v>
       </c>
       <c r="CF9" t="n">
-        <v>-0.12</v>
+        <v>0.34</v>
       </c>
       <c r="CG9" t="inlineStr">
         <is>
           <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="CH9" t="n">
+        <v>2695.85</v>
+      </c>
+      <c r="CI9" t="n">
+        <v>0.89</v>
+      </c>
+      <c r="CJ9" t="n">
+        <v>-0.24</v>
+      </c>
+      <c r="CK9" t="inlineStr">
+        <is>
+          <t>2026-10-07</t>
         </is>
       </c>
     </row>
@@ -3597,17 +3729,31 @@
         </is>
       </c>
       <c r="CD10" t="n">
-        <v>2403.88</v>
+        <v>2406.4</v>
       </c>
       <c r="CE10" t="n">
-        <v>0.82</v>
+        <v>0.93</v>
       </c>
       <c r="CF10" t="n">
-        <v>-0.96</v>
+        <v>-0.54</v>
       </c>
       <c r="CG10" t="inlineStr">
         <is>
           <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="CH10" t="n">
+        <v>2404.5</v>
+      </c>
+      <c r="CI10" t="n">
+        <v>0.42</v>
+      </c>
+      <c r="CJ10" t="n">
+        <v>-0.32</v>
+      </c>
+      <c r="CK10" t="inlineStr">
+        <is>
+          <t>2026-10-07</t>
         </is>
       </c>
     </row>
@@ -3904,17 +4050,31 @@
         </is>
       </c>
       <c r="CD11" t="n">
-        <v>290.47</v>
+        <v>291.06</v>
       </c>
       <c r="CE11" t="n">
-        <v>6.2</v>
+        <v>6.41</v>
       </c>
       <c r="CF11" t="n">
-        <v>7.14</v>
+        <v>8.01</v>
       </c>
       <c r="CG11" t="inlineStr">
         <is>
           <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="CH11" t="n">
+        <v>291.34</v>
+      </c>
+      <c r="CI11" t="n">
+        <v>4.96</v>
+      </c>
+      <c r="CJ11" t="n">
+        <v>0.39</v>
+      </c>
+      <c r="CK11" t="inlineStr">
+        <is>
+          <t>2026-10-07</t>
         </is>
       </c>
     </row>
@@ -4211,17 +4371,31 @@
         </is>
       </c>
       <c r="CD12" t="n">
-        <v>1927.84</v>
+        <v>1927.73</v>
       </c>
       <c r="CE12" t="n">
-        <v>4.96</v>
+        <v>4.95</v>
       </c>
       <c r="CF12" t="n">
-        <v>5.14</v>
+        <v>5.12</v>
       </c>
       <c r="CG12" t="inlineStr">
         <is>
           <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="CH12" t="n">
+        <v>1935.67</v>
+      </c>
+      <c r="CI12" t="n">
+        <v>4.16</v>
+      </c>
+      <c r="CJ12" t="n">
+        <v>1.66</v>
+      </c>
+      <c r="CK12" t="inlineStr">
+        <is>
+          <t>2026-10-07</t>
         </is>
       </c>
     </row>
@@ -4518,7 +4692,7 @@
         </is>
       </c>
       <c r="CD13" t="n">
-        <v>1096.39</v>
+        <v>1096.38</v>
       </c>
       <c r="CE13" t="n">
         <v>4.27</v>
@@ -4529,6 +4703,20 @@
       <c r="CG13" t="inlineStr">
         <is>
           <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="CH13" t="n">
+        <v>1104.06</v>
+      </c>
+      <c r="CI13" t="n">
+        <v>3.82</v>
+      </c>
+      <c r="CJ13" t="n">
+        <v>2.83</v>
+      </c>
+      <c r="CK13" t="inlineStr">
+        <is>
+          <t>2026-10-07</t>
         </is>
       </c>
     </row>
@@ -4825,17 +5013,31 @@
         </is>
       </c>
       <c r="CD14" t="n">
-        <v>831.45</v>
+        <v>831.35</v>
       </c>
       <c r="CE14" t="n">
-        <v>5.89</v>
+        <v>5.88</v>
       </c>
       <c r="CF14" t="n">
-        <v>7.78</v>
+        <v>7.73</v>
       </c>
       <c r="CG14" t="inlineStr">
         <is>
           <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="CH14" t="n">
+        <v>831.61</v>
+      </c>
+      <c r="CI14" t="n">
+        <v>4.61</v>
+      </c>
+      <c r="CJ14" t="n">
+        <v>0.13</v>
+      </c>
+      <c r="CK14" t="inlineStr">
+        <is>
+          <t>2026-10-07</t>
         </is>
       </c>
     </row>
@@ -5132,17 +5334,31 @@
         </is>
       </c>
       <c r="CD15" t="n">
-        <v>524.47</v>
+        <v>524.4299999999999</v>
       </c>
       <c r="CE15" t="n">
         <v>5.65</v>
       </c>
       <c r="CF15" t="n">
-        <v>5.13</v>
+        <v>5.09</v>
       </c>
       <c r="CG15" t="inlineStr">
         <is>
           <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="CH15" t="n">
+        <v>524.4</v>
+      </c>
+      <c r="CI15" t="n">
+        <v>3.81</v>
+      </c>
+      <c r="CJ15" t="n">
+        <v>-0.02</v>
+      </c>
+      <c r="CK15" t="inlineStr">
+        <is>
+          <t>2026-10-07</t>
         </is>
       </c>
     </row>
@@ -5439,17 +5655,31 @@
         </is>
       </c>
       <c r="CD16" t="n">
-        <v>2720.07</v>
+        <v>2720.18</v>
       </c>
       <c r="CE16" t="n">
         <v>17.45</v>
       </c>
       <c r="CF16" t="n">
-        <v>16.51</v>
+        <v>16.53</v>
       </c>
       <c r="CG16" t="inlineStr">
         <is>
           <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="CH16" t="n">
+        <v>2729.57</v>
+      </c>
+      <c r="CI16" t="n">
+        <v>12.37</v>
+      </c>
+      <c r="CJ16" t="n">
+        <v>1.39</v>
+      </c>
+      <c r="CK16" t="inlineStr">
+        <is>
+          <t>2026-10-07</t>
         </is>
       </c>
     </row>
@@ -5746,17 +5976,31 @@
         </is>
       </c>
       <c r="CD17" t="n">
-        <v>1547.37</v>
+        <v>1547.48</v>
       </c>
       <c r="CE17" t="n">
         <v>22.46</v>
       </c>
       <c r="CF17" t="n">
-        <v>22.16</v>
+        <v>22.2</v>
       </c>
       <c r="CG17" t="inlineStr">
         <is>
           <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="CH17" t="n">
+        <v>1559.17</v>
+      </c>
+      <c r="CI17" t="n">
+        <v>14.43</v>
+      </c>
+      <c r="CJ17" t="n">
+        <v>3.06</v>
+      </c>
+      <c r="CK17" t="inlineStr">
+        <is>
+          <t>2026-10-07</t>
         </is>
       </c>
     </row>
@@ -6053,17 +6297,31 @@
         </is>
       </c>
       <c r="CD18" t="n">
-        <v>18088.12</v>
+        <v>18089.39</v>
       </c>
       <c r="CE18" t="n">
-        <v>6.27</v>
+        <v>6.28</v>
       </c>
       <c r="CF18" t="n">
-        <v>4.92</v>
+        <v>4.95</v>
       </c>
       <c r="CG18" t="inlineStr">
         <is>
           <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="CH18" t="n">
+        <v>18129.3</v>
+      </c>
+      <c r="CI18" t="n">
+        <v>5.59</v>
+      </c>
+      <c r="CJ18" t="n">
+        <v>0.89</v>
+      </c>
+      <c r="CK18" t="inlineStr">
+        <is>
+          <t>2026-10-07</t>
         </is>
       </c>
     </row>
@@ -6360,17 +6618,31 @@
         </is>
       </c>
       <c r="CD19" t="n">
-        <v>1653.14</v>
+        <v>1654.15</v>
       </c>
       <c r="CE19" t="n">
-        <v>7.25</v>
+        <v>7.32</v>
       </c>
       <c r="CF19" t="n">
-        <v>8.890000000000001</v>
+        <v>9.16</v>
       </c>
       <c r="CG19" t="inlineStr">
         <is>
           <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="CH19" t="n">
+        <v>1662.12</v>
+      </c>
+      <c r="CI19" t="n">
+        <v>5.07</v>
+      </c>
+      <c r="CJ19" t="n">
+        <v>1.94</v>
+      </c>
+      <c r="CK19" t="inlineStr">
+        <is>
+          <t>2026-10-07</t>
         </is>
       </c>
     </row>
@@ -6667,17 +6939,31 @@
         </is>
       </c>
       <c r="CD20" t="n">
-        <v>16434.97</v>
+        <v>16435.24</v>
       </c>
       <c r="CE20" t="n">
         <v>6.17</v>
       </c>
       <c r="CF20" t="n">
-        <v>4.53</v>
+        <v>4.54</v>
       </c>
       <c r="CG20" t="inlineStr">
         <is>
           <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="CH20" t="n">
+        <v>16467.18</v>
+      </c>
+      <c r="CI20" t="n">
+        <v>5.64</v>
+      </c>
+      <c r="CJ20" t="n">
+        <v>0.78</v>
+      </c>
+      <c r="CK20" t="inlineStr">
+        <is>
+          <t>2026-10-07</t>
         </is>
       </c>
     </row>
@@ -6987,6 +7273,20 @@
           <t>2026-09-30</t>
         </is>
       </c>
+      <c r="CH21" t="n">
+        <v>7983.45</v>
+      </c>
+      <c r="CI21" t="n">
+        <v>6.49</v>
+      </c>
+      <c r="CJ21" t="n">
+        <v>1.48</v>
+      </c>
+      <c r="CK21" t="inlineStr">
+        <is>
+          <t>2026-10-07</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -7294,6 +7594,20 @@
           <t>2026-09-30</t>
         </is>
       </c>
+      <c r="CH22" t="n">
+        <v>1616.81</v>
+      </c>
+      <c r="CI22" t="n">
+        <v>11.08</v>
+      </c>
+      <c r="CJ22" t="n">
+        <v>5.06</v>
+      </c>
+      <c r="CK22" t="inlineStr">
+        <is>
+          <t>2026-10-07</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -7601,6 +7915,20 @@
           <t>2026-09-30</t>
         </is>
       </c>
+      <c r="CH23" t="n">
+        <v>915.78</v>
+      </c>
+      <c r="CI23" t="n">
+        <v>2.71</v>
+      </c>
+      <c r="CJ23" t="n">
+        <v>1.44</v>
+      </c>
+      <c r="CK23" t="inlineStr">
+        <is>
+          <t>2026-10-07</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -7908,6 +8236,20 @@
           <t>2026-09-30</t>
         </is>
       </c>
+      <c r="CH24" t="n">
+        <v>125.77</v>
+      </c>
+      <c r="CI24" t="n">
+        <v>-1.55</v>
+      </c>
+      <c r="CJ24" t="n">
+        <v>2.38</v>
+      </c>
+      <c r="CK24" t="inlineStr">
+        <is>
+          <t>2026-10-07</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -8215,6 +8557,20 @@
           <t>2026-09-30</t>
         </is>
       </c>
+      <c r="CH25" t="n">
+        <v>6.26</v>
+      </c>
+      <c r="CI25" t="n">
+        <v>-2.61</v>
+      </c>
+      <c r="CJ25" t="n">
+        <v>-6.6</v>
+      </c>
+      <c r="CK25" t="inlineStr">
+        <is>
+          <t>2026-10-07</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -8522,6 +8878,20 @@
           <t>2026-09-30</t>
         </is>
       </c>
+      <c r="CH26" t="n">
+        <v>255.22</v>
+      </c>
+      <c r="CI26" t="n">
+        <v>5.45</v>
+      </c>
+      <c r="CJ26" t="n">
+        <v>3.35</v>
+      </c>
+      <c r="CK26" t="inlineStr">
+        <is>
+          <t>2026-10-07</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -8829,6 +9199,20 @@
           <t>2026-09-30</t>
         </is>
       </c>
+      <c r="CH27" t="n">
+        <v>528.52</v>
+      </c>
+      <c r="CI27" t="n">
+        <v>2.55</v>
+      </c>
+      <c r="CJ27" t="n">
+        <v>0.42</v>
+      </c>
+      <c r="CK27" t="inlineStr">
+        <is>
+          <t>2026-10-07</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -9136,6 +9520,20 @@
           <t>2026-09-30</t>
         </is>
       </c>
+      <c r="CH28" t="n">
+        <v>1656.65</v>
+      </c>
+      <c r="CI28" t="n">
+        <v>-0.11</v>
+      </c>
+      <c r="CJ28" t="n">
+        <v>-0.71</v>
+      </c>
+      <c r="CK28" t="inlineStr">
+        <is>
+          <t>2026-10-07</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -9443,6 +9841,20 @@
           <t>2026-09-30</t>
         </is>
       </c>
+      <c r="CH29" t="n">
+        <v>1495.27</v>
+      </c>
+      <c r="CI29" t="n">
+        <v>-0.35</v>
+      </c>
+      <c r="CJ29" t="n">
+        <v>-0.8100000000000001</v>
+      </c>
+      <c r="CK29" t="inlineStr">
+        <is>
+          <t>2026-10-07</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -9750,6 +10162,20 @@
           <t>2026-09-30</t>
         </is>
       </c>
+      <c r="CH30" t="n">
+        <v>161.38</v>
+      </c>
+      <c r="CI30" t="n">
+        <v>2.22</v>
+      </c>
+      <c r="CJ30" t="n">
+        <v>0.17</v>
+      </c>
+      <c r="CK30" t="inlineStr">
+        <is>
+          <t>2026-10-07</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -10057,6 +10483,20 @@
           <t>2026-09-30</t>
         </is>
       </c>
+      <c r="CH31" t="n">
+        <v>1583.32</v>
+      </c>
+      <c r="CI31" t="n">
+        <v>2.88</v>
+      </c>
+      <c r="CJ31" t="n">
+        <v>-0.73</v>
+      </c>
+      <c r="CK31" t="inlineStr">
+        <is>
+          <t>2026-10-07</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -10364,6 +10804,20 @@
           <t>2026-09-30</t>
         </is>
       </c>
+      <c r="CH32" t="n">
+        <v>1000.63</v>
+      </c>
+      <c r="CI32" t="n">
+        <v>3.64</v>
+      </c>
+      <c r="CJ32" t="n">
+        <v>-0.79</v>
+      </c>
+      <c r="CK32" t="inlineStr">
+        <is>
+          <t>2026-10-07</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -10671,6 +11125,20 @@
           <t>2026-09-30</t>
         </is>
       </c>
+      <c r="CH33" t="n">
+        <v>582.6900000000001</v>
+      </c>
+      <c r="CI33" t="n">
+        <v>1.59</v>
+      </c>
+      <c r="CJ33" t="n">
+        <v>-0.62</v>
+      </c>
+      <c r="CK33" t="inlineStr">
+        <is>
+          <t>2026-10-07</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -10978,6 +11446,20 @@
           <t>2026-09-30</t>
         </is>
       </c>
+      <c r="CH34" t="n">
+        <v>436.32</v>
+      </c>
+      <c r="CI34" t="n">
+        <v>2</v>
+      </c>
+      <c r="CJ34" t="n">
+        <v>-0.53</v>
+      </c>
+      <c r="CK34" t="inlineStr">
+        <is>
+          <t>2026-10-07</t>
+        </is>
+      </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -11285,6 +11767,20 @@
           <t>2026-09-30</t>
         </is>
       </c>
+      <c r="CH35" t="n">
+        <v>2210.88</v>
+      </c>
+      <c r="CI35" t="n">
+        <v>13.26</v>
+      </c>
+      <c r="CJ35" t="n">
+        <v>2.21</v>
+      </c>
+      <c r="CK35" t="inlineStr">
+        <is>
+          <t>2026-10-07</t>
+        </is>
+      </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -11592,6 +12088,20 @@
           <t>2026-09-30</t>
         </is>
       </c>
+      <c r="CH36" t="n">
+        <v>1358.51</v>
+      </c>
+      <c r="CI36" t="n">
+        <v>14.97</v>
+      </c>
+      <c r="CJ36" t="n">
+        <v>4.19</v>
+      </c>
+      <c r="CK36" t="inlineStr">
+        <is>
+          <t>2026-10-07</t>
+        </is>
+      </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
@@ -11899,6 +12409,20 @@
           <t>2026-09-30</t>
         </is>
       </c>
+      <c r="CH37" t="n">
+        <v>12441.01</v>
+      </c>
+      <c r="CI37" t="n">
+        <v>6.57</v>
+      </c>
+      <c r="CJ37" t="n">
+        <v>0.85</v>
+      </c>
+      <c r="CK37" t="inlineStr">
+        <is>
+          <t>2026-10-07</t>
+        </is>
+      </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -12206,6 +12730,20 @@
           <t>2026-09-30</t>
         </is>
       </c>
+      <c r="CH38" t="n">
+        <v>914.62</v>
+      </c>
+      <c r="CI38" t="n">
+        <v>9.300000000000001</v>
+      </c>
+      <c r="CJ38" t="n">
+        <v>-1.77</v>
+      </c>
+      <c r="CK38" t="inlineStr">
+        <is>
+          <t>2026-10-07</t>
+        </is>
+      </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
@@ -12513,6 +13051,20 @@
           <t>2026-09-30</t>
         </is>
       </c>
+      <c r="CH39" t="n">
+        <v>11526.39</v>
+      </c>
+      <c r="CI39" t="n">
+        <v>6.36</v>
+      </c>
+      <c r="CJ39" t="n">
+        <v>1.06</v>
+      </c>
+      <c r="CK39" t="inlineStr">
+        <is>
+          <t>2026-10-07</t>
+        </is>
+      </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
@@ -12807,17 +13359,31 @@
         </is>
       </c>
       <c r="CD40" t="n">
-        <v>4742.75</v>
+        <v>4753.14</v>
       </c>
       <c r="CE40" t="n">
-        <v>5.29</v>
+        <v>5.52</v>
       </c>
       <c r="CF40" t="n">
+        <v>5.42</v>
+      </c>
+      <c r="CG40" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="CH40" t="n">
+        <v>4768.51</v>
+      </c>
+      <c r="CI40" t="n">
         <v>4.5</v>
       </c>
-      <c r="CG40" t="inlineStr">
-        <is>
-          <t>2026-09-30</t>
+      <c r="CJ40" t="n">
+        <v>1.3</v>
+      </c>
+      <c r="CK40" t="inlineStr">
+        <is>
+          <t>2026-10-07</t>
         </is>
       </c>
     </row>
@@ -13114,17 +13680,31 @@
         </is>
       </c>
       <c r="CD41" t="n">
-        <v>739.54</v>
+        <v>740.26</v>
       </c>
       <c r="CE41" t="n">
-        <v>5.12</v>
+        <v>5.22</v>
       </c>
       <c r="CF41" t="n">
-        <v>5.55</v>
+        <v>5.96</v>
       </c>
       <c r="CG41" t="inlineStr">
         <is>
           <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="CH41" t="n">
+        <v>742.22</v>
+      </c>
+      <c r="CI41" t="n">
+        <v>5.81</v>
+      </c>
+      <c r="CJ41" t="n">
+        <v>1.06</v>
+      </c>
+      <c r="CK41" t="inlineStr">
+        <is>
+          <t>2026-10-07</t>
         </is>
       </c>
     </row>
@@ -13421,17 +14001,31 @@
         </is>
       </c>
       <c r="CD42" t="n">
-        <v>2105.61</v>
+        <v>2112.18</v>
       </c>
       <c r="CE42" t="n">
-        <v>3.57</v>
+        <v>3.89</v>
       </c>
       <c r="CF42" t="n">
-        <v>3.1</v>
+        <v>4.39</v>
       </c>
       <c r="CG42" t="inlineStr">
         <is>
           <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="CH42" t="n">
+        <v>2116.06</v>
+      </c>
+      <c r="CI42" t="n">
+        <v>3.13</v>
+      </c>
+      <c r="CJ42" t="n">
+        <v>0.74</v>
+      </c>
+      <c r="CK42" t="inlineStr">
+        <is>
+          <t>2026-10-07</t>
         </is>
       </c>
     </row>
@@ -13728,17 +14322,31 @@
         </is>
       </c>
       <c r="CD43" t="n">
-        <v>307.9</v>
+        <v>309.05</v>
       </c>
       <c r="CE43" t="n">
-        <v>-0.63</v>
+        <v>-0.26</v>
       </c>
       <c r="CF43" t="n">
-        <v>5.76</v>
+        <v>7.35</v>
       </c>
       <c r="CG43" t="inlineStr">
         <is>
           <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="CH43" t="n">
+        <v>310.39</v>
+      </c>
+      <c r="CI43" t="n">
+        <v>1.51</v>
+      </c>
+      <c r="CJ43" t="n">
+        <v>1.74</v>
+      </c>
+      <c r="CK43" t="inlineStr">
+        <is>
+          <t>2026-10-07</t>
         </is>
       </c>
     </row>
@@ -14035,17 +14643,31 @@
         </is>
       </c>
       <c r="CD44" t="n">
-        <v>116.48</v>
+        <v>117.02</v>
       </c>
       <c r="CE44" t="n">
-        <v>4.8</v>
+        <v>5.29</v>
       </c>
       <c r="CF44" t="n">
-        <v>3.27</v>
+        <v>5.22</v>
       </c>
       <c r="CG44" t="inlineStr">
         <is>
           <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="CH44" t="n">
+        <v>117.25</v>
+      </c>
+      <c r="CI44" t="n">
+        <v>4.19</v>
+      </c>
+      <c r="CJ44" t="n">
+        <v>0.76</v>
+      </c>
+      <c r="CK44" t="inlineStr">
+        <is>
+          <t>2026-10-07</t>
         </is>
       </c>
     </row>
@@ -14342,17 +14964,31 @@
         </is>
       </c>
       <c r="CD45" t="n">
-        <v>366.76</v>
+        <v>368.31</v>
       </c>
       <c r="CE45" t="n">
-        <v>2</v>
+        <v>2.43</v>
       </c>
       <c r="CF45" t="n">
-        <v>0.47</v>
+        <v>2.18</v>
       </c>
       <c r="CG45" t="inlineStr">
         <is>
           <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="CH45" t="n">
+        <v>369.07</v>
+      </c>
+      <c r="CI45" t="n">
+        <v>1.57</v>
+      </c>
+      <c r="CJ45" t="n">
+        <v>0.83</v>
+      </c>
+      <c r="CK45" t="inlineStr">
+        <is>
+          <t>2026-10-07</t>
         </is>
       </c>
     </row>
@@ -14649,17 +15285,31 @@
         </is>
       </c>
       <c r="CD46" t="n">
-        <v>1314.48</v>
+        <v>1317.8</v>
       </c>
       <c r="CE46" t="n">
-        <v>4.95</v>
+        <v>5.21</v>
       </c>
       <c r="CF46" t="n">
-        <v>3.22</v>
+        <v>4.27</v>
       </c>
       <c r="CG46" t="inlineStr">
         <is>
           <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="CH46" t="n">
+        <v>1319.36</v>
+      </c>
+      <c r="CI46" t="n">
+        <v>3.87</v>
+      </c>
+      <c r="CJ46" t="n">
+        <v>0.47</v>
+      </c>
+      <c r="CK46" t="inlineStr">
+        <is>
+          <t>2026-10-07</t>
         </is>
       </c>
     </row>
@@ -14956,17 +15606,31 @@
         </is>
       </c>
       <c r="CD47" t="n">
-        <v>1034.74</v>
+        <v>1037.86</v>
       </c>
       <c r="CE47" t="n">
-        <v>3.11</v>
+        <v>3.42</v>
       </c>
       <c r="CF47" t="n">
-        <v>1.14</v>
+        <v>2.36</v>
       </c>
       <c r="CG47" t="inlineStr">
         <is>
           <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="CH47" t="n">
+        <v>1039.2</v>
+      </c>
+      <c r="CI47" t="n">
+        <v>2.53</v>
+      </c>
+      <c r="CJ47" t="n">
+        <v>0.52</v>
+      </c>
+      <c r="CK47" t="inlineStr">
+        <is>
+          <t>2026-10-07</t>
         </is>
       </c>
     </row>
@@ -15263,17 +15927,31 @@
         </is>
       </c>
       <c r="CD48" t="n">
-        <v>905.58</v>
+        <v>908.1</v>
       </c>
       <c r="CE48" t="n">
-        <v>2.08</v>
+        <v>2.36</v>
       </c>
       <c r="CF48" t="n">
-        <v>-0.21</v>
+        <v>0.91</v>
       </c>
       <c r="CG48" t="inlineStr">
         <is>
           <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="CH48" t="n">
+        <v>909.23</v>
+      </c>
+      <c r="CI48" t="n">
+        <v>1.72</v>
+      </c>
+      <c r="CJ48" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="CK48" t="inlineStr">
+        <is>
+          <t>2026-10-07</t>
         </is>
       </c>
     </row>
@@ -15570,17 +16248,31 @@
         </is>
       </c>
       <c r="CD49" t="n">
-        <v>129.16</v>
+        <v>129.75</v>
       </c>
       <c r="CE49" t="n">
-        <v>10.93</v>
+        <v>11.44</v>
       </c>
       <c r="CF49" t="n">
-        <v>11.26</v>
+        <v>13.32</v>
       </c>
       <c r="CG49" t="inlineStr">
         <is>
           <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="CH49" t="n">
+        <v>129.96</v>
+      </c>
+      <c r="CI49" t="n">
+        <v>8.59</v>
+      </c>
+      <c r="CJ49" t="n">
+        <v>0.66</v>
+      </c>
+      <c r="CK49" t="inlineStr">
+        <is>
+          <t>2026-10-07</t>
         </is>
       </c>
     </row>
@@ -15877,17 +16569,31 @@
         </is>
       </c>
       <c r="CD50" t="n">
-        <v>341.62</v>
+        <v>341.51</v>
       </c>
       <c r="CE50" t="n">
-        <v>9.039999999999999</v>
+        <v>9</v>
       </c>
       <c r="CF50" t="n">
-        <v>15.23</v>
+        <v>15.07</v>
       </c>
       <c r="CG50" t="inlineStr">
         <is>
           <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="CH50" t="n">
+        <v>352.34</v>
+      </c>
+      <c r="CI50" t="n">
+        <v>10.32</v>
+      </c>
+      <c r="CJ50" t="n">
+        <v>13.31</v>
+      </c>
+      <c r="CK50" t="inlineStr">
+        <is>
+          <t>2026-10-07</t>
         </is>
       </c>
     </row>
@@ -16184,17 +16890,31 @@
         </is>
       </c>
       <c r="CD51" t="n">
-        <v>93.78</v>
+        <v>93.77</v>
       </c>
       <c r="CE51" t="n">
-        <v>-2.38</v>
+        <v>-2.39</v>
       </c>
       <c r="CF51" t="n">
-        <v>-5.09</v>
+        <v>-5.14</v>
       </c>
       <c r="CG51" t="inlineStr">
         <is>
           <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="CH51" t="n">
+        <v>103.43</v>
+      </c>
+      <c r="CI51" t="n">
+        <v>5.6</v>
+      </c>
+      <c r="CJ51" t="n">
+        <v>48.05</v>
+      </c>
+      <c r="CK51" t="inlineStr">
+        <is>
+          <t>2026-10-07</t>
         </is>
       </c>
     </row>
@@ -16491,17 +17211,31 @@
         </is>
       </c>
       <c r="CD52" t="n">
-        <v>247.84</v>
+        <v>247.74</v>
       </c>
       <c r="CE52" t="n">
-        <v>14.08</v>
+        <v>14.04</v>
       </c>
       <c r="CF52" t="n">
-        <v>24.31</v>
+        <v>24.11</v>
       </c>
       <c r="CG52" t="inlineStr">
         <is>
           <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="CH52" t="n">
+        <v>248.91</v>
+      </c>
+      <c r="CI52" t="n">
+        <v>12.41</v>
+      </c>
+      <c r="CJ52" t="n">
+        <v>1.91</v>
+      </c>
+      <c r="CK52" t="inlineStr">
+        <is>
+          <t>2026-10-07</t>
         </is>
       </c>
     </row>
@@ -16798,17 +17532,31 @@
         </is>
       </c>
       <c r="CD53" t="n">
-        <v>87.58</v>
+        <v>87.53</v>
       </c>
       <c r="CE53" t="n">
-        <v>14.76</v>
+        <v>14.7</v>
       </c>
       <c r="CF53" t="n">
-        <v>26.06</v>
+        <v>25.8</v>
       </c>
       <c r="CG53" t="inlineStr">
         <is>
           <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="CH53" t="n">
+        <v>88.08</v>
+      </c>
+      <c r="CI53" t="n">
+        <v>13.85</v>
+      </c>
+      <c r="CJ53" t="n">
+        <v>2.54</v>
+      </c>
+      <c r="CK53" t="inlineStr">
+        <is>
+          <t>2026-10-07</t>
         </is>
       </c>
     </row>
@@ -17105,17 +17853,31 @@
         </is>
       </c>
       <c r="CD54" t="n">
-        <v>521.23</v>
+        <v>521.34</v>
       </c>
       <c r="CE54" t="n">
-        <v>15.6</v>
+        <v>15.62</v>
       </c>
       <c r="CF54" t="n">
-        <v>9.06</v>
+        <v>9.15</v>
       </c>
       <c r="CG54" t="inlineStr">
         <is>
           <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="CH54" t="n">
+        <v>518.6900000000001</v>
+      </c>
+      <c r="CI54" t="n">
+        <v>8.75</v>
+      </c>
+      <c r="CJ54" t="n">
+        <v>-2.02</v>
+      </c>
+      <c r="CK54" t="inlineStr">
+        <is>
+          <t>2026-10-07</t>
         </is>
       </c>
     </row>
@@ -17412,17 +18174,31 @@
         </is>
       </c>
       <c r="CD55" t="n">
-        <v>202.72</v>
+        <v>202.83</v>
       </c>
       <c r="CE55" t="n">
-        <v>27.02</v>
+        <v>27.08</v>
       </c>
       <c r="CF55" t="n">
-        <v>6.12</v>
+        <v>6.34</v>
       </c>
       <c r="CG55" t="inlineStr">
         <is>
           <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="CH55" t="n">
+        <v>200.67</v>
+      </c>
+      <c r="CI55" t="n">
+        <v>10.84</v>
+      </c>
+      <c r="CJ55" t="n">
+        <v>-4.2</v>
+      </c>
+      <c r="CK55" t="inlineStr">
+        <is>
+          <t>2026-10-07</t>
         </is>
       </c>
     </row>
@@ -17719,17 +18495,31 @@
         </is>
       </c>
       <c r="CD56" t="n">
-        <v>5673.38</v>
+        <v>5674.65</v>
       </c>
       <c r="CE56" t="n">
-        <v>4.28</v>
+        <v>4.3</v>
       </c>
       <c r="CF56" t="n">
-        <v>2.05</v>
+        <v>2.14</v>
       </c>
       <c r="CG56" t="inlineStr">
         <is>
           <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="CH56" t="n">
+        <v>5688.29</v>
+      </c>
+      <c r="CI56" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="CJ56" t="n">
+        <v>0.96</v>
+      </c>
+      <c r="CK56" t="inlineStr">
+        <is>
+          <t>2026-10-07</t>
         </is>
       </c>
     </row>
@@ -18026,17 +18816,31 @@
         </is>
       </c>
       <c r="CD57" t="n">
-        <v>734.4299999999999</v>
+        <v>735.4400000000001</v>
       </c>
       <c r="CE57" t="n">
-        <v>0.29</v>
+        <v>0.43</v>
       </c>
       <c r="CF57" t="n">
-        <v>-1.25</v>
+        <v>-0.7</v>
       </c>
       <c r="CG57" t="inlineStr">
         <is>
           <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="CH57" t="n">
+        <v>747.5</v>
+      </c>
+      <c r="CI57" t="n">
+        <v>0.31</v>
+      </c>
+      <c r="CJ57" t="n">
+        <v>6.72</v>
+      </c>
+      <c r="CK57" t="inlineStr">
+        <is>
+          <t>2026-10-07</t>
         </is>
       </c>
     </row>
@@ -18333,17 +19137,31 @@
         </is>
       </c>
       <c r="CD58" t="n">
-        <v>4938.95</v>
+        <v>4939.21</v>
       </c>
       <c r="CE58" t="n">
         <v>4.9</v>
       </c>
       <c r="CF58" t="n">
-        <v>2.55</v>
+        <v>2.58</v>
       </c>
       <c r="CG58" t="inlineStr">
         <is>
           <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="CH58" t="n">
+        <v>4940.79</v>
+      </c>
+      <c r="CI58" t="n">
+        <v>4</v>
+      </c>
+      <c r="CJ58" t="n">
+        <v>0.13</v>
+      </c>
+      <c r="CK58" t="inlineStr">
+        <is>
+          <t>2026-10-07</t>
         </is>
       </c>
     </row>
@@ -18365,7 +19183,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:CG60"/>
+  <dimension ref="A1:CK60"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -18794,6 +19612,26 @@
           <t>Q3 2026 weeks in qtr</t>
         </is>
       </c>
+      <c r="CH1" s="1" t="inlineStr">
+        <is>
+          <t>Q4 2026 QTD level ($bn)</t>
+        </is>
+      </c>
+      <c r="CI1" s="1" t="inlineStr">
+        <is>
+          <t>Q4 2026 QTD YoY %</t>
+        </is>
+      </c>
+      <c r="CJ1" s="1" t="inlineStr">
+        <is>
+          <t>Q4 2026 QTD LQA %</t>
+        </is>
+      </c>
+      <c r="CK1" s="1" t="inlineStr">
+        <is>
+          <t>Q4 2026 QTD weeks in qtr</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -19050,16 +19888,28 @@
         <v>13</v>
       </c>
       <c r="CD2" t="n">
-        <v>12592.32</v>
+        <v>12594.27</v>
       </c>
       <c r="CE2" t="n">
-        <v>6.65</v>
+        <v>6.67</v>
       </c>
       <c r="CF2" t="n">
-        <v>5.64</v>
+        <v>5.7</v>
       </c>
       <c r="CG2" t="n">
         <v>14</v>
+      </c>
+      <c r="CH2" t="n">
+        <v>12751.96</v>
+      </c>
+      <c r="CI2" t="n">
+        <v>6.43</v>
+      </c>
+      <c r="CJ2" t="n">
+        <v>5.1</v>
+      </c>
+      <c r="CK2" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="3">
@@ -19317,16 +20167,28 @@
         <v>13</v>
       </c>
       <c r="CD3" t="n">
-        <v>2307.44</v>
+        <v>2307.6</v>
       </c>
       <c r="CE3" t="n">
-        <v>7.58</v>
+        <v>7.59</v>
       </c>
       <c r="CF3" t="n">
-        <v>7.42</v>
+        <v>7.45</v>
       </c>
       <c r="CG3" t="n">
         <v>14</v>
+      </c>
+      <c r="CH3" t="n">
+        <v>2359.03</v>
+      </c>
+      <c r="CI3" t="n">
+        <v>9.449999999999999</v>
+      </c>
+      <c r="CJ3" t="n">
+        <v>9.220000000000001</v>
+      </c>
+      <c r="CK3" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="4">
@@ -19584,16 +20446,28 @@
         <v>13</v>
       </c>
       <c r="CD4" t="n">
-        <v>3004.61</v>
+        <v>3005.76</v>
       </c>
       <c r="CE4" t="n">
-        <v>3.32</v>
+        <v>3.36</v>
       </c>
       <c r="CF4" t="n">
-        <v>3.65</v>
+        <v>3.81</v>
       </c>
       <c r="CG4" t="n">
         <v>14</v>
+      </c>
+      <c r="CH4" t="n">
+        <v>3031.84</v>
+      </c>
+      <c r="CI4" t="n">
+        <v>3.39</v>
+      </c>
+      <c r="CJ4" t="n">
+        <v>3.52</v>
+      </c>
+      <c r="CK4" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="5">
@@ -19851,16 +20725,28 @@
         <v>13</v>
       </c>
       <c r="CD5" t="n">
-        <v>431.42</v>
+        <v>431.62</v>
       </c>
       <c r="CE5" t="n">
-        <v>-2.13</v>
+        <v>-2.08</v>
       </c>
       <c r="CF5" t="n">
-        <v>3.13</v>
+        <v>3.32</v>
       </c>
       <c r="CG5" t="n">
         <v>14</v>
+      </c>
+      <c r="CH5" t="n">
+        <v>436.16</v>
+      </c>
+      <c r="CI5" t="n">
+        <v>0.24</v>
+      </c>
+      <c r="CJ5" t="n">
+        <v>4.27</v>
+      </c>
+      <c r="CK5" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="6">
@@ -20118,16 +21004,28 @@
         <v>13</v>
       </c>
       <c r="CD6" t="n">
-        <v>122.46</v>
+        <v>122.56</v>
       </c>
       <c r="CE6" t="n">
-        <v>4.31</v>
+        <v>4.39</v>
       </c>
       <c r="CF6" t="n">
-        <v>4.31</v>
+        <v>4.64</v>
       </c>
       <c r="CG6" t="n">
         <v>14</v>
+      </c>
+      <c r="CH6" t="n">
+        <v>123.51</v>
+      </c>
+      <c r="CI6" t="n">
+        <v>4.37</v>
+      </c>
+      <c r="CJ6" t="n">
+        <v>3.14</v>
+      </c>
+      <c r="CK6" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="7">
@@ -20385,16 +21283,28 @@
         <v>13</v>
       </c>
       <c r="CD7" t="n">
-        <v>617.99</v>
+        <v>618.25</v>
       </c>
       <c r="CE7" t="n">
-        <v>4.06</v>
+        <v>4.1</v>
       </c>
       <c r="CF7" t="n">
-        <v>1.97</v>
+        <v>2.14</v>
       </c>
       <c r="CG7" t="n">
         <v>14</v>
+      </c>
+      <c r="CH7" t="n">
+        <v>624.29</v>
+      </c>
+      <c r="CI7" t="n">
+        <v>3.6</v>
+      </c>
+      <c r="CJ7" t="n">
+        <v>3.97</v>
+      </c>
+      <c r="CK7" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="8">
@@ -20652,16 +21562,28 @@
         <v>13</v>
       </c>
       <c r="CD8" t="n">
-        <v>1832.74</v>
+        <v>1833.34</v>
       </c>
       <c r="CE8" t="n">
-        <v>4.38</v>
+        <v>4.41</v>
       </c>
       <c r="CF8" t="n">
-        <v>4.31</v>
+        <v>4.45</v>
       </c>
       <c r="CG8" t="n">
         <v>14</v>
+      </c>
+      <c r="CH8" t="n">
+        <v>1847.88</v>
+      </c>
+      <c r="CI8" t="n">
+        <v>4.02</v>
+      </c>
+      <c r="CJ8" t="n">
+        <v>3.21</v>
+      </c>
+      <c r="CK8" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="9">
@@ -20919,16 +21841,28 @@
         <v>13</v>
       </c>
       <c r="CD9" t="n">
-        <v>2696.11</v>
+        <v>2696.66</v>
       </c>
       <c r="CE9" t="n">
-        <v>1.62</v>
+        <v>1.64</v>
       </c>
       <c r="CF9" t="n">
-        <v>1.32</v>
+        <v>1.41</v>
       </c>
       <c r="CG9" t="n">
         <v>14</v>
+      </c>
+      <c r="CH9" t="n">
+        <v>2695.85</v>
+      </c>
+      <c r="CI9" t="n">
+        <v>1.08</v>
+      </c>
+      <c r="CJ9" t="n">
+        <v>-0.12</v>
+      </c>
+      <c r="CK9" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="10">
@@ -21186,16 +22120,28 @@
         <v>13</v>
       </c>
       <c r="CD10" t="n">
-        <v>2407.69</v>
+        <v>2408.14</v>
       </c>
       <c r="CE10" t="n">
-        <v>1.11</v>
+        <v>1.13</v>
       </c>
       <c r="CF10" t="n">
-        <v>0.59</v>
+        <v>0.66</v>
       </c>
       <c r="CG10" t="n">
         <v>14</v>
+      </c>
+      <c r="CH10" t="n">
+        <v>2404.5</v>
+      </c>
+      <c r="CI10" t="n">
+        <v>0.57</v>
+      </c>
+      <c r="CJ10" t="n">
+        <v>-0.6</v>
+      </c>
+      <c r="CK10" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="11">
@@ -21453,16 +22399,28 @@
         <v>13</v>
       </c>
       <c r="CD11" t="n">
-        <v>288.42</v>
+        <v>288.52</v>
       </c>
       <c r="CE11" t="n">
-        <v>6.06</v>
+        <v>6.1</v>
       </c>
       <c r="CF11" t="n">
-        <v>7.76</v>
+        <v>7.91</v>
       </c>
       <c r="CG11" t="n">
         <v>14</v>
+      </c>
+      <c r="CH11" t="n">
+        <v>291.34</v>
+      </c>
+      <c r="CI11" t="n">
+        <v>5.57</v>
+      </c>
+      <c r="CJ11" t="n">
+        <v>3.97</v>
+      </c>
+      <c r="CK11" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="12">
@@ -21720,16 +22678,28 @@
         <v>13</v>
       </c>
       <c r="CD12" t="n">
-        <v>1919.39</v>
+        <v>1919.37</v>
       </c>
       <c r="CE12" t="n">
-        <v>5.09</v>
+        <v>5.08</v>
       </c>
       <c r="CF12" t="n">
         <v>5.5</v>
       </c>
       <c r="CG12" t="n">
         <v>14</v>
+      </c>
+      <c r="CH12" t="n">
+        <v>1935.67</v>
+      </c>
+      <c r="CI12" t="n">
+        <v>4.64</v>
+      </c>
+      <c r="CJ12" t="n">
+        <v>3.44</v>
+      </c>
+      <c r="CK12" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="13">
@@ -21998,6 +22968,18 @@
       <c r="CG13" t="n">
         <v>14</v>
       </c>
+      <c r="CH13" t="n">
+        <v>1104.06</v>
+      </c>
+      <c r="CI13" t="n">
+        <v>4.27</v>
+      </c>
+      <c r="CJ13" t="n">
+        <v>5.2</v>
+      </c>
+      <c r="CK13" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -22254,16 +23236,28 @@
         <v>13</v>
       </c>
       <c r="CD14" t="n">
-        <v>829.24</v>
+        <v>829.22</v>
       </c>
       <c r="CE14" t="n">
         <v>6.43</v>
       </c>
       <c r="CF14" t="n">
-        <v>9.32</v>
+        <v>9.31</v>
       </c>
       <c r="CG14" t="n">
         <v>14</v>
+      </c>
+      <c r="CH14" t="n">
+        <v>831.61</v>
+      </c>
+      <c r="CI14" t="n">
+        <v>5.13</v>
+      </c>
+      <c r="CJ14" t="n">
+        <v>1.16</v>
+      </c>
+      <c r="CK14" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="15">
@@ -22521,16 +23515,28 @@
         <v>13</v>
       </c>
       <c r="CD15" t="n">
-        <v>524.11</v>
+        <v>524.1</v>
       </c>
       <c r="CE15" t="n">
         <v>6.29</v>
       </c>
       <c r="CF15" t="n">
-        <v>7</v>
+        <v>6.99</v>
       </c>
       <c r="CG15" t="n">
         <v>14</v>
+      </c>
+      <c r="CH15" t="n">
+        <v>524.4</v>
+      </c>
+      <c r="CI15" t="n">
+        <v>4.78</v>
+      </c>
+      <c r="CJ15" t="n">
+        <v>0.23</v>
+      </c>
+      <c r="CK15" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="16">
@@ -22788,16 +23794,28 @@
         <v>13</v>
       </c>
       <c r="CD16" t="n">
-        <v>2664.76</v>
+        <v>2664.87</v>
       </c>
       <c r="CE16" t="n">
-        <v>17.16</v>
+        <v>17.17</v>
       </c>
       <c r="CF16" t="n">
-        <v>11.11</v>
+        <v>11.13</v>
       </c>
       <c r="CG16" t="n">
         <v>14</v>
+      </c>
+      <c r="CH16" t="n">
+        <v>2729.57</v>
+      </c>
+      <c r="CI16" t="n">
+        <v>14.82</v>
+      </c>
+      <c r="CJ16" t="n">
+        <v>10.07</v>
+      </c>
+      <c r="CK16" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="17">
@@ -23055,16 +24073,28 @@
         <v>13</v>
       </c>
       <c r="CD17" t="n">
-        <v>1509.49</v>
+        <v>1509.57</v>
       </c>
       <c r="CE17" t="n">
-        <v>22.52</v>
+        <v>22.53</v>
       </c>
       <c r="CF17" t="n">
-        <v>10.43</v>
+        <v>10.45</v>
       </c>
       <c r="CG17" t="n">
         <v>14</v>
+      </c>
+      <c r="CH17" t="n">
+        <v>1559.17</v>
+      </c>
+      <c r="CI17" t="n">
+        <v>18.7</v>
+      </c>
+      <c r="CJ17" t="n">
+        <v>13.81</v>
+      </c>
+      <c r="CK17" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="18">
@@ -23322,16 +24352,28 @@
         <v>13</v>
       </c>
       <c r="CD18" t="n">
-        <v>17938.57</v>
+        <v>17939.06</v>
       </c>
       <c r="CE18" t="n">
-        <v>5.98</v>
+        <v>5.99</v>
       </c>
       <c r="CF18" t="n">
-        <v>4.56</v>
+        <v>4.57</v>
       </c>
       <c r="CG18" t="n">
         <v>14</v>
+      </c>
+      <c r="CH18" t="n">
+        <v>18129.3</v>
+      </c>
+      <c r="CI18" t="n">
+        <v>5.85</v>
+      </c>
+      <c r="CJ18" t="n">
+        <v>4.31</v>
+      </c>
+      <c r="CK18" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="19">
@@ -23589,16 +24631,28 @@
         <v>13</v>
       </c>
       <c r="CD19" t="n">
-        <v>1632.9</v>
+        <v>1633.07</v>
       </c>
       <c r="CE19" t="n">
-        <v>5.96</v>
+        <v>5.97</v>
       </c>
       <c r="CF19" t="n">
-        <v>-0.8</v>
+        <v>-0.76</v>
       </c>
       <c r="CG19" t="n">
         <v>14</v>
+      </c>
+      <c r="CH19" t="n">
+        <v>1662.12</v>
+      </c>
+      <c r="CI19" t="n">
+        <v>5.75</v>
+      </c>
+      <c r="CJ19" t="n">
+        <v>7.31</v>
+      </c>
+      <c r="CK19" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="20">
@@ -23856,7 +24910,7 @@
         <v>13</v>
       </c>
       <c r="CD20" t="n">
-        <v>16305.67</v>
+        <v>16306</v>
       </c>
       <c r="CE20" t="n">
         <v>5.99</v>
@@ -23866,6 +24920,18 @@
       </c>
       <c r="CG20" t="n">
         <v>14</v>
+      </c>
+      <c r="CH20" t="n">
+        <v>16467.18</v>
+      </c>
+      <c r="CI20" t="n">
+        <v>5.86</v>
+      </c>
+      <c r="CJ20" t="n">
+        <v>4.01</v>
+      </c>
+      <c r="CK20" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="21">
@@ -24134,6 +25200,18 @@
       <c r="CG21" t="n">
         <v>14</v>
       </c>
+      <c r="CH21" t="n">
+        <v>7983.45</v>
+      </c>
+      <c r="CI21" t="n">
+        <v>7.25</v>
+      </c>
+      <c r="CJ21" t="n">
+        <v>5.8</v>
+      </c>
+      <c r="CK21" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -24401,6 +25479,18 @@
       <c r="CG22" t="n">
         <v>14</v>
       </c>
+      <c r="CH22" t="n">
+        <v>1616.81</v>
+      </c>
+      <c r="CI22" t="n">
+        <v>11.22</v>
+      </c>
+      <c r="CJ22" t="n">
+        <v>11.35</v>
+      </c>
+      <c r="CK22" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -24668,6 +25758,18 @@
       <c r="CG23" t="n">
         <v>14</v>
       </c>
+      <c r="CH23" t="n">
+        <v>915.78</v>
+      </c>
+      <c r="CI23" t="n">
+        <v>3.15</v>
+      </c>
+      <c r="CJ23" t="n">
+        <v>4.53</v>
+      </c>
+      <c r="CK23" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -24935,6 +26037,18 @@
       <c r="CG24" t="n">
         <v>14</v>
       </c>
+      <c r="CH24" t="n">
+        <v>125.77</v>
+      </c>
+      <c r="CI24" t="n">
+        <v>-1.14</v>
+      </c>
+      <c r="CJ24" t="n">
+        <v>4.52</v>
+      </c>
+      <c r="CK24" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -25202,6 +26316,18 @@
       <c r="CG25" t="n">
         <v>14</v>
       </c>
+      <c r="CH25" t="n">
+        <v>6.26</v>
+      </c>
+      <c r="CI25" t="n">
+        <v>-2.12</v>
+      </c>
+      <c r="CJ25" t="n">
+        <v>-1.13</v>
+      </c>
+      <c r="CK25" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -25469,6 +26595,18 @@
       <c r="CG26" t="n">
         <v>14</v>
       </c>
+      <c r="CH26" t="n">
+        <v>255.22</v>
+      </c>
+      <c r="CI26" t="n">
+        <v>5.9</v>
+      </c>
+      <c r="CJ26" t="n">
+        <v>7.05</v>
+      </c>
+      <c r="CK26" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -25736,6 +26874,18 @@
       <c r="CG27" t="n">
         <v>14</v>
       </c>
+      <c r="CH27" t="n">
+        <v>528.52</v>
+      </c>
+      <c r="CI27" t="n">
+        <v>2.99</v>
+      </c>
+      <c r="CJ27" t="n">
+        <v>3.41</v>
+      </c>
+      <c r="CK27" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -26003,6 +27153,18 @@
       <c r="CG28" t="n">
         <v>14</v>
       </c>
+      <c r="CH28" t="n">
+        <v>1656.65</v>
+      </c>
+      <c r="CI28" t="n">
+        <v>-0.03</v>
+      </c>
+      <c r="CJ28" t="n">
+        <v>-0.75</v>
+      </c>
+      <c r="CK28" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -26270,6 +27432,18 @@
       <c r="CG29" t="n">
         <v>14</v>
       </c>
+      <c r="CH29" t="n">
+        <v>1495.27</v>
+      </c>
+      <c r="CI29" t="n">
+        <v>-0.29</v>
+      </c>
+      <c r="CJ29" t="n">
+        <v>-1.04</v>
+      </c>
+      <c r="CK29" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -26537,6 +27711,18 @@
       <c r="CG30" t="n">
         <v>14</v>
       </c>
+      <c r="CH30" t="n">
+        <v>161.38</v>
+      </c>
+      <c r="CI30" t="n">
+        <v>2.37</v>
+      </c>
+      <c r="CJ30" t="n">
+        <v>1.97</v>
+      </c>
+      <c r="CK30" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -26804,6 +27990,18 @@
       <c r="CG31" t="n">
         <v>14</v>
       </c>
+      <c r="CH31" t="n">
+        <v>1583.32</v>
+      </c>
+      <c r="CI31" t="n">
+        <v>3.29</v>
+      </c>
+      <c r="CJ31" t="n">
+        <v>0.55</v>
+      </c>
+      <c r="CK31" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -27071,6 +28269,18 @@
       <c r="CG32" t="n">
         <v>14</v>
       </c>
+      <c r="CH32" t="n">
+        <v>1000.63</v>
+      </c>
+      <c r="CI32" t="n">
+        <v>4.06</v>
+      </c>
+      <c r="CJ32" t="n">
+        <v>2.32</v>
+      </c>
+      <c r="CK32" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -27338,6 +28548,18 @@
       <c r="CG33" t="n">
         <v>14</v>
       </c>
+      <c r="CH33" t="n">
+        <v>582.6900000000001</v>
+      </c>
+      <c r="CI33" t="n">
+        <v>1.98</v>
+      </c>
+      <c r="CJ33" t="n">
+        <v>-2.41</v>
+      </c>
+      <c r="CK33" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -27605,6 +28827,18 @@
       <c r="CG34" t="n">
         <v>14</v>
       </c>
+      <c r="CH34" t="n">
+        <v>436.32</v>
+      </c>
+      <c r="CI34" t="n">
+        <v>2.97</v>
+      </c>
+      <c r="CJ34" t="n">
+        <v>-1.99</v>
+      </c>
+      <c r="CK34" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -27872,6 +29106,18 @@
       <c r="CG35" t="n">
         <v>14</v>
       </c>
+      <c r="CH35" t="n">
+        <v>2210.88</v>
+      </c>
+      <c r="CI35" t="n">
+        <v>15.64</v>
+      </c>
+      <c r="CJ35" t="n">
+        <v>11.57</v>
+      </c>
+      <c r="CK35" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -28139,6 +29385,18 @@
       <c r="CG36" t="n">
         <v>14</v>
       </c>
+      <c r="CH36" t="n">
+        <v>1358.51</v>
+      </c>
+      <c r="CI36" t="n">
+        <v>18.93</v>
+      </c>
+      <c r="CJ36" t="n">
+        <v>15.22</v>
+      </c>
+      <c r="CK36" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
@@ -28406,6 +29664,18 @@
       <c r="CG37" t="n">
         <v>14</v>
       </c>
+      <c r="CH37" t="n">
+        <v>12441.01</v>
+      </c>
+      <c r="CI37" t="n">
+        <v>6.78</v>
+      </c>
+      <c r="CJ37" t="n">
+        <v>5.53</v>
+      </c>
+      <c r="CK37" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -28673,6 +29943,18 @@
       <c r="CG38" t="n">
         <v>14</v>
       </c>
+      <c r="CH38" t="n">
+        <v>914.62</v>
+      </c>
+      <c r="CI38" t="n">
+        <v>10.7</v>
+      </c>
+      <c r="CJ38" t="n">
+        <v>8.01</v>
+      </c>
+      <c r="CK38" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
@@ -28940,6 +30222,18 @@
       <c r="CG39" t="n">
         <v>14</v>
       </c>
+      <c r="CH39" t="n">
+        <v>11526.39</v>
+      </c>
+      <c r="CI39" t="n">
+        <v>6.48</v>
+      </c>
+      <c r="CJ39" t="n">
+        <v>5.33</v>
+      </c>
+      <c r="CK39" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
@@ -29196,16 +30490,28 @@
         <v>13</v>
       </c>
       <c r="CD40" t="n">
-        <v>4720.58</v>
+        <v>4722.53</v>
       </c>
       <c r="CE40" t="n">
-        <v>5.34</v>
+        <v>5.38</v>
       </c>
       <c r="CF40" t="n">
-        <v>5.52</v>
+        <v>5.7</v>
       </c>
       <c r="CG40" t="n">
         <v>14</v>
+      </c>
+      <c r="CH40" t="n">
+        <v>4768.51</v>
+      </c>
+      <c r="CI40" t="n">
+        <v>5.07</v>
+      </c>
+      <c r="CJ40" t="n">
+        <v>3.95</v>
+      </c>
+      <c r="CK40" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="41">
@@ -29463,16 +30769,28 @@
         <v>13</v>
       </c>
       <c r="CD41" t="n">
-        <v>733.51</v>
+        <v>733.67</v>
       </c>
       <c r="CE41" t="n">
-        <v>5.08</v>
+        <v>5.1</v>
       </c>
       <c r="CF41" t="n">
-        <v>8.140000000000001</v>
+        <v>8.24</v>
       </c>
       <c r="CG41" t="n">
         <v>14</v>
+      </c>
+      <c r="CH41" t="n">
+        <v>742.22</v>
+      </c>
+      <c r="CI41" t="n">
+        <v>5.78</v>
+      </c>
+      <c r="CJ41" t="n">
+        <v>4.74</v>
+      </c>
+      <c r="CK41" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="42">
@@ -29730,16 +31048,28 @@
         <v>13</v>
       </c>
       <c r="CD42" t="n">
-        <v>2098.92</v>
+        <v>2100.07</v>
       </c>
       <c r="CE42" t="n">
-        <v>3.52</v>
+        <v>3.58</v>
       </c>
       <c r="CF42" t="n">
-        <v>3.62</v>
+        <v>3.85</v>
       </c>
       <c r="CG42" t="n">
         <v>14</v>
+      </c>
+      <c r="CH42" t="n">
+        <v>2116.06</v>
+      </c>
+      <c r="CI42" t="n">
+        <v>3.49</v>
+      </c>
+      <c r="CJ42" t="n">
+        <v>3.08</v>
+      </c>
+      <c r="CK42" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="43">
@@ -29997,16 +31327,28 @@
         <v>13</v>
       </c>
       <c r="CD43" t="n">
-        <v>307.03</v>
+        <v>307.23</v>
       </c>
       <c r="CE43" t="n">
-        <v>-1.26</v>
+        <v>-1.19</v>
       </c>
       <c r="CF43" t="n">
-        <v>3.39</v>
+        <v>3.66</v>
       </c>
       <c r="CG43" t="n">
         <v>14</v>
+      </c>
+      <c r="CH43" t="n">
+        <v>310.39</v>
+      </c>
+      <c r="CI43" t="n">
+        <v>0.8100000000000001</v>
+      </c>
+      <c r="CJ43" t="n">
+        <v>4.17</v>
+      </c>
+      <c r="CK43" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="44">
@@ -30264,16 +31606,28 @@
         <v>13</v>
       </c>
       <c r="CD44" t="n">
-        <v>116.18</v>
+        <v>116.27</v>
       </c>
       <c r="CE44" t="n">
-        <v>4.63</v>
+        <v>4.71</v>
       </c>
       <c r="CF44" t="n">
-        <v>4.5</v>
+        <v>4.85</v>
       </c>
       <c r="CG44" t="n">
         <v>14</v>
+      </c>
+      <c r="CH44" t="n">
+        <v>117.25</v>
+      </c>
+      <c r="CI44" t="n">
+        <v>4.74</v>
+      </c>
+      <c r="CJ44" t="n">
+        <v>3.38</v>
+      </c>
+      <c r="CK44" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="45">
@@ -30531,16 +31885,28 @@
         <v>13</v>
       </c>
       <c r="CD45" t="n">
-        <v>367.08</v>
+        <v>367.34</v>
       </c>
       <c r="CE45" t="n">
-        <v>2.38</v>
+        <v>2.45</v>
       </c>
       <c r="CF45" t="n">
-        <v>1.59</v>
+        <v>1.87</v>
       </c>
       <c r="CG45" t="n">
         <v>14</v>
+      </c>
+      <c r="CH45" t="n">
+        <v>369.07</v>
+      </c>
+      <c r="CI45" t="n">
+        <v>2.07</v>
+      </c>
+      <c r="CJ45" t="n">
+        <v>1.9</v>
+      </c>
+      <c r="CK45" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="46">
@@ -30798,16 +32164,28 @@
         <v>13</v>
       </c>
       <c r="CD46" t="n">
-        <v>1308.63</v>
+        <v>1309.22</v>
       </c>
       <c r="CE46" t="n">
-        <v>4.95</v>
+        <v>5</v>
       </c>
       <c r="CF46" t="n">
-        <v>4.18</v>
+        <v>4.37</v>
       </c>
       <c r="CG46" t="n">
         <v>14</v>
+      </c>
+      <c r="CH46" t="n">
+        <v>1319.36</v>
+      </c>
+      <c r="CI46" t="n">
+        <v>4.44</v>
+      </c>
+      <c r="CJ46" t="n">
+        <v>3.13</v>
+      </c>
+      <c r="CK46" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="47">
@@ -31065,16 +32443,28 @@
         <v>13</v>
       </c>
       <c r="CD47" t="n">
-        <v>1036.35</v>
+        <v>1036.9</v>
       </c>
       <c r="CE47" t="n">
-        <v>3.66</v>
+        <v>3.72</v>
       </c>
       <c r="CF47" t="n">
-        <v>3.22</v>
+        <v>3.44</v>
       </c>
       <c r="CG47" t="n">
         <v>14</v>
+      </c>
+      <c r="CH47" t="n">
+        <v>1039.2</v>
+      </c>
+      <c r="CI47" t="n">
+        <v>2.92</v>
+      </c>
+      <c r="CJ47" t="n">
+        <v>0.89</v>
+      </c>
+      <c r="CK47" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="48">
@@ -31332,16 +32722,28 @@
         <v>13</v>
       </c>
       <c r="CD48" t="n">
-        <v>908.52</v>
+        <v>908.97</v>
       </c>
       <c r="CE48" t="n">
-        <v>2.7</v>
+        <v>2.75</v>
       </c>
       <c r="CF48" t="n">
-        <v>2.1</v>
+        <v>2.31</v>
       </c>
       <c r="CG48" t="n">
         <v>14</v>
+      </c>
+      <c r="CH48" t="n">
+        <v>909.23</v>
+      </c>
+      <c r="CI48" t="n">
+        <v>2</v>
+      </c>
+      <c r="CJ48" t="n">
+        <v>0.12</v>
+      </c>
+      <c r="CK48" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="49">
@@ -31599,16 +33001,28 @@
         <v>13</v>
       </c>
       <c r="CD49" t="n">
-        <v>127.82</v>
+        <v>127.93</v>
       </c>
       <c r="CE49" t="n">
-        <v>11.02</v>
+        <v>11.11</v>
       </c>
       <c r="CF49" t="n">
-        <v>11.57</v>
+        <v>11.93</v>
       </c>
       <c r="CG49" t="n">
         <v>14</v>
+      </c>
+      <c r="CH49" t="n">
+        <v>129.96</v>
+      </c>
+      <c r="CI49" t="n">
+        <v>9.83</v>
+      </c>
+      <c r="CJ49" t="n">
+        <v>6.52</v>
+      </c>
+      <c r="CK49" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="50">
@@ -31866,16 +33280,28 @@
         <v>13</v>
       </c>
       <c r="CD50" t="n">
-        <v>338.23</v>
+        <v>338.21</v>
       </c>
       <c r="CE50" t="n">
-        <v>8.83</v>
+        <v>8.82</v>
       </c>
       <c r="CF50" t="n">
-        <v>14.53</v>
+        <v>14.5</v>
       </c>
       <c r="CG50" t="n">
         <v>14</v>
+      </c>
+      <c r="CH50" t="n">
+        <v>352.34</v>
+      </c>
+      <c r="CI50" t="n">
+        <v>11.19</v>
+      </c>
+      <c r="CJ50" t="n">
+        <v>17.8</v>
+      </c>
+      <c r="CK50" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="51">
@@ -32139,10 +33565,22 @@
         <v>-0.07000000000000001</v>
       </c>
       <c r="CF51" t="n">
-        <v>-4.58</v>
+        <v>-4.59</v>
       </c>
       <c r="CG51" t="n">
         <v>14</v>
+      </c>
+      <c r="CH51" t="n">
+        <v>103.43</v>
+      </c>
+      <c r="CI51" t="n">
+        <v>6.35</v>
+      </c>
+      <c r="CJ51" t="n">
+        <v>39.02</v>
+      </c>
+      <c r="CK51" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="52">
@@ -32400,16 +33838,28 @@
         <v>13</v>
       </c>
       <c r="CD52" t="n">
-        <v>242.98</v>
+        <v>242.95</v>
       </c>
       <c r="CE52" t="n">
-        <v>12.77</v>
+        <v>12.76</v>
       </c>
       <c r="CF52" t="n">
-        <v>23.32</v>
+        <v>23.28</v>
       </c>
       <c r="CG52" t="n">
         <v>14</v>
+      </c>
+      <c r="CH52" t="n">
+        <v>248.91</v>
+      </c>
+      <c r="CI52" t="n">
+        <v>13.33</v>
+      </c>
+      <c r="CJ52" t="n">
+        <v>10.18</v>
+      </c>
+      <c r="CK52" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="53">
@@ -32667,16 +34117,28 @@
         <v>13</v>
       </c>
       <c r="CD53" t="n">
-        <v>85.59</v>
+        <v>85.58</v>
       </c>
       <c r="CE53" t="n">
-        <v>12.84</v>
+        <v>12.83</v>
       </c>
       <c r="CF53" t="n">
-        <v>25.47</v>
+        <v>25.43</v>
       </c>
       <c r="CG53" t="n">
         <v>14</v>
+      </c>
+      <c r="CH53" t="n">
+        <v>88.08</v>
+      </c>
+      <c r="CI53" t="n">
+        <v>14.74</v>
+      </c>
+      <c r="CJ53" t="n">
+        <v>12.21</v>
+      </c>
+      <c r="CK53" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="54">
@@ -32934,16 +34396,28 @@
         <v>13</v>
       </c>
       <c r="CD54" t="n">
-        <v>513.59</v>
+        <v>513.6900000000001</v>
       </c>
       <c r="CE54" t="n">
-        <v>15.34</v>
+        <v>15.37</v>
       </c>
       <c r="CF54" t="n">
-        <v>8.83</v>
+        <v>8.92</v>
       </c>
       <c r="CG54" t="n">
         <v>14</v>
+      </c>
+      <c r="CH54" t="n">
+        <v>518.6900000000001</v>
+      </c>
+      <c r="CI54" t="n">
+        <v>11.45</v>
+      </c>
+      <c r="CJ54" t="n">
+        <v>3.95</v>
+      </c>
+      <c r="CK54" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="55">
@@ -33201,16 +34675,28 @@
         <v>13</v>
       </c>
       <c r="CD55" t="n">
-        <v>198.24</v>
+        <v>198.32</v>
       </c>
       <c r="CE55" t="n">
-        <v>27.4</v>
+        <v>27.46</v>
       </c>
       <c r="CF55" t="n">
-        <v>5.09</v>
+        <v>5.26</v>
       </c>
       <c r="CG55" t="n">
         <v>14</v>
+      </c>
+      <c r="CH55" t="n">
+        <v>200.67</v>
+      </c>
+      <c r="CI55" t="n">
+        <v>17.11</v>
+      </c>
+      <c r="CJ55" t="n">
+        <v>4.8</v>
+      </c>
+      <c r="CK55" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="56">
@@ -33468,16 +34954,28 @@
         <v>13</v>
       </c>
       <c r="CD56" t="n">
-        <v>5663.78</v>
+        <v>5664.27</v>
       </c>
       <c r="CE56" t="n">
-        <v>4.57</v>
+        <v>4.58</v>
       </c>
       <c r="CF56" t="n">
-        <v>3.42</v>
+        <v>3.46</v>
       </c>
       <c r="CG56" t="n">
         <v>14</v>
+      </c>
+      <c r="CH56" t="n">
+        <v>5688.29</v>
+      </c>
+      <c r="CI56" t="n">
+        <v>3.86</v>
+      </c>
+      <c r="CJ56" t="n">
+        <v>1.71</v>
+      </c>
+      <c r="CK56" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="57">
@@ -33735,16 +35233,28 @@
         <v>13</v>
       </c>
       <c r="CD57" t="n">
-        <v>735.73</v>
+        <v>735.9</v>
       </c>
       <c r="CE57" t="n">
-        <v>0.17</v>
+        <v>0.19</v>
       </c>
       <c r="CF57" t="n">
-        <v>-0.1</v>
+        <v>-0.01</v>
       </c>
       <c r="CG57" t="n">
         <v>14</v>
+      </c>
+      <c r="CH57" t="n">
+        <v>747.5</v>
+      </c>
+      <c r="CI57" t="n">
+        <v>0.27</v>
+      </c>
+      <c r="CJ57" t="n">
+        <v>6.46</v>
+      </c>
+      <c r="CK57" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="58">
@@ -34002,16 +35512,28 @@
         <v>13</v>
       </c>
       <c r="CD58" t="n">
-        <v>4928.05</v>
+        <v>4928.37</v>
       </c>
       <c r="CE58" t="n">
         <v>5.27</v>
       </c>
       <c r="CF58" t="n">
-        <v>3.96</v>
+        <v>3.99</v>
       </c>
       <c r="CG58" t="n">
         <v>14</v>
+      </c>
+      <c r="CH58" t="n">
+        <v>4940.79</v>
+      </c>
+      <c r="CI58" t="n">
+        <v>4.42</v>
+      </c>
+      <c r="CJ58" t="n">
+        <v>1.01</v>
+      </c>
+      <c r="CK58" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="60">

</xml_diff>

<commit_message>
data: refresh 2026-10-23 23:55 UTC
</commit_message>
<xml_diff>
--- a/data/h8-growth5y.xlsx
+++ b/data/h8-growth5y.xlsx
@@ -1161,13 +1161,13 @@
         </is>
       </c>
       <c r="CD2" t="n">
-        <v>12707.3</v>
+        <v>12709</v>
       </c>
       <c r="CE2" t="n">
-        <v>6.93</v>
+        <v>6.94</v>
       </c>
       <c r="CF2" t="n">
-        <v>6.97</v>
+        <v>7.03</v>
       </c>
       <c r="CG2" t="inlineStr">
         <is>
@@ -1175,17 +1175,17 @@
         </is>
       </c>
       <c r="CH2" t="n">
-        <v>12751.96</v>
+        <v>12772.34</v>
       </c>
       <c r="CI2" t="n">
-        <v>5.74</v>
+        <v>5.91</v>
       </c>
       <c r="CJ2" t="n">
-        <v>1.41</v>
+        <v>2.01</v>
       </c>
       <c r="CK2" t="inlineStr">
         <is>
-          <t>2026-10-07</t>
+          <t>2026-10-14</t>
         </is>
       </c>
     </row>
@@ -1482,13 +1482,13 @@
         </is>
       </c>
       <c r="CD3" t="n">
-        <v>2337.26</v>
+        <v>2336.89</v>
       </c>
       <c r="CE3" t="n">
-        <v>8.23</v>
+        <v>8.210000000000001</v>
       </c>
       <c r="CF3" t="n">
-        <v>8.800000000000001</v>
+        <v>8.73</v>
       </c>
       <c r="CG3" t="inlineStr">
         <is>
@@ -1496,17 +1496,17 @@
         </is>
       </c>
       <c r="CH3" t="n">
-        <v>2359.03</v>
+        <v>2357.01</v>
       </c>
       <c r="CI3" t="n">
-        <v>9.369999999999999</v>
+        <v>9.27</v>
       </c>
       <c r="CJ3" t="n">
-        <v>3.78</v>
+        <v>3.49</v>
       </c>
       <c r="CK3" t="inlineStr">
         <is>
-          <t>2026-10-07</t>
+          <t>2026-10-14</t>
         </is>
       </c>
     </row>
@@ -1803,13 +1803,13 @@
         </is>
       </c>
       <c r="CD4" t="n">
-        <v>3024.68</v>
+        <v>3024.66</v>
       </c>
       <c r="CE4" t="n">
         <v>3.8</v>
       </c>
       <c r="CF4" t="n">
-        <v>4.8</v>
+        <v>4.79</v>
       </c>
       <c r="CG4" t="inlineStr">
         <is>
@@ -1817,17 +1817,17 @@
         </is>
       </c>
       <c r="CH4" t="n">
-        <v>3031.84</v>
+        <v>3034.05</v>
       </c>
       <c r="CI4" t="n">
-        <v>3</v>
+        <v>3.08</v>
       </c>
       <c r="CJ4" t="n">
-        <v>0.95</v>
+        <v>1.25</v>
       </c>
       <c r="CK4" t="inlineStr">
         <is>
-          <t>2026-10-07</t>
+          <t>2026-10-14</t>
         </is>
       </c>
     </row>
@@ -2124,13 +2124,13 @@
         </is>
       </c>
       <c r="CD5" t="n">
-        <v>434.08</v>
+        <v>434.13</v>
       </c>
       <c r="CE5" t="n">
-        <v>-1.15</v>
+        <v>-1.14</v>
       </c>
       <c r="CF5" t="n">
-        <v>8.449999999999999</v>
+        <v>8.49</v>
       </c>
       <c r="CG5" t="inlineStr">
         <is>
@@ -2138,17 +2138,17 @@
         </is>
       </c>
       <c r="CH5" t="n">
-        <v>436.16</v>
+        <v>435.31</v>
       </c>
       <c r="CI5" t="n">
-        <v>0.61</v>
+        <v>0.41</v>
       </c>
       <c r="CJ5" t="n">
-        <v>1.93</v>
+        <v>1.09</v>
       </c>
       <c r="CK5" t="inlineStr">
         <is>
-          <t>2026-10-07</t>
+          <t>2026-10-14</t>
         </is>
       </c>
     </row>
@@ -2445,13 +2445,13 @@
         </is>
       </c>
       <c r="CD6" t="n">
-        <v>123.39</v>
+        <v>123.33</v>
       </c>
       <c r="CE6" t="n">
-        <v>5.06</v>
+        <v>5</v>
       </c>
       <c r="CF6" t="n">
-        <v>6.17</v>
+        <v>5.93</v>
       </c>
       <c r="CG6" t="inlineStr">
         <is>
@@ -2459,17 +2459,17 @@
         </is>
       </c>
       <c r="CH6" t="n">
-        <v>123.51</v>
+        <v>123.47</v>
       </c>
       <c r="CI6" t="n">
-        <v>3.82</v>
+        <v>3.78</v>
       </c>
       <c r="CJ6" t="n">
-        <v>0.37</v>
+        <v>0.46</v>
       </c>
       <c r="CK6" t="inlineStr">
         <is>
-          <t>2026-10-07</t>
+          <t>2026-10-14</t>
         </is>
       </c>
     </row>
@@ -2766,13 +2766,13 @@
         </is>
       </c>
       <c r="CD7" t="n">
-        <v>621.4400000000001</v>
+        <v>621.38</v>
       </c>
       <c r="CE7" t="n">
-        <v>4.6</v>
+        <v>4.59</v>
       </c>
       <c r="CF7" t="n">
-        <v>2.83</v>
+        <v>2.79</v>
       </c>
       <c r="CG7" t="inlineStr">
         <is>
@@ -2780,17 +2780,17 @@
         </is>
       </c>
       <c r="CH7" t="n">
-        <v>624.29</v>
+        <v>623.28</v>
       </c>
       <c r="CI7" t="n">
-        <v>3.12</v>
+        <v>2.95</v>
       </c>
       <c r="CJ7" t="n">
-        <v>1.85</v>
+        <v>1.23</v>
       </c>
       <c r="CK7" t="inlineStr">
         <is>
-          <t>2026-10-07</t>
+          <t>2026-10-14</t>
         </is>
       </c>
     </row>
@@ -3087,13 +3087,13 @@
         </is>
       </c>
       <c r="CD8" t="n">
-        <v>1845.77</v>
+        <v>1845.82</v>
       </c>
       <c r="CE8" t="n">
-        <v>4.67</v>
+        <v>4.68</v>
       </c>
       <c r="CF8" t="n">
-        <v>4.54</v>
+        <v>4.55</v>
       </c>
       <c r="CG8" t="inlineStr">
         <is>
@@ -3101,17 +3101,17 @@
         </is>
       </c>
       <c r="CH8" t="n">
-        <v>1847.88</v>
+        <v>1852</v>
       </c>
       <c r="CI8" t="n">
-        <v>3.49</v>
+        <v>3.72</v>
       </c>
       <c r="CJ8" t="n">
-        <v>0.46</v>
+        <v>1.34</v>
       </c>
       <c r="CK8" t="inlineStr">
         <is>
-          <t>2026-10-07</t>
+          <t>2026-10-14</t>
         </is>
       </c>
     </row>
@@ -3408,7 +3408,7 @@
         </is>
       </c>
       <c r="CD9" t="n">
-        <v>2697.46</v>
+        <v>2697.47</v>
       </c>
       <c r="CE9" t="n">
         <v>1.49</v>
@@ -3422,17 +3422,17 @@
         </is>
       </c>
       <c r="CH9" t="n">
-        <v>2695.85</v>
+        <v>2695.49</v>
       </c>
       <c r="CI9" t="n">
-        <v>0.89</v>
+        <v>0.88</v>
       </c>
       <c r="CJ9" t="n">
-        <v>-0.24</v>
+        <v>-0.29</v>
       </c>
       <c r="CK9" t="inlineStr">
         <is>
-          <t>2026-10-07</t>
+          <t>2026-10-14</t>
         </is>
       </c>
     </row>
@@ -3729,7 +3729,7 @@
         </is>
       </c>
       <c r="CD10" t="n">
-        <v>2406.4</v>
+        <v>2406.39</v>
       </c>
       <c r="CE10" t="n">
         <v>0.93</v>
@@ -3743,17 +3743,17 @@
         </is>
       </c>
       <c r="CH10" t="n">
-        <v>2404.5</v>
+        <v>2404.02</v>
       </c>
       <c r="CI10" t="n">
-        <v>0.42</v>
+        <v>0.4</v>
       </c>
       <c r="CJ10" t="n">
-        <v>-0.32</v>
+        <v>-0.39</v>
       </c>
       <c r="CK10" t="inlineStr">
         <is>
-          <t>2026-10-07</t>
+          <t>2026-10-14</t>
         </is>
       </c>
     </row>
@@ -4050,13 +4050,13 @@
         </is>
       </c>
       <c r="CD11" t="n">
-        <v>291.06</v>
+        <v>291.08</v>
       </c>
       <c r="CE11" t="n">
-        <v>6.41</v>
+        <v>6.42</v>
       </c>
       <c r="CF11" t="n">
-        <v>8.01</v>
+        <v>8.039999999999999</v>
       </c>
       <c r="CG11" t="inlineStr">
         <is>
@@ -4064,17 +4064,17 @@
         </is>
       </c>
       <c r="CH11" t="n">
-        <v>291.34</v>
+        <v>291.47</v>
       </c>
       <c r="CI11" t="n">
-        <v>4.96</v>
+        <v>5.01</v>
       </c>
       <c r="CJ11" t="n">
-        <v>0.39</v>
+        <v>0.54</v>
       </c>
       <c r="CK11" t="inlineStr">
         <is>
-          <t>2026-10-07</t>
+          <t>2026-10-14</t>
         </is>
       </c>
     </row>
@@ -4371,13 +4371,13 @@
         </is>
       </c>
       <c r="CD12" t="n">
-        <v>1927.73</v>
+        <v>1927.84</v>
       </c>
       <c r="CE12" t="n">
-        <v>4.95</v>
+        <v>4.96</v>
       </c>
       <c r="CF12" t="n">
-        <v>5.12</v>
+        <v>5.14</v>
       </c>
       <c r="CG12" t="inlineStr">
         <is>
@@ -4385,17 +4385,17 @@
         </is>
       </c>
       <c r="CH12" t="n">
-        <v>1935.67</v>
+        <v>1938.17</v>
       </c>
       <c r="CI12" t="n">
-        <v>4.16</v>
+        <v>4.29</v>
       </c>
       <c r="CJ12" t="n">
-        <v>1.66</v>
+        <v>2.16</v>
       </c>
       <c r="CK12" t="inlineStr">
         <is>
-          <t>2026-10-07</t>
+          <t>2026-10-14</t>
         </is>
       </c>
     </row>
@@ -4692,13 +4692,13 @@
         </is>
       </c>
       <c r="CD13" t="n">
-        <v>1096.38</v>
+        <v>1096.41</v>
       </c>
       <c r="CE13" t="n">
         <v>4.27</v>
       </c>
       <c r="CF13" t="n">
-        <v>3.19</v>
+        <v>3.2</v>
       </c>
       <c r="CG13" t="inlineStr">
         <is>
@@ -4706,17 +4706,17 @@
         </is>
       </c>
       <c r="CH13" t="n">
-        <v>1104.06</v>
+        <v>1105.85</v>
       </c>
       <c r="CI13" t="n">
-        <v>3.82</v>
+        <v>3.99</v>
       </c>
       <c r="CJ13" t="n">
-        <v>2.83</v>
+        <v>3.49</v>
       </c>
       <c r="CK13" t="inlineStr">
         <is>
-          <t>2026-10-07</t>
+          <t>2026-10-14</t>
         </is>
       </c>
     </row>
@@ -5013,13 +5013,13 @@
         </is>
       </c>
       <c r="CD14" t="n">
-        <v>831.35</v>
+        <v>831.42</v>
       </c>
       <c r="CE14" t="n">
-        <v>5.88</v>
+        <v>5.89</v>
       </c>
       <c r="CF14" t="n">
-        <v>7.73</v>
+        <v>7.77</v>
       </c>
       <c r="CG14" t="inlineStr">
         <is>
@@ -5027,17 +5027,17 @@
         </is>
       </c>
       <c r="CH14" t="n">
-        <v>831.61</v>
+        <v>832.3200000000001</v>
       </c>
       <c r="CI14" t="n">
-        <v>4.61</v>
+        <v>4.7</v>
       </c>
       <c r="CJ14" t="n">
-        <v>0.13</v>
+        <v>0.43</v>
       </c>
       <c r="CK14" t="inlineStr">
         <is>
-          <t>2026-10-07</t>
+          <t>2026-10-14</t>
         </is>
       </c>
     </row>
@@ -5334,13 +5334,13 @@
         </is>
       </c>
       <c r="CD15" t="n">
-        <v>524.4299999999999</v>
+        <v>524.4400000000001</v>
       </c>
       <c r="CE15" t="n">
         <v>5.65</v>
       </c>
       <c r="CF15" t="n">
-        <v>5.09</v>
+        <v>5.1</v>
       </c>
       <c r="CG15" t="inlineStr">
         <is>
@@ -5348,17 +5348,17 @@
         </is>
       </c>
       <c r="CH15" t="n">
-        <v>524.4</v>
+        <v>524.49</v>
       </c>
       <c r="CI15" t="n">
-        <v>3.81</v>
+        <v>3.83</v>
       </c>
       <c r="CJ15" t="n">
-        <v>-0.02</v>
+        <v>0.04</v>
       </c>
       <c r="CK15" t="inlineStr">
         <is>
-          <t>2026-10-07</t>
+          <t>2026-10-14</t>
         </is>
       </c>
     </row>
@@ -5655,13 +5655,13 @@
         </is>
       </c>
       <c r="CD16" t="n">
-        <v>2720.18</v>
+        <v>2722.14</v>
       </c>
       <c r="CE16" t="n">
-        <v>17.45</v>
+        <v>17.54</v>
       </c>
       <c r="CF16" t="n">
-        <v>16.53</v>
+        <v>16.87</v>
       </c>
       <c r="CG16" t="inlineStr">
         <is>
@@ -5669,17 +5669,17 @@
         </is>
       </c>
       <c r="CH16" t="n">
-        <v>2729.57</v>
+        <v>2747.61</v>
       </c>
       <c r="CI16" t="n">
-        <v>12.37</v>
+        <v>13.12</v>
       </c>
       <c r="CJ16" t="n">
-        <v>1.39</v>
+        <v>3.8</v>
       </c>
       <c r="CK16" t="inlineStr">
         <is>
-          <t>2026-10-07</t>
+          <t>2026-10-14</t>
         </is>
       </c>
     </row>
@@ -5976,13 +5976,13 @@
         </is>
       </c>
       <c r="CD17" t="n">
-        <v>1547.48</v>
+        <v>1547.57</v>
       </c>
       <c r="CE17" t="n">
-        <v>22.46</v>
+        <v>22.47</v>
       </c>
       <c r="CF17" t="n">
-        <v>22.2</v>
+        <v>22.23</v>
       </c>
       <c r="CG17" t="inlineStr">
         <is>
@@ -5990,17 +5990,17 @@
         </is>
       </c>
       <c r="CH17" t="n">
-        <v>1559.17</v>
+        <v>1566.27</v>
       </c>
       <c r="CI17" t="n">
-        <v>14.43</v>
+        <v>14.95</v>
       </c>
       <c r="CJ17" t="n">
-        <v>3.06</v>
+        <v>4.92</v>
       </c>
       <c r="CK17" t="inlineStr">
         <is>
-          <t>2026-10-07</t>
+          <t>2026-10-14</t>
         </is>
       </c>
     </row>
@@ -6297,7 +6297,7 @@
         </is>
       </c>
       <c r="CD18" t="n">
-        <v>18089.39</v>
+        <v>18089.34</v>
       </c>
       <c r="CE18" t="n">
         <v>6.28</v>
@@ -6311,17 +6311,17 @@
         </is>
       </c>
       <c r="CH18" t="n">
-        <v>18129.3</v>
+        <v>18161.6</v>
       </c>
       <c r="CI18" t="n">
-        <v>5.59</v>
+        <v>5.78</v>
       </c>
       <c r="CJ18" t="n">
-        <v>0.89</v>
+        <v>1.61</v>
       </c>
       <c r="CK18" t="inlineStr">
         <is>
-          <t>2026-10-07</t>
+          <t>2026-10-14</t>
         </is>
       </c>
     </row>
@@ -6618,13 +6618,13 @@
         </is>
       </c>
       <c r="CD19" t="n">
-        <v>1654.15</v>
+        <v>1654.67</v>
       </c>
       <c r="CE19" t="n">
-        <v>7.32</v>
+        <v>7.35</v>
       </c>
       <c r="CF19" t="n">
-        <v>9.16</v>
+        <v>9.300000000000001</v>
       </c>
       <c r="CG19" t="inlineStr">
         <is>
@@ -6632,17 +6632,17 @@
         </is>
       </c>
       <c r="CH19" t="n">
-        <v>1662.12</v>
+        <v>1675.79</v>
       </c>
       <c r="CI19" t="n">
-        <v>5.07</v>
+        <v>5.93</v>
       </c>
       <c r="CJ19" t="n">
-        <v>1.94</v>
+        <v>5.2</v>
       </c>
       <c r="CK19" t="inlineStr">
         <is>
-          <t>2026-10-07</t>
+          <t>2026-10-14</t>
         </is>
       </c>
     </row>
@@ -6939,13 +6939,13 @@
         </is>
       </c>
       <c r="CD20" t="n">
-        <v>16435.24</v>
+        <v>16434.67</v>
       </c>
       <c r="CE20" t="n">
         <v>6.17</v>
       </c>
       <c r="CF20" t="n">
-        <v>4.54</v>
+        <v>4.52</v>
       </c>
       <c r="CG20" t="inlineStr">
         <is>
@@ -6953,17 +6953,17 @@
         </is>
       </c>
       <c r="CH20" t="n">
-        <v>16467.18</v>
+        <v>16485.81</v>
       </c>
       <c r="CI20" t="n">
-        <v>5.64</v>
+        <v>5.76</v>
       </c>
       <c r="CJ20" t="n">
-        <v>0.78</v>
+        <v>1.25</v>
       </c>
       <c r="CK20" t="inlineStr">
         <is>
-          <t>2026-10-07</t>
+          <t>2026-10-14</t>
         </is>
       </c>
     </row>
@@ -7274,17 +7274,17 @@
         </is>
       </c>
       <c r="CH21" t="n">
-        <v>7983.45</v>
+        <v>7999.72</v>
       </c>
       <c r="CI21" t="n">
-        <v>6.49</v>
+        <v>6.71</v>
       </c>
       <c r="CJ21" t="n">
-        <v>1.48</v>
+        <v>2.31</v>
       </c>
       <c r="CK21" t="inlineStr">
         <is>
-          <t>2026-10-07</t>
+          <t>2026-10-14</t>
         </is>
       </c>
     </row>
@@ -7595,17 +7595,17 @@
         </is>
       </c>
       <c r="CH22" t="n">
-        <v>1616.81</v>
+        <v>1614.97</v>
       </c>
       <c r="CI22" t="n">
-        <v>11.08</v>
+        <v>10.95</v>
       </c>
       <c r="CJ22" t="n">
-        <v>5.06</v>
+        <v>4.58</v>
       </c>
       <c r="CK22" t="inlineStr">
         <is>
-          <t>2026-10-07</t>
+          <t>2026-10-14</t>
         </is>
       </c>
     </row>
@@ -7916,17 +7916,17 @@
         </is>
       </c>
       <c r="CH23" t="n">
-        <v>915.78</v>
+        <v>918.39</v>
       </c>
       <c r="CI23" t="n">
-        <v>2.71</v>
+        <v>3</v>
       </c>
       <c r="CJ23" t="n">
-        <v>1.44</v>
+        <v>2.6</v>
       </c>
       <c r="CK23" t="inlineStr">
         <is>
-          <t>2026-10-07</t>
+          <t>2026-10-14</t>
         </is>
       </c>
     </row>
@@ -8237,17 +8237,17 @@
         </is>
       </c>
       <c r="CH24" t="n">
-        <v>125.77</v>
+        <v>125.46</v>
       </c>
       <c r="CI24" t="n">
-        <v>-1.55</v>
+        <v>-1.79</v>
       </c>
       <c r="CJ24" t="n">
-        <v>2.38</v>
+        <v>1.38</v>
       </c>
       <c r="CK24" t="inlineStr">
         <is>
-          <t>2026-10-07</t>
+          <t>2026-10-14</t>
         </is>
       </c>
     </row>
@@ -8558,17 +8558,17 @@
         </is>
       </c>
       <c r="CH25" t="n">
-        <v>6.26</v>
+        <v>6.24</v>
       </c>
       <c r="CI25" t="n">
-        <v>-2.61</v>
+        <v>-2.97</v>
       </c>
       <c r="CJ25" t="n">
-        <v>-6.6</v>
+        <v>-7.97</v>
       </c>
       <c r="CK25" t="inlineStr">
         <is>
-          <t>2026-10-07</t>
+          <t>2026-10-14</t>
         </is>
       </c>
     </row>
@@ -8879,17 +8879,17 @@
         </is>
       </c>
       <c r="CH26" t="n">
-        <v>255.22</v>
+        <v>254.71</v>
       </c>
       <c r="CI26" t="n">
-        <v>5.45</v>
+        <v>5.23</v>
       </c>
       <c r="CJ26" t="n">
-        <v>3.35</v>
+        <v>2.52</v>
       </c>
       <c r="CK26" t="inlineStr">
         <is>
-          <t>2026-10-07</t>
+          <t>2026-10-14</t>
         </is>
       </c>
     </row>
@@ -9200,17 +9200,17 @@
         </is>
       </c>
       <c r="CH27" t="n">
-        <v>528.52</v>
+        <v>531.97</v>
       </c>
       <c r="CI27" t="n">
-        <v>2.55</v>
+        <v>3.22</v>
       </c>
       <c r="CJ27" t="n">
-        <v>0.42</v>
+        <v>3.06</v>
       </c>
       <c r="CK27" t="inlineStr">
         <is>
-          <t>2026-10-07</t>
+          <t>2026-10-14</t>
         </is>
       </c>
     </row>
@@ -9521,17 +9521,17 @@
         </is>
       </c>
       <c r="CH28" t="n">
-        <v>1656.65</v>
+        <v>1657.24</v>
       </c>
       <c r="CI28" t="n">
-        <v>-0.11</v>
+        <v>-0.07000000000000001</v>
       </c>
       <c r="CJ28" t="n">
-        <v>-0.71</v>
+        <v>-0.57</v>
       </c>
       <c r="CK28" t="inlineStr">
         <is>
-          <t>2026-10-07</t>
+          <t>2026-10-14</t>
         </is>
       </c>
     </row>
@@ -9842,17 +9842,17 @@
         </is>
       </c>
       <c r="CH29" t="n">
-        <v>1495.27</v>
+        <v>1495.64</v>
       </c>
       <c r="CI29" t="n">
-        <v>-0.35</v>
+        <v>-0.33</v>
       </c>
       <c r="CJ29" t="n">
-        <v>-0.8100000000000001</v>
+        <v>-0.71</v>
       </c>
       <c r="CK29" t="inlineStr">
         <is>
-          <t>2026-10-07</t>
+          <t>2026-10-14</t>
         </is>
       </c>
     </row>
@@ -10163,17 +10163,17 @@
         </is>
       </c>
       <c r="CH30" t="n">
-        <v>161.38</v>
+        <v>161.6</v>
       </c>
       <c r="CI30" t="n">
-        <v>2.22</v>
+        <v>2.35</v>
       </c>
       <c r="CJ30" t="n">
-        <v>0.17</v>
+        <v>0.72</v>
       </c>
       <c r="CK30" t="inlineStr">
         <is>
-          <t>2026-10-07</t>
+          <t>2026-10-14</t>
         </is>
       </c>
     </row>
@@ -10484,17 +10484,17 @@
         </is>
       </c>
       <c r="CH31" t="n">
-        <v>1583.32</v>
+        <v>1584.56</v>
       </c>
       <c r="CI31" t="n">
-        <v>2.88</v>
+        <v>2.96</v>
       </c>
       <c r="CJ31" t="n">
-        <v>-0.73</v>
+        <v>-0.42</v>
       </c>
       <c r="CK31" t="inlineStr">
         <is>
-          <t>2026-10-07</t>
+          <t>2026-10-14</t>
         </is>
       </c>
     </row>
@@ -10805,17 +10805,17 @@
         </is>
       </c>
       <c r="CH32" t="n">
-        <v>1000.63</v>
+        <v>1002.07</v>
       </c>
       <c r="CI32" t="n">
-        <v>3.64</v>
+        <v>3.79</v>
       </c>
       <c r="CJ32" t="n">
-        <v>-0.79</v>
+        <v>-0.22</v>
       </c>
       <c r="CK32" t="inlineStr">
         <is>
-          <t>2026-10-07</t>
+          <t>2026-10-14</t>
         </is>
       </c>
     </row>
@@ -11126,17 +11126,17 @@
         </is>
       </c>
       <c r="CH33" t="n">
-        <v>582.6900000000001</v>
+        <v>582.49</v>
       </c>
       <c r="CI33" t="n">
-        <v>1.59</v>
+        <v>1.56</v>
       </c>
       <c r="CJ33" t="n">
-        <v>-0.62</v>
+        <v>-0.76</v>
       </c>
       <c r="CK33" t="inlineStr">
         <is>
-          <t>2026-10-07</t>
+          <t>2026-10-14</t>
         </is>
       </c>
     </row>
@@ -11447,17 +11447,17 @@
         </is>
       </c>
       <c r="CH34" t="n">
-        <v>436.32</v>
+        <v>436.15</v>
       </c>
       <c r="CI34" t="n">
-        <v>2</v>
+        <v>1.96</v>
       </c>
       <c r="CJ34" t="n">
-        <v>-0.53</v>
+        <v>-0.6899999999999999</v>
       </c>
       <c r="CK34" t="inlineStr">
         <is>
-          <t>2026-10-07</t>
+          <t>2026-10-14</t>
         </is>
       </c>
     </row>
@@ -11768,17 +11768,17 @@
         </is>
       </c>
       <c r="CH35" t="n">
-        <v>2210.88</v>
+        <v>2224.56</v>
       </c>
       <c r="CI35" t="n">
-        <v>13.26</v>
+        <v>13.96</v>
       </c>
       <c r="CJ35" t="n">
-        <v>2.21</v>
+        <v>4.76</v>
       </c>
       <c r="CK35" t="inlineStr">
         <is>
-          <t>2026-10-07</t>
+          <t>2026-10-14</t>
         </is>
       </c>
     </row>
@@ -12089,17 +12089,17 @@
         </is>
       </c>
       <c r="CH36" t="n">
-        <v>1358.51</v>
+        <v>1363.98</v>
       </c>
       <c r="CI36" t="n">
-        <v>14.97</v>
+        <v>15.44</v>
       </c>
       <c r="CJ36" t="n">
-        <v>4.19</v>
+        <v>5.88</v>
       </c>
       <c r="CK36" t="inlineStr">
         <is>
-          <t>2026-10-07</t>
+          <t>2026-10-14</t>
         </is>
       </c>
     </row>
@@ -12410,17 +12410,17 @@
         </is>
       </c>
       <c r="CH37" t="n">
-        <v>12441.01</v>
+        <v>12466.24</v>
       </c>
       <c r="CI37" t="n">
-        <v>6.57</v>
+        <v>6.79</v>
       </c>
       <c r="CJ37" t="n">
-        <v>0.85</v>
+        <v>1.67</v>
       </c>
       <c r="CK37" t="inlineStr">
         <is>
-          <t>2026-10-07</t>
+          <t>2026-10-14</t>
         </is>
       </c>
     </row>
@@ -12731,17 +12731,17 @@
         </is>
       </c>
       <c r="CH38" t="n">
-        <v>914.62</v>
+        <v>931.27</v>
       </c>
       <c r="CI38" t="n">
-        <v>9.300000000000001</v>
+        <v>11.29</v>
       </c>
       <c r="CJ38" t="n">
-        <v>-1.77</v>
+        <v>5.58</v>
       </c>
       <c r="CK38" t="inlineStr">
         <is>
-          <t>2026-10-07</t>
+          <t>2026-10-14</t>
         </is>
       </c>
     </row>
@@ -13052,17 +13052,17 @@
         </is>
       </c>
       <c r="CH39" t="n">
-        <v>11526.39</v>
+        <v>11534.97</v>
       </c>
       <c r="CI39" t="n">
-        <v>6.36</v>
+        <v>6.44</v>
       </c>
       <c r="CJ39" t="n">
-        <v>1.06</v>
+        <v>1.36</v>
       </c>
       <c r="CK39" t="inlineStr">
         <is>
-          <t>2026-10-07</t>
+          <t>2026-10-14</t>
         </is>
       </c>
     </row>
@@ -13359,13 +13359,13 @@
         </is>
       </c>
       <c r="CD40" t="n">
-        <v>4753.14</v>
+        <v>4754.84</v>
       </c>
       <c r="CE40" t="n">
-        <v>5.52</v>
+        <v>5.56</v>
       </c>
       <c r="CF40" t="n">
-        <v>5.42</v>
+        <v>5.57</v>
       </c>
       <c r="CG40" t="inlineStr">
         <is>
@@ -13373,17 +13373,17 @@
         </is>
       </c>
       <c r="CH40" t="n">
-        <v>4768.51</v>
+        <v>4772.62</v>
       </c>
       <c r="CI40" t="n">
-        <v>4.5</v>
+        <v>4.59</v>
       </c>
       <c r="CJ40" t="n">
-        <v>1.3</v>
+        <v>1.5</v>
       </c>
       <c r="CK40" t="inlineStr">
         <is>
-          <t>2026-10-07</t>
+          <t>2026-10-14</t>
         </is>
       </c>
     </row>
@@ -13680,13 +13680,13 @@
         </is>
       </c>
       <c r="CD41" t="n">
-        <v>740.26</v>
+        <v>739.9</v>
       </c>
       <c r="CE41" t="n">
-        <v>5.22</v>
+        <v>5.17</v>
       </c>
       <c r="CF41" t="n">
-        <v>5.96</v>
+        <v>5.76</v>
       </c>
       <c r="CG41" t="inlineStr">
         <is>
@@ -13694,17 +13694,17 @@
         </is>
       </c>
       <c r="CH41" t="n">
-        <v>742.22</v>
+        <v>742.04</v>
       </c>
       <c r="CI41" t="n">
-        <v>5.81</v>
+        <v>5.78</v>
       </c>
       <c r="CJ41" t="n">
-        <v>1.06</v>
+        <v>1.16</v>
       </c>
       <c r="CK41" t="inlineStr">
         <is>
-          <t>2026-10-07</t>
+          <t>2026-10-14</t>
         </is>
       </c>
     </row>
@@ -14001,7 +14001,7 @@
         </is>
       </c>
       <c r="CD42" t="n">
-        <v>2112.18</v>
+        <v>2112.15</v>
       </c>
       <c r="CE42" t="n">
         <v>3.89</v>
@@ -14015,17 +14015,17 @@
         </is>
       </c>
       <c r="CH42" t="n">
-        <v>2116.06</v>
+        <v>2115.67</v>
       </c>
       <c r="CI42" t="n">
-        <v>3.13</v>
+        <v>3.11</v>
       </c>
       <c r="CJ42" t="n">
-        <v>0.74</v>
+        <v>0.67</v>
       </c>
       <c r="CK42" t="inlineStr">
         <is>
-          <t>2026-10-07</t>
+          <t>2026-10-14</t>
         </is>
       </c>
     </row>
@@ -14322,13 +14322,13 @@
         </is>
       </c>
       <c r="CD43" t="n">
-        <v>309.05</v>
+        <v>309.1</v>
       </c>
       <c r="CE43" t="n">
-        <v>-0.26</v>
+        <v>-0.24</v>
       </c>
       <c r="CF43" t="n">
-        <v>7.35</v>
+        <v>7.42</v>
       </c>
       <c r="CG43" t="inlineStr">
         <is>
@@ -14336,17 +14336,17 @@
         </is>
       </c>
       <c r="CH43" t="n">
-        <v>310.39</v>
+        <v>309.85</v>
       </c>
       <c r="CI43" t="n">
-        <v>1.51</v>
+        <v>1.33</v>
       </c>
       <c r="CJ43" t="n">
-        <v>1.74</v>
+        <v>0.97</v>
       </c>
       <c r="CK43" t="inlineStr">
         <is>
-          <t>2026-10-07</t>
+          <t>2026-10-14</t>
         </is>
       </c>
     </row>
@@ -14643,13 +14643,13 @@
         </is>
       </c>
       <c r="CD44" t="n">
-        <v>117.02</v>
+        <v>116.95</v>
       </c>
       <c r="CE44" t="n">
-        <v>5.29</v>
+        <v>5.23</v>
       </c>
       <c r="CF44" t="n">
-        <v>5.22</v>
+        <v>4.97</v>
       </c>
       <c r="CG44" t="inlineStr">
         <is>
@@ -14657,17 +14657,17 @@
         </is>
       </c>
       <c r="CH44" t="n">
-        <v>117.25</v>
+        <v>117.22</v>
       </c>
       <c r="CI44" t="n">
-        <v>4.19</v>
+        <v>4.17</v>
       </c>
       <c r="CJ44" t="n">
-        <v>0.76</v>
+        <v>0.93</v>
       </c>
       <c r="CK44" t="inlineStr">
         <is>
-          <t>2026-10-07</t>
+          <t>2026-10-14</t>
         </is>
       </c>
     </row>
@@ -14964,13 +14964,13 @@
         </is>
       </c>
       <c r="CD45" t="n">
-        <v>368.31</v>
+        <v>368.25</v>
       </c>
       <c r="CE45" t="n">
-        <v>2.43</v>
+        <v>2.41</v>
       </c>
       <c r="CF45" t="n">
-        <v>2.18</v>
+        <v>2.11</v>
       </c>
       <c r="CG45" t="inlineStr">
         <is>
@@ -14978,17 +14978,17 @@
         </is>
       </c>
       <c r="CH45" t="n">
-        <v>369.07</v>
+        <v>368.57</v>
       </c>
       <c r="CI45" t="n">
-        <v>1.57</v>
+        <v>1.43</v>
       </c>
       <c r="CJ45" t="n">
-        <v>0.83</v>
+        <v>0.35</v>
       </c>
       <c r="CK45" t="inlineStr">
         <is>
-          <t>2026-10-07</t>
+          <t>2026-10-14</t>
         </is>
       </c>
     </row>
@@ -15285,13 +15285,13 @@
         </is>
       </c>
       <c r="CD46" t="n">
-        <v>1317.8</v>
+        <v>1317.85</v>
       </c>
       <c r="CE46" t="n">
-        <v>5.21</v>
+        <v>5.22</v>
       </c>
       <c r="CF46" t="n">
-        <v>4.27</v>
+        <v>4.28</v>
       </c>
       <c r="CG46" t="inlineStr">
         <is>
@@ -15299,17 +15299,17 @@
         </is>
       </c>
       <c r="CH46" t="n">
-        <v>1319.36</v>
+        <v>1320.02</v>
       </c>
       <c r="CI46" t="n">
-        <v>3.87</v>
+        <v>3.92</v>
       </c>
       <c r="CJ46" t="n">
-        <v>0.47</v>
+        <v>0.66</v>
       </c>
       <c r="CK46" t="inlineStr">
         <is>
-          <t>2026-10-07</t>
+          <t>2026-10-14</t>
         </is>
       </c>
     </row>
@@ -15606,13 +15606,13 @@
         </is>
       </c>
       <c r="CD47" t="n">
-        <v>1037.86</v>
+        <v>1037.87</v>
       </c>
       <c r="CE47" t="n">
         <v>3.42</v>
       </c>
       <c r="CF47" t="n">
-        <v>2.36</v>
+        <v>2.37</v>
       </c>
       <c r="CG47" t="inlineStr">
         <is>
@@ -15620,17 +15620,17 @@
         </is>
       </c>
       <c r="CH47" t="n">
-        <v>1039.2</v>
+        <v>1038.25</v>
       </c>
       <c r="CI47" t="n">
-        <v>2.53</v>
+        <v>2.44</v>
       </c>
       <c r="CJ47" t="n">
-        <v>0.52</v>
+        <v>0.15</v>
       </c>
       <c r="CK47" t="inlineStr">
         <is>
-          <t>2026-10-07</t>
+          <t>2026-10-14</t>
         </is>
       </c>
     </row>
@@ -15941,17 +15941,17 @@
         </is>
       </c>
       <c r="CH48" t="n">
-        <v>909.23</v>
+        <v>908.37</v>
       </c>
       <c r="CI48" t="n">
-        <v>1.72</v>
+        <v>1.62</v>
       </c>
       <c r="CJ48" t="n">
-        <v>0.5</v>
+        <v>0.12</v>
       </c>
       <c r="CK48" t="inlineStr">
         <is>
-          <t>2026-10-07</t>
+          <t>2026-10-14</t>
         </is>
       </c>
     </row>
@@ -16248,13 +16248,13 @@
         </is>
       </c>
       <c r="CD49" t="n">
-        <v>129.75</v>
+        <v>129.77</v>
       </c>
       <c r="CE49" t="n">
-        <v>11.44</v>
+        <v>11.46</v>
       </c>
       <c r="CF49" t="n">
-        <v>13.32</v>
+        <v>13.38</v>
       </c>
       <c r="CG49" t="inlineStr">
         <is>
@@ -16262,17 +16262,17 @@
         </is>
       </c>
       <c r="CH49" t="n">
-        <v>129.96</v>
+        <v>129.88</v>
       </c>
       <c r="CI49" t="n">
-        <v>8.59</v>
+        <v>8.52</v>
       </c>
       <c r="CJ49" t="n">
-        <v>0.66</v>
+        <v>0.33</v>
       </c>
       <c r="CK49" t="inlineStr">
         <is>
-          <t>2026-10-07</t>
+          <t>2026-10-14</t>
         </is>
       </c>
     </row>
@@ -16569,13 +16569,13 @@
         </is>
       </c>
       <c r="CD50" t="n">
-        <v>341.51</v>
+        <v>341.62</v>
       </c>
       <c r="CE50" t="n">
-        <v>9</v>
+        <v>9.039999999999999</v>
       </c>
       <c r="CF50" t="n">
-        <v>15.07</v>
+        <v>15.22</v>
       </c>
       <c r="CG50" t="inlineStr">
         <is>
@@ -16583,17 +16583,17 @@
         </is>
       </c>
       <c r="CH50" t="n">
-        <v>352.34</v>
+        <v>353.61</v>
       </c>
       <c r="CI50" t="n">
-        <v>10.32</v>
+        <v>10.72</v>
       </c>
       <c r="CJ50" t="n">
-        <v>13.31</v>
+        <v>14.8</v>
       </c>
       <c r="CK50" t="inlineStr">
         <is>
-          <t>2026-10-07</t>
+          <t>2026-10-14</t>
         </is>
       </c>
     </row>
@@ -16890,13 +16890,13 @@
         </is>
       </c>
       <c r="CD51" t="n">
-        <v>93.77</v>
+        <v>93.8</v>
       </c>
       <c r="CE51" t="n">
-        <v>-2.39</v>
+        <v>-2.36</v>
       </c>
       <c r="CF51" t="n">
-        <v>-5.14</v>
+        <v>-5</v>
       </c>
       <c r="CG51" t="inlineStr">
         <is>
@@ -16904,17 +16904,17 @@
         </is>
       </c>
       <c r="CH51" t="n">
-        <v>103.43</v>
+        <v>103.78</v>
       </c>
       <c r="CI51" t="n">
-        <v>5.6</v>
+        <v>5.96</v>
       </c>
       <c r="CJ51" t="n">
-        <v>48.05</v>
+        <v>49.86</v>
       </c>
       <c r="CK51" t="inlineStr">
         <is>
-          <t>2026-10-07</t>
+          <t>2026-10-14</t>
         </is>
       </c>
     </row>
@@ -17211,13 +17211,13 @@
         </is>
       </c>
       <c r="CD52" t="n">
-        <v>247.74</v>
+        <v>247.82</v>
       </c>
       <c r="CE52" t="n">
-        <v>14.04</v>
+        <v>14.07</v>
       </c>
       <c r="CF52" t="n">
-        <v>24.11</v>
+        <v>24.27</v>
       </c>
       <c r="CG52" t="inlineStr">
         <is>
@@ -17225,17 +17225,17 @@
         </is>
       </c>
       <c r="CH52" t="n">
-        <v>248.91</v>
+        <v>249.83</v>
       </c>
       <c r="CI52" t="n">
-        <v>12.41</v>
+        <v>12.82</v>
       </c>
       <c r="CJ52" t="n">
-        <v>1.91</v>
+        <v>3.28</v>
       </c>
       <c r="CK52" t="inlineStr">
         <is>
-          <t>2026-10-07</t>
+          <t>2026-10-14</t>
         </is>
       </c>
     </row>
@@ -17532,13 +17532,13 @@
         </is>
       </c>
       <c r="CD53" t="n">
-        <v>87.53</v>
+        <v>87.54000000000001</v>
       </c>
       <c r="CE53" t="n">
-        <v>14.7</v>
+        <v>14.72</v>
       </c>
       <c r="CF53" t="n">
-        <v>25.8</v>
+        <v>25.87</v>
       </c>
       <c r="CG53" t="inlineStr">
         <is>
@@ -17546,17 +17546,17 @@
         </is>
       </c>
       <c r="CH53" t="n">
-        <v>88.08</v>
+        <v>88.34</v>
       </c>
       <c r="CI53" t="n">
-        <v>13.85</v>
+        <v>14.19</v>
       </c>
       <c r="CJ53" t="n">
-        <v>2.54</v>
+        <v>3.7</v>
       </c>
       <c r="CK53" t="inlineStr">
         <is>
-          <t>2026-10-07</t>
+          <t>2026-10-14</t>
         </is>
       </c>
     </row>
@@ -17853,13 +17853,13 @@
         </is>
       </c>
       <c r="CD54" t="n">
-        <v>521.34</v>
+        <v>523.3</v>
       </c>
       <c r="CE54" t="n">
-        <v>15.62</v>
+        <v>16.06</v>
       </c>
       <c r="CF54" t="n">
-        <v>9.15</v>
+        <v>10.81</v>
       </c>
       <c r="CG54" t="inlineStr">
         <is>
@@ -17867,17 +17867,17 @@
         </is>
       </c>
       <c r="CH54" t="n">
-        <v>518.6900000000001</v>
+        <v>523.05</v>
       </c>
       <c r="CI54" t="n">
-        <v>8.75</v>
+        <v>9.67</v>
       </c>
       <c r="CJ54" t="n">
-        <v>-2.02</v>
+        <v>-0.19</v>
       </c>
       <c r="CK54" t="inlineStr">
         <is>
-          <t>2026-10-07</t>
+          <t>2026-10-14</t>
         </is>
       </c>
     </row>
@@ -18174,13 +18174,13 @@
         </is>
       </c>
       <c r="CD55" t="n">
-        <v>202.83</v>
+        <v>202.92</v>
       </c>
       <c r="CE55" t="n">
-        <v>27.08</v>
+        <v>27.14</v>
       </c>
       <c r="CF55" t="n">
-        <v>6.34</v>
+        <v>6.54</v>
       </c>
       <c r="CG55" t="inlineStr">
         <is>
@@ -18188,17 +18188,17 @@
         </is>
       </c>
       <c r="CH55" t="n">
-        <v>200.67</v>
+        <v>202.29</v>
       </c>
       <c r="CI55" t="n">
-        <v>10.84</v>
+        <v>11.74</v>
       </c>
       <c r="CJ55" t="n">
-        <v>-4.2</v>
+        <v>-1.24</v>
       </c>
       <c r="CK55" t="inlineStr">
         <is>
-          <t>2026-10-07</t>
+          <t>2026-10-14</t>
         </is>
       </c>
     </row>
@@ -18495,7 +18495,7 @@
         </is>
       </c>
       <c r="CD56" t="n">
-        <v>5674.65</v>
+        <v>5674.6</v>
       </c>
       <c r="CE56" t="n">
         <v>4.3</v>
@@ -18509,17 +18509,17 @@
         </is>
       </c>
       <c r="CH56" t="n">
-        <v>5688.29</v>
+        <v>5695.36</v>
       </c>
       <c r="CI56" t="n">
-        <v>3.5</v>
+        <v>3.63</v>
       </c>
       <c r="CJ56" t="n">
-        <v>0.96</v>
+        <v>1.47</v>
       </c>
       <c r="CK56" t="inlineStr">
         <is>
-          <t>2026-10-07</t>
+          <t>2026-10-14</t>
         </is>
       </c>
     </row>
@@ -18816,13 +18816,13 @@
         </is>
       </c>
       <c r="CD57" t="n">
-        <v>735.4400000000001</v>
+        <v>735.96</v>
       </c>
       <c r="CE57" t="n">
-        <v>0.43</v>
+        <v>0.5</v>
       </c>
       <c r="CF57" t="n">
-        <v>-0.7</v>
+        <v>-0.42</v>
       </c>
       <c r="CG57" t="inlineStr">
         <is>
@@ -18830,17 +18830,17 @@
         </is>
       </c>
       <c r="CH57" t="n">
-        <v>747.5</v>
+        <v>744.52</v>
       </c>
       <c r="CI57" t="n">
-        <v>0.31</v>
+        <v>-0.09</v>
       </c>
       <c r="CJ57" t="n">
-        <v>6.72</v>
+        <v>4.73</v>
       </c>
       <c r="CK57" t="inlineStr">
         <is>
-          <t>2026-10-07</t>
+          <t>2026-10-14</t>
         </is>
       </c>
     </row>
@@ -19137,13 +19137,13 @@
         </is>
       </c>
       <c r="CD58" t="n">
-        <v>4939.21</v>
+        <v>4938.65</v>
       </c>
       <c r="CE58" t="n">
-        <v>4.9</v>
+        <v>4.89</v>
       </c>
       <c r="CF58" t="n">
-        <v>2.58</v>
+        <v>2.53</v>
       </c>
       <c r="CG58" t="inlineStr">
         <is>
@@ -19151,17 +19151,17 @@
         </is>
       </c>
       <c r="CH58" t="n">
-        <v>4940.79</v>
+        <v>4950.84</v>
       </c>
       <c r="CI58" t="n">
-        <v>4</v>
+        <v>4.21</v>
       </c>
       <c r="CJ58" t="n">
-        <v>0.13</v>
+        <v>0.99</v>
       </c>
       <c r="CK58" t="inlineStr">
         <is>
-          <t>2026-10-07</t>
+          <t>2026-10-14</t>
         </is>
       </c>
     </row>
@@ -19888,28 +19888,28 @@
         <v>13</v>
       </c>
       <c r="CD2" t="n">
-        <v>12594.27</v>
+        <v>12594.54</v>
       </c>
       <c r="CE2" t="n">
         <v>6.67</v>
       </c>
       <c r="CF2" t="n">
-        <v>5.7</v>
+        <v>5.71</v>
       </c>
       <c r="CG2" t="n">
         <v>14</v>
       </c>
       <c r="CH2" t="n">
-        <v>12751.96</v>
+        <v>12763.08</v>
       </c>
       <c r="CI2" t="n">
-        <v>6.43</v>
+        <v>6.52</v>
       </c>
       <c r="CJ2" t="n">
-        <v>5.1</v>
+        <v>5.46</v>
       </c>
       <c r="CK2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="3">
@@ -20167,28 +20167,28 @@
         <v>13</v>
       </c>
       <c r="CD3" t="n">
-        <v>2307.6</v>
+        <v>2307.32</v>
       </c>
       <c r="CE3" t="n">
-        <v>7.59</v>
+        <v>7.58</v>
       </c>
       <c r="CF3" t="n">
-        <v>7.45</v>
+        <v>7.4</v>
       </c>
       <c r="CG3" t="n">
         <v>14</v>
       </c>
       <c r="CH3" t="n">
-        <v>2359.03</v>
+        <v>2358.01</v>
       </c>
       <c r="CI3" t="n">
-        <v>9.449999999999999</v>
+        <v>9.4</v>
       </c>
       <c r="CJ3" t="n">
-        <v>9.220000000000001</v>
+        <v>9.08</v>
       </c>
       <c r="CK3" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="4">
@@ -20446,28 +20446,28 @@
         <v>13</v>
       </c>
       <c r="CD4" t="n">
-        <v>3005.76</v>
+        <v>3004.46</v>
       </c>
       <c r="CE4" t="n">
-        <v>3.36</v>
+        <v>3.32</v>
       </c>
       <c r="CF4" t="n">
-        <v>3.81</v>
+        <v>3.63</v>
       </c>
       <c r="CG4" t="n">
         <v>14</v>
       </c>
       <c r="CH4" t="n">
-        <v>3031.84</v>
+        <v>3032.63</v>
       </c>
       <c r="CI4" t="n">
-        <v>3.39</v>
+        <v>3.42</v>
       </c>
       <c r="CJ4" t="n">
-        <v>3.52</v>
+        <v>3.8</v>
       </c>
       <c r="CK4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="5">
@@ -20725,28 +20725,28 @@
         <v>13</v>
       </c>
       <c r="CD5" t="n">
-        <v>431.62</v>
+        <v>431.7</v>
       </c>
       <c r="CE5" t="n">
-        <v>-2.08</v>
+        <v>-2.06</v>
       </c>
       <c r="CF5" t="n">
-        <v>3.32</v>
+        <v>3.4</v>
       </c>
       <c r="CG5" t="n">
         <v>14</v>
       </c>
       <c r="CH5" t="n">
-        <v>436.16</v>
+        <v>435.78</v>
       </c>
       <c r="CI5" t="n">
-        <v>0.24</v>
+        <v>0.15</v>
       </c>
       <c r="CJ5" t="n">
-        <v>4.27</v>
+        <v>3.83</v>
       </c>
       <c r="CK5" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="6">
@@ -21004,28 +21004,28 @@
         <v>13</v>
       </c>
       <c r="CD6" t="n">
-        <v>122.56</v>
+        <v>122.54</v>
       </c>
       <c r="CE6" t="n">
-        <v>4.39</v>
+        <v>4.38</v>
       </c>
       <c r="CF6" t="n">
-        <v>4.64</v>
+        <v>4.59</v>
       </c>
       <c r="CG6" t="n">
         <v>14</v>
       </c>
       <c r="CH6" t="n">
-        <v>123.51</v>
+        <v>123.44</v>
       </c>
       <c r="CI6" t="n">
-        <v>4.37</v>
+        <v>4.31</v>
       </c>
       <c r="CJ6" t="n">
-        <v>3.14</v>
+        <v>2.97</v>
       </c>
       <c r="CK6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="7">
@@ -21283,28 +21283,28 @@
         <v>13</v>
       </c>
       <c r="CD7" t="n">
-        <v>618.25</v>
+        <v>617.0599999999999</v>
       </c>
       <c r="CE7" t="n">
-        <v>4.1</v>
+        <v>3.9</v>
       </c>
       <c r="CF7" t="n">
-        <v>2.14</v>
+        <v>1.36</v>
       </c>
       <c r="CG7" t="n">
         <v>14</v>
       </c>
       <c r="CH7" t="n">
-        <v>624.29</v>
+        <v>623.5</v>
       </c>
       <c r="CI7" t="n">
-        <v>3.6</v>
+        <v>3.47</v>
       </c>
       <c r="CJ7" t="n">
-        <v>3.97</v>
+        <v>4.24</v>
       </c>
       <c r="CK7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="8">
@@ -21562,28 +21562,28 @@
         <v>13</v>
       </c>
       <c r="CD8" t="n">
-        <v>1833.34</v>
+        <v>1833.16</v>
       </c>
       <c r="CE8" t="n">
-        <v>4.41</v>
+        <v>4.4</v>
       </c>
       <c r="CF8" t="n">
-        <v>4.45</v>
+        <v>4.4</v>
       </c>
       <c r="CG8" t="n">
         <v>14</v>
       </c>
       <c r="CH8" t="n">
-        <v>1847.88</v>
+        <v>1849.92</v>
       </c>
       <c r="CI8" t="n">
-        <v>4.02</v>
+        <v>4.14</v>
       </c>
       <c r="CJ8" t="n">
-        <v>3.21</v>
+        <v>3.71</v>
       </c>
       <c r="CK8" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="9">
@@ -21841,7 +21841,7 @@
         <v>13</v>
       </c>
       <c r="CD9" t="n">
-        <v>2696.66</v>
+        <v>2696.68</v>
       </c>
       <c r="CE9" t="n">
         <v>1.64</v>
@@ -21853,16 +21853,16 @@
         <v>14</v>
       </c>
       <c r="CH9" t="n">
-        <v>2695.85</v>
+        <v>2695.73</v>
       </c>
       <c r="CI9" t="n">
         <v>1.08</v>
       </c>
       <c r="CJ9" t="n">
-        <v>-0.12</v>
+        <v>-0.14</v>
       </c>
       <c r="CK9" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="10">
@@ -22120,28 +22120,28 @@
         <v>13</v>
       </c>
       <c r="CD10" t="n">
-        <v>2408.14</v>
+        <v>2408.06</v>
       </c>
       <c r="CE10" t="n">
         <v>1.13</v>
       </c>
       <c r="CF10" t="n">
-        <v>0.66</v>
+        <v>0.65</v>
       </c>
       <c r="CG10" t="n">
         <v>14</v>
       </c>
       <c r="CH10" t="n">
-        <v>2404.5</v>
+        <v>2404.28</v>
       </c>
       <c r="CI10" t="n">
-        <v>0.57</v>
+        <v>0.5600000000000001</v>
       </c>
       <c r="CJ10" t="n">
-        <v>-0.6</v>
+        <v>-0.63</v>
       </c>
       <c r="CK10" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="11">
@@ -22399,28 +22399,28 @@
         <v>13</v>
       </c>
       <c r="CD11" t="n">
-        <v>288.52</v>
+        <v>288.62</v>
       </c>
       <c r="CE11" t="n">
-        <v>6.1</v>
+        <v>6.14</v>
       </c>
       <c r="CF11" t="n">
-        <v>7.91</v>
+        <v>8.07</v>
       </c>
       <c r="CG11" t="n">
         <v>14</v>
       </c>
       <c r="CH11" t="n">
-        <v>291.34</v>
+        <v>291.44</v>
       </c>
       <c r="CI11" t="n">
-        <v>5.57</v>
+        <v>5.6</v>
       </c>
       <c r="CJ11" t="n">
         <v>3.97</v>
       </c>
       <c r="CK11" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="12">
@@ -22678,28 +22678,28 @@
         <v>13</v>
       </c>
       <c r="CD12" t="n">
-        <v>1919.37</v>
+        <v>1919.39</v>
       </c>
       <c r="CE12" t="n">
-        <v>5.08</v>
+        <v>5.09</v>
       </c>
       <c r="CF12" t="n">
-        <v>5.5</v>
+        <v>5.51</v>
       </c>
       <c r="CG12" t="n">
         <v>14</v>
       </c>
       <c r="CH12" t="n">
-        <v>1935.67</v>
+        <v>1937.05</v>
       </c>
       <c r="CI12" t="n">
-        <v>4.64</v>
+        <v>4.71</v>
       </c>
       <c r="CJ12" t="n">
-        <v>3.44</v>
+        <v>3.73</v>
       </c>
       <c r="CK12" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="13">
@@ -22957,7 +22957,7 @@
         <v>13</v>
       </c>
       <c r="CD13" t="n">
-        <v>1090.15</v>
+        <v>1090.16</v>
       </c>
       <c r="CE13" t="n">
         <v>4.08</v>
@@ -22969,16 +22969,16 @@
         <v>14</v>
       </c>
       <c r="CH13" t="n">
-        <v>1104.06</v>
+        <v>1105.01</v>
       </c>
       <c r="CI13" t="n">
-        <v>4.27</v>
+        <v>4.36</v>
       </c>
       <c r="CJ13" t="n">
-        <v>5.2</v>
+        <v>5.56</v>
       </c>
       <c r="CK13" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="14">
@@ -23236,28 +23236,28 @@
         <v>13</v>
       </c>
       <c r="CD14" t="n">
-        <v>829.22</v>
+        <v>829.24</v>
       </c>
       <c r="CE14" t="n">
         <v>6.43</v>
       </c>
       <c r="CF14" t="n">
-        <v>9.31</v>
+        <v>9.32</v>
       </c>
       <c r="CG14" t="n">
         <v>14</v>
       </c>
       <c r="CH14" t="n">
-        <v>831.61</v>
+        <v>832.04</v>
       </c>
       <c r="CI14" t="n">
-        <v>5.13</v>
+        <v>5.19</v>
       </c>
       <c r="CJ14" t="n">
-        <v>1.16</v>
+        <v>1.36</v>
       </c>
       <c r="CK14" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="15">
@@ -23515,28 +23515,28 @@
         <v>13</v>
       </c>
       <c r="CD15" t="n">
-        <v>524.1</v>
+        <v>524.11</v>
       </c>
       <c r="CE15" t="n">
         <v>6.29</v>
       </c>
       <c r="CF15" t="n">
-        <v>6.99</v>
+        <v>7</v>
       </c>
       <c r="CG15" t="n">
         <v>14</v>
       </c>
       <c r="CH15" t="n">
-        <v>524.4</v>
+        <v>524.46</v>
       </c>
       <c r="CI15" t="n">
-        <v>4.78</v>
+        <v>4.79</v>
       </c>
       <c r="CJ15" t="n">
-        <v>0.23</v>
+        <v>0.27</v>
       </c>
       <c r="CK15" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="16">
@@ -23794,28 +23794,28 @@
         <v>13</v>
       </c>
       <c r="CD16" t="n">
-        <v>2664.87</v>
+        <v>2666.68</v>
       </c>
       <c r="CE16" t="n">
-        <v>17.17</v>
+        <v>17.25</v>
       </c>
       <c r="CF16" t="n">
-        <v>11.13</v>
+        <v>11.43</v>
       </c>
       <c r="CG16" t="n">
         <v>14</v>
       </c>
       <c r="CH16" t="n">
-        <v>2729.57</v>
+        <v>2739.66</v>
       </c>
       <c r="CI16" t="n">
-        <v>14.82</v>
+        <v>15.24</v>
       </c>
       <c r="CJ16" t="n">
-        <v>10.07</v>
+        <v>11.4</v>
       </c>
       <c r="CK16" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="17">
@@ -24073,28 +24073,28 @@
         <v>13</v>
       </c>
       <c r="CD17" t="n">
-        <v>1509.57</v>
+        <v>1509.68</v>
       </c>
       <c r="CE17" t="n">
-        <v>22.53</v>
+        <v>22.54</v>
       </c>
       <c r="CF17" t="n">
-        <v>10.45</v>
+        <v>10.48</v>
       </c>
       <c r="CG17" t="n">
         <v>14</v>
       </c>
       <c r="CH17" t="n">
-        <v>1559.17</v>
+        <v>1562.81</v>
       </c>
       <c r="CI17" t="n">
-        <v>18.7</v>
+        <v>18.97</v>
       </c>
       <c r="CJ17" t="n">
-        <v>13.81</v>
+        <v>14.84</v>
       </c>
       <c r="CK17" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="18">
@@ -24352,28 +24352,28 @@
         <v>13</v>
       </c>
       <c r="CD18" t="n">
-        <v>17939.06</v>
+        <v>17938.38</v>
       </c>
       <c r="CE18" t="n">
-        <v>5.99</v>
+        <v>5.98</v>
       </c>
       <c r="CF18" t="n">
-        <v>4.57</v>
+        <v>4.55</v>
       </c>
       <c r="CG18" t="n">
         <v>14</v>
       </c>
       <c r="CH18" t="n">
-        <v>18129.3</v>
+        <v>18145.52</v>
       </c>
       <c r="CI18" t="n">
-        <v>5.85</v>
+        <v>5.94</v>
       </c>
       <c r="CJ18" t="n">
-        <v>4.31</v>
+        <v>4.7</v>
       </c>
       <c r="CK18" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="19">
@@ -24631,28 +24631,28 @@
         <v>13</v>
       </c>
       <c r="CD19" t="n">
-        <v>1633.07</v>
+        <v>1633.32</v>
       </c>
       <c r="CE19" t="n">
-        <v>5.97</v>
+        <v>5.98</v>
       </c>
       <c r="CF19" t="n">
-        <v>-0.76</v>
+        <v>-0.6899999999999999</v>
       </c>
       <c r="CG19" t="n">
         <v>14</v>
       </c>
       <c r="CH19" t="n">
-        <v>1662.12</v>
+        <v>1669.25</v>
       </c>
       <c r="CI19" t="n">
-        <v>5.75</v>
+        <v>6.2</v>
       </c>
       <c r="CJ19" t="n">
-        <v>7.31</v>
+        <v>9.09</v>
       </c>
       <c r="CK19" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="20">
@@ -24910,28 +24910,28 @@
         <v>13</v>
       </c>
       <c r="CD20" t="n">
-        <v>16306</v>
+        <v>16305.07</v>
       </c>
       <c r="CE20" t="n">
-        <v>5.99</v>
+        <v>5.98</v>
       </c>
       <c r="CF20" t="n">
-        <v>5.12</v>
+        <v>5.1</v>
       </c>
       <c r="CG20" t="n">
         <v>14</v>
       </c>
       <c r="CH20" t="n">
-        <v>16467.18</v>
+        <v>16476.27</v>
       </c>
       <c r="CI20" t="n">
-        <v>5.86</v>
+        <v>5.92</v>
       </c>
       <c r="CJ20" t="n">
-        <v>4.01</v>
+        <v>4.27</v>
       </c>
       <c r="CK20" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="21">
@@ -25201,16 +25201,16 @@
         <v>14</v>
       </c>
       <c r="CH21" t="n">
-        <v>7983.45</v>
+        <v>7991.58</v>
       </c>
       <c r="CI21" t="n">
-        <v>7.25</v>
+        <v>7.36</v>
       </c>
       <c r="CJ21" t="n">
-        <v>5.8</v>
+        <v>6.23</v>
       </c>
       <c r="CK21" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="22">
@@ -25480,16 +25480,16 @@
         <v>14</v>
       </c>
       <c r="CH22" t="n">
-        <v>1616.81</v>
+        <v>1615.89</v>
       </c>
       <c r="CI22" t="n">
-        <v>11.22</v>
+        <v>11.16</v>
       </c>
       <c r="CJ22" t="n">
-        <v>11.35</v>
+        <v>11.1</v>
       </c>
       <c r="CK22" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="23">
@@ -25759,16 +25759,16 @@
         <v>14</v>
       </c>
       <c r="CH23" t="n">
-        <v>915.78</v>
+        <v>917.08</v>
       </c>
       <c r="CI23" t="n">
-        <v>3.15</v>
+        <v>3.3</v>
       </c>
       <c r="CJ23" t="n">
-        <v>4.53</v>
+        <v>5.12</v>
       </c>
       <c r="CK23" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="24">
@@ -26038,16 +26038,16 @@
         <v>14</v>
       </c>
       <c r="CH24" t="n">
-        <v>125.77</v>
+        <v>125.61</v>
       </c>
       <c r="CI24" t="n">
-        <v>-1.14</v>
+        <v>-1.26</v>
       </c>
       <c r="CJ24" t="n">
-        <v>4.52</v>
+        <v>4.01</v>
       </c>
       <c r="CK24" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="25">
@@ -26317,16 +26317,16 @@
         <v>14</v>
       </c>
       <c r="CH25" t="n">
-        <v>6.26</v>
+        <v>6.25</v>
       </c>
       <c r="CI25" t="n">
-        <v>-2.12</v>
+        <v>-2.3</v>
       </c>
       <c r="CJ25" t="n">
-        <v>-1.13</v>
+        <v>-1.86</v>
       </c>
       <c r="CK25" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="26">
@@ -26596,16 +26596,16 @@
         <v>14</v>
       </c>
       <c r="CH26" t="n">
-        <v>255.22</v>
+        <v>254.97</v>
       </c>
       <c r="CI26" t="n">
-        <v>5.9</v>
+        <v>5.79</v>
       </c>
       <c r="CJ26" t="n">
-        <v>7.05</v>
+        <v>6.62</v>
       </c>
       <c r="CK26" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="27">
@@ -26875,16 +26875,16 @@
         <v>14</v>
       </c>
       <c r="CH27" t="n">
-        <v>528.52</v>
+        <v>530.25</v>
       </c>
       <c r="CI27" t="n">
-        <v>2.99</v>
+        <v>3.33</v>
       </c>
       <c r="CJ27" t="n">
-        <v>3.41</v>
+        <v>4.76</v>
       </c>
       <c r="CK27" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="28">
@@ -27154,16 +27154,16 @@
         <v>14</v>
       </c>
       <c r="CH28" t="n">
-        <v>1656.65</v>
+        <v>1656.95</v>
       </c>
       <c r="CI28" t="n">
-        <v>-0.03</v>
+        <v>-0.02</v>
       </c>
       <c r="CJ28" t="n">
-        <v>-0.75</v>
+        <v>-0.68</v>
       </c>
       <c r="CK28" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="29">
@@ -27433,16 +27433,16 @@
         <v>14</v>
       </c>
       <c r="CH29" t="n">
-        <v>1495.27</v>
+        <v>1495.46</v>
       </c>
       <c r="CI29" t="n">
-        <v>-0.29</v>
+        <v>-0.27</v>
       </c>
       <c r="CJ29" t="n">
-        <v>-1.04</v>
+        <v>-0.99</v>
       </c>
       <c r="CK29" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="30">
@@ -27712,16 +27712,16 @@
         <v>14</v>
       </c>
       <c r="CH30" t="n">
-        <v>161.38</v>
+        <v>161.49</v>
       </c>
       <c r="CI30" t="n">
-        <v>2.37</v>
+        <v>2.44</v>
       </c>
       <c r="CJ30" t="n">
-        <v>1.97</v>
+        <v>2.25</v>
       </c>
       <c r="CK30" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="31">
@@ -27991,16 +27991,16 @@
         <v>14</v>
       </c>
       <c r="CH31" t="n">
-        <v>1583.32</v>
+        <v>1583.94</v>
       </c>
       <c r="CI31" t="n">
-        <v>3.29</v>
+        <v>3.33</v>
       </c>
       <c r="CJ31" t="n">
-        <v>0.55</v>
+        <v>0.71</v>
       </c>
       <c r="CK31" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="32">
@@ -28270,16 +28270,16 @@
         <v>14</v>
       </c>
       <c r="CH32" t="n">
-        <v>1000.63</v>
+        <v>1001.35</v>
       </c>
       <c r="CI32" t="n">
-        <v>4.06</v>
+        <v>4.14</v>
       </c>
       <c r="CJ32" t="n">
-        <v>2.32</v>
+        <v>2.62</v>
       </c>
       <c r="CK32" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="33">
@@ -28549,16 +28549,16 @@
         <v>14</v>
       </c>
       <c r="CH33" t="n">
-        <v>582.6900000000001</v>
+        <v>582.59</v>
       </c>
       <c r="CI33" t="n">
-        <v>1.98</v>
+        <v>1.96</v>
       </c>
       <c r="CJ33" t="n">
-        <v>-2.41</v>
+        <v>-2.48</v>
       </c>
       <c r="CK33" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="34">
@@ -28828,16 +28828,16 @@
         <v>14</v>
       </c>
       <c r="CH34" t="n">
-        <v>436.32</v>
+        <v>436.23</v>
       </c>
       <c r="CI34" t="n">
-        <v>2.97</v>
+        <v>2.95</v>
       </c>
       <c r="CJ34" t="n">
-        <v>-1.99</v>
+        <v>-2.07</v>
       </c>
       <c r="CK34" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="35">
@@ -29107,16 +29107,16 @@
         <v>14</v>
       </c>
       <c r="CH35" t="n">
-        <v>2210.88</v>
+        <v>2217.72</v>
       </c>
       <c r="CI35" t="n">
-        <v>15.64</v>
+        <v>16</v>
       </c>
       <c r="CJ35" t="n">
-        <v>11.57</v>
+        <v>12.96</v>
       </c>
       <c r="CK35" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="36">
@@ -29386,16 +29386,16 @@
         <v>14</v>
       </c>
       <c r="CH36" t="n">
-        <v>1358.51</v>
+        <v>1361.24</v>
       </c>
       <c r="CI36" t="n">
-        <v>18.93</v>
+        <v>19.17</v>
       </c>
       <c r="CJ36" t="n">
-        <v>15.22</v>
+        <v>16.15</v>
       </c>
       <c r="CK36" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="37">
@@ -29665,16 +29665,16 @@
         <v>14</v>
       </c>
       <c r="CH37" t="n">
-        <v>12441.01</v>
+        <v>12453.63</v>
       </c>
       <c r="CI37" t="n">
-        <v>6.78</v>
+        <v>6.89</v>
       </c>
       <c r="CJ37" t="n">
-        <v>5.53</v>
+        <v>5.96</v>
       </c>
       <c r="CK37" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="38">
@@ -29944,16 +29944,16 @@
         <v>14</v>
       </c>
       <c r="CH38" t="n">
-        <v>914.62</v>
+        <v>922.95</v>
       </c>
       <c r="CI38" t="n">
-        <v>10.7</v>
+        <v>11.71</v>
       </c>
       <c r="CJ38" t="n">
-        <v>8.01</v>
+        <v>12</v>
       </c>
       <c r="CK38" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="39">
@@ -30223,16 +30223,16 @@
         <v>14</v>
       </c>
       <c r="CH39" t="n">
-        <v>11526.39</v>
+        <v>11530.68</v>
       </c>
       <c r="CI39" t="n">
-        <v>6.48</v>
+        <v>6.52</v>
       </c>
       <c r="CJ39" t="n">
-        <v>5.33</v>
+        <v>5.49</v>
       </c>
       <c r="CK39" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="40">
@@ -30490,28 +30490,28 @@
         <v>13</v>
       </c>
       <c r="CD40" t="n">
-        <v>4722.53</v>
+        <v>4722.8</v>
       </c>
       <c r="CE40" t="n">
-        <v>5.38</v>
+        <v>5.39</v>
       </c>
       <c r="CF40" t="n">
-        <v>5.7</v>
+        <v>5.72</v>
       </c>
       <c r="CG40" t="n">
         <v>14</v>
       </c>
       <c r="CH40" t="n">
-        <v>4768.51</v>
+        <v>4771.49</v>
       </c>
       <c r="CI40" t="n">
-        <v>5.07</v>
+        <v>5.14</v>
       </c>
       <c r="CJ40" t="n">
-        <v>3.95</v>
+        <v>4.19</v>
       </c>
       <c r="CK40" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="41">
@@ -30769,28 +30769,28 @@
         <v>13</v>
       </c>
       <c r="CD41" t="n">
-        <v>733.67</v>
+        <v>733.39</v>
       </c>
       <c r="CE41" t="n">
-        <v>5.1</v>
+        <v>5.06</v>
       </c>
       <c r="CF41" t="n">
-        <v>8.24</v>
+        <v>8.07</v>
       </c>
       <c r="CG41" t="n">
         <v>14</v>
       </c>
       <c r="CH41" t="n">
-        <v>742.22</v>
+        <v>742.12</v>
       </c>
       <c r="CI41" t="n">
-        <v>5.78</v>
+        <v>5.76</v>
       </c>
       <c r="CJ41" t="n">
-        <v>4.74</v>
+        <v>4.85</v>
       </c>
       <c r="CK41" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="42">
@@ -31048,28 +31048,28 @@
         <v>13</v>
       </c>
       <c r="CD42" t="n">
-        <v>2100.07</v>
+        <v>2098.77</v>
       </c>
       <c r="CE42" t="n">
-        <v>3.58</v>
+        <v>3.52</v>
       </c>
       <c r="CF42" t="n">
-        <v>3.85</v>
+        <v>3.59</v>
       </c>
       <c r="CG42" t="n">
         <v>14</v>
       </c>
       <c r="CH42" t="n">
-        <v>2116.06</v>
+        <v>2115.55</v>
       </c>
       <c r="CI42" t="n">
-        <v>3.49</v>
+        <v>3.47</v>
       </c>
       <c r="CJ42" t="n">
-        <v>3.08</v>
+        <v>3.24</v>
       </c>
       <c r="CK42" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="43">
@@ -31327,28 +31327,28 @@
         <v>13</v>
       </c>
       <c r="CD43" t="n">
-        <v>307.23</v>
+        <v>307.32</v>
       </c>
       <c r="CE43" t="n">
-        <v>-1.19</v>
+        <v>-1.17</v>
       </c>
       <c r="CF43" t="n">
-        <v>3.66</v>
+        <v>3.77</v>
       </c>
       <c r="CG43" t="n">
         <v>14</v>
       </c>
       <c r="CH43" t="n">
-        <v>310.39</v>
+        <v>310.16</v>
       </c>
       <c r="CI43" t="n">
-        <v>0.8100000000000001</v>
+        <v>0.73</v>
       </c>
       <c r="CJ43" t="n">
-        <v>4.17</v>
+        <v>3.76</v>
       </c>
       <c r="CK43" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="44">
@@ -31606,28 +31606,28 @@
         <v>13</v>
       </c>
       <c r="CD44" t="n">
-        <v>116.27</v>
+        <v>116.26</v>
       </c>
       <c r="CE44" t="n">
-        <v>4.71</v>
+        <v>4.7</v>
       </c>
       <c r="CF44" t="n">
-        <v>4.85</v>
+        <v>4.8</v>
       </c>
       <c r="CG44" t="n">
         <v>14</v>
       </c>
       <c r="CH44" t="n">
-        <v>117.25</v>
+        <v>117.19</v>
       </c>
       <c r="CI44" t="n">
-        <v>4.74</v>
+        <v>4.69</v>
       </c>
       <c r="CJ44" t="n">
-        <v>3.38</v>
+        <v>3.24</v>
       </c>
       <c r="CK44" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="45">
@@ -31885,28 +31885,28 @@
         <v>13</v>
       </c>
       <c r="CD45" t="n">
-        <v>367.34</v>
+        <v>366.15</v>
       </c>
       <c r="CE45" t="n">
-        <v>2.45</v>
+        <v>2.12</v>
       </c>
       <c r="CF45" t="n">
-        <v>1.87</v>
+        <v>0.5600000000000001</v>
       </c>
       <c r="CG45" t="n">
         <v>14</v>
       </c>
       <c r="CH45" t="n">
-        <v>369.07</v>
+        <v>368.53</v>
       </c>
       <c r="CI45" t="n">
-        <v>2.07</v>
+        <v>1.92</v>
       </c>
       <c r="CJ45" t="n">
-        <v>1.9</v>
+        <v>2.62</v>
       </c>
       <c r="CK45" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="46">
@@ -32164,28 +32164,28 @@
         <v>13</v>
       </c>
       <c r="CD46" t="n">
-        <v>1309.22</v>
+        <v>1309.04</v>
       </c>
       <c r="CE46" t="n">
-        <v>5</v>
+        <v>4.98</v>
       </c>
       <c r="CF46" t="n">
-        <v>4.37</v>
+        <v>4.31</v>
       </c>
       <c r="CG46" t="n">
         <v>14</v>
       </c>
       <c r="CH46" t="n">
-        <v>1319.36</v>
+        <v>1319.67</v>
       </c>
       <c r="CI46" t="n">
-        <v>4.44</v>
+        <v>4.47</v>
       </c>
       <c r="CJ46" t="n">
-        <v>3.13</v>
+        <v>3.29</v>
       </c>
       <c r="CK46" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="47">
@@ -32443,7 +32443,7 @@
         <v>13</v>
       </c>
       <c r="CD47" t="n">
-        <v>1036.9</v>
+        <v>1036.92</v>
       </c>
       <c r="CE47" t="n">
         <v>3.72</v>
@@ -32455,16 +32455,16 @@
         <v>14</v>
       </c>
       <c r="CH47" t="n">
-        <v>1039.2</v>
+        <v>1038.78</v>
       </c>
       <c r="CI47" t="n">
-        <v>2.92</v>
+        <v>2.87</v>
       </c>
       <c r="CJ47" t="n">
-        <v>0.89</v>
+        <v>0.72</v>
       </c>
       <c r="CK47" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="48">
@@ -32722,28 +32722,28 @@
         <v>13</v>
       </c>
       <c r="CD48" t="n">
-        <v>908.97</v>
+        <v>908.89</v>
       </c>
       <c r="CE48" t="n">
-        <v>2.75</v>
+        <v>2.74</v>
       </c>
       <c r="CF48" t="n">
-        <v>2.31</v>
+        <v>2.27</v>
       </c>
       <c r="CG48" t="n">
         <v>14</v>
       </c>
       <c r="CH48" t="n">
-        <v>909.23</v>
+        <v>908.83</v>
       </c>
       <c r="CI48" t="n">
+        <v>1.95</v>
+      </c>
+      <c r="CJ48" t="n">
+        <v>-0.03</v>
+      </c>
+      <c r="CK48" t="n">
         <v>2</v>
-      </c>
-      <c r="CJ48" t="n">
-        <v>0.12</v>
-      </c>
-      <c r="CK48" t="n">
-        <v>1</v>
       </c>
     </row>
     <row r="49">
@@ -33001,28 +33001,28 @@
         <v>13</v>
       </c>
       <c r="CD49" t="n">
-        <v>127.93</v>
+        <v>128.03</v>
       </c>
       <c r="CE49" t="n">
-        <v>11.11</v>
+        <v>11.2</v>
       </c>
       <c r="CF49" t="n">
-        <v>11.93</v>
+        <v>12.29</v>
       </c>
       <c r="CG49" t="n">
         <v>14</v>
       </c>
       <c r="CH49" t="n">
-        <v>129.96</v>
+        <v>129.95</v>
       </c>
       <c r="CI49" t="n">
         <v>9.83</v>
       </c>
       <c r="CJ49" t="n">
-        <v>6.52</v>
+        <v>6.15</v>
       </c>
       <c r="CK49" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="50">
@@ -33280,28 +33280,28 @@
         <v>13</v>
       </c>
       <c r="CD50" t="n">
-        <v>338.21</v>
+        <v>338.23</v>
       </c>
       <c r="CE50" t="n">
-        <v>8.82</v>
+        <v>8.83</v>
       </c>
       <c r="CF50" t="n">
-        <v>14.5</v>
+        <v>14.54</v>
       </c>
       <c r="CG50" t="n">
         <v>14</v>
       </c>
       <c r="CH50" t="n">
-        <v>352.34</v>
+        <v>353.11</v>
       </c>
       <c r="CI50" t="n">
-        <v>11.19</v>
+        <v>11.43</v>
       </c>
       <c r="CJ50" t="n">
-        <v>17.8</v>
+        <v>18.78</v>
       </c>
       <c r="CK50" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="51">
@@ -33559,28 +33559,28 @@
         <v>13</v>
       </c>
       <c r="CD51" t="n">
-        <v>95.25</v>
+        <v>95.26000000000001</v>
       </c>
       <c r="CE51" t="n">
-        <v>-0.07000000000000001</v>
+        <v>-0.06</v>
       </c>
       <c r="CF51" t="n">
-        <v>-4.59</v>
+        <v>-4.56</v>
       </c>
       <c r="CG51" t="n">
         <v>14</v>
       </c>
       <c r="CH51" t="n">
-        <v>103.43</v>
+        <v>103.66</v>
       </c>
       <c r="CI51" t="n">
-        <v>6.35</v>
+        <v>6.59</v>
       </c>
       <c r="CJ51" t="n">
-        <v>39.02</v>
+        <v>40.2</v>
       </c>
       <c r="CK51" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="52">
@@ -33838,28 +33838,28 @@
         <v>13</v>
       </c>
       <c r="CD52" t="n">
-        <v>242.95</v>
+        <v>242.97</v>
       </c>
       <c r="CE52" t="n">
-        <v>12.76</v>
+        <v>12.77</v>
       </c>
       <c r="CF52" t="n">
-        <v>23.28</v>
+        <v>23.31</v>
       </c>
       <c r="CG52" t="n">
         <v>14</v>
       </c>
       <c r="CH52" t="n">
-        <v>248.91</v>
+        <v>249.45</v>
       </c>
       <c r="CI52" t="n">
-        <v>13.33</v>
+        <v>13.57</v>
       </c>
       <c r="CJ52" t="n">
-        <v>10.18</v>
+        <v>11.09</v>
       </c>
       <c r="CK52" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="53">
@@ -34120,25 +34120,25 @@
         <v>85.58</v>
       </c>
       <c r="CE53" t="n">
-        <v>12.83</v>
+        <v>12.84</v>
       </c>
       <c r="CF53" t="n">
-        <v>25.43</v>
+        <v>25.45</v>
       </c>
       <c r="CG53" t="n">
         <v>14</v>
       </c>
       <c r="CH53" t="n">
-        <v>88.08</v>
+        <v>88.22</v>
       </c>
       <c r="CI53" t="n">
-        <v>14.74</v>
+        <v>14.93</v>
       </c>
       <c r="CJ53" t="n">
-        <v>12.21</v>
+        <v>12.93</v>
       </c>
       <c r="CK53" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="54">
@@ -34396,28 +34396,28 @@
         <v>13</v>
       </c>
       <c r="CD54" t="n">
-        <v>513.6900000000001</v>
+        <v>515.5</v>
       </c>
       <c r="CE54" t="n">
-        <v>15.37</v>
+        <v>15.77</v>
       </c>
       <c r="CF54" t="n">
-        <v>8.92</v>
+        <v>10.46</v>
       </c>
       <c r="CG54" t="n">
         <v>14</v>
       </c>
       <c r="CH54" t="n">
-        <v>518.6900000000001</v>
+        <v>521.9400000000001</v>
       </c>
       <c r="CI54" t="n">
-        <v>11.45</v>
+        <v>12.15</v>
       </c>
       <c r="CJ54" t="n">
-        <v>3.95</v>
+        <v>5.09</v>
       </c>
       <c r="CK54" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="55">
@@ -34675,28 +34675,28 @@
         <v>13</v>
       </c>
       <c r="CD55" t="n">
-        <v>198.32</v>
+        <v>198.43</v>
       </c>
       <c r="CE55" t="n">
-        <v>27.46</v>
+        <v>27.53</v>
       </c>
       <c r="CF55" t="n">
-        <v>5.26</v>
+        <v>5.48</v>
       </c>
       <c r="CG55" t="n">
         <v>14</v>
       </c>
       <c r="CH55" t="n">
-        <v>200.67</v>
+        <v>201.56</v>
       </c>
       <c r="CI55" t="n">
-        <v>17.11</v>
+        <v>17.63</v>
       </c>
       <c r="CJ55" t="n">
-        <v>4.8</v>
+        <v>6.46</v>
       </c>
       <c r="CK55" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="56">
@@ -34954,28 +34954,28 @@
         <v>13</v>
       </c>
       <c r="CD56" t="n">
-        <v>5664.27</v>
+        <v>5663.59</v>
       </c>
       <c r="CE56" t="n">
-        <v>4.58</v>
+        <v>4.57</v>
       </c>
       <c r="CF56" t="n">
-        <v>3.46</v>
+        <v>3.41</v>
       </c>
       <c r="CG56" t="n">
         <v>14</v>
       </c>
       <c r="CH56" t="n">
-        <v>5688.29</v>
+        <v>5691.89</v>
       </c>
       <c r="CI56" t="n">
-        <v>3.86</v>
+        <v>3.92</v>
       </c>
       <c r="CJ56" t="n">
-        <v>1.71</v>
+        <v>2.01</v>
       </c>
       <c r="CK56" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="57">
@@ -35233,28 +35233,28 @@
         <v>13</v>
       </c>
       <c r="CD57" t="n">
-        <v>735.9</v>
+        <v>736.15</v>
       </c>
       <c r="CE57" t="n">
-        <v>0.19</v>
+        <v>0.23</v>
       </c>
       <c r="CF57" t="n">
-        <v>-0.01</v>
+        <v>0.13</v>
       </c>
       <c r="CG57" t="n">
         <v>14</v>
       </c>
       <c r="CH57" t="n">
-        <v>747.5</v>
+        <v>746.3</v>
       </c>
       <c r="CI57" t="n">
-        <v>0.27</v>
+        <v>0.11</v>
       </c>
       <c r="CJ57" t="n">
-        <v>6.46</v>
+        <v>5.63</v>
       </c>
       <c r="CK57" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="58">
@@ -35512,28 +35512,28 @@
         <v>13</v>
       </c>
       <c r="CD58" t="n">
-        <v>4928.37</v>
+        <v>4927.44</v>
       </c>
       <c r="CE58" t="n">
-        <v>5.27</v>
+        <v>5.25</v>
       </c>
       <c r="CF58" t="n">
-        <v>3.99</v>
+        <v>3.91</v>
       </c>
       <c r="CG58" t="n">
         <v>14</v>
       </c>
       <c r="CH58" t="n">
-        <v>4940.79</v>
+        <v>4945.59</v>
       </c>
       <c r="CI58" t="n">
-        <v>4.42</v>
+        <v>4.53</v>
       </c>
       <c r="CJ58" t="n">
-        <v>1.01</v>
+        <v>1.48</v>
       </c>
       <c r="CK58" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="60">

</xml_diff>

<commit_message>
data: refresh 2026-10-30 20:44 UTC
</commit_message>
<xml_diff>
--- a/data/h8-growth5y.xlsx
+++ b/data/h8-growth5y.xlsx
@@ -1161,13 +1161,13 @@
         </is>
       </c>
       <c r="CD2" t="n">
-        <v>12709</v>
+        <v>12710.04</v>
       </c>
       <c r="CE2" t="n">
-        <v>6.94</v>
+        <v>6.95</v>
       </c>
       <c r="CF2" t="n">
-        <v>7.03</v>
+        <v>7.06</v>
       </c>
       <c r="CG2" t="inlineStr">
         <is>
@@ -1175,17 +1175,17 @@
         </is>
       </c>
       <c r="CH2" t="n">
-        <v>12772.34</v>
+        <v>12769.36</v>
       </c>
       <c r="CI2" t="n">
-        <v>5.91</v>
+        <v>5.88</v>
       </c>
       <c r="CJ2" t="n">
-        <v>2.01</v>
+        <v>1.88</v>
       </c>
       <c r="CK2" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-21</t>
         </is>
       </c>
     </row>
@@ -1482,7 +1482,7 @@
         </is>
       </c>
       <c r="CD3" t="n">
-        <v>2336.89</v>
+        <v>2336.9</v>
       </c>
       <c r="CE3" t="n">
         <v>8.210000000000001</v>
@@ -1496,17 +1496,17 @@
         </is>
       </c>
       <c r="CH3" t="n">
-        <v>2357.01</v>
+        <v>2356.91</v>
       </c>
       <c r="CI3" t="n">
         <v>9.27</v>
       </c>
       <c r="CJ3" t="n">
-        <v>3.49</v>
+        <v>3.47</v>
       </c>
       <c r="CK3" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-21</t>
         </is>
       </c>
     </row>
@@ -1803,13 +1803,13 @@
         </is>
       </c>
       <c r="CD4" t="n">
-        <v>3024.66</v>
+        <v>3025.06</v>
       </c>
       <c r="CE4" t="n">
-        <v>3.8</v>
+        <v>3.81</v>
       </c>
       <c r="CF4" t="n">
-        <v>4.79</v>
+        <v>4.85</v>
       </c>
       <c r="CG4" t="inlineStr">
         <is>
@@ -1817,17 +1817,17 @@
         </is>
       </c>
       <c r="CH4" t="n">
-        <v>3034.05</v>
+        <v>3025.83</v>
       </c>
       <c r="CI4" t="n">
-        <v>3.08</v>
+        <v>2.8</v>
       </c>
       <c r="CJ4" t="n">
-        <v>1.25</v>
+        <v>0.1</v>
       </c>
       <c r="CK4" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-21</t>
         </is>
       </c>
     </row>
@@ -2124,13 +2124,13 @@
         </is>
       </c>
       <c r="CD5" t="n">
-        <v>434.13</v>
+        <v>433.99</v>
       </c>
       <c r="CE5" t="n">
-        <v>-1.14</v>
+        <v>-1.18</v>
       </c>
       <c r="CF5" t="n">
-        <v>8.49</v>
+        <v>8.35</v>
       </c>
       <c r="CG5" t="inlineStr">
         <is>
@@ -2138,17 +2138,17 @@
         </is>
       </c>
       <c r="CH5" t="n">
-        <v>435.31</v>
+        <v>436.05</v>
       </c>
       <c r="CI5" t="n">
-        <v>0.41</v>
+        <v>0.58</v>
       </c>
       <c r="CJ5" t="n">
-        <v>1.09</v>
+        <v>1.92</v>
       </c>
       <c r="CK5" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-21</t>
         </is>
       </c>
     </row>
@@ -2445,13 +2445,13 @@
         </is>
       </c>
       <c r="CD6" t="n">
-        <v>123.33</v>
+        <v>123.39</v>
       </c>
       <c r="CE6" t="n">
-        <v>5</v>
+        <v>5.05</v>
       </c>
       <c r="CF6" t="n">
-        <v>5.93</v>
+        <v>6.16</v>
       </c>
       <c r="CG6" t="inlineStr">
         <is>
@@ -2459,17 +2459,17 @@
         </is>
       </c>
       <c r="CH6" t="n">
-        <v>123.47</v>
+        <v>123.48</v>
       </c>
       <c r="CI6" t="n">
-        <v>3.78</v>
+        <v>3.8</v>
       </c>
       <c r="CJ6" t="n">
-        <v>0.46</v>
+        <v>0.31</v>
       </c>
       <c r="CK6" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-21</t>
         </is>
       </c>
     </row>
@@ -2766,13 +2766,13 @@
         </is>
       </c>
       <c r="CD7" t="n">
-        <v>621.38</v>
+        <v>621.91</v>
       </c>
       <c r="CE7" t="n">
-        <v>4.59</v>
+        <v>4.68</v>
       </c>
       <c r="CF7" t="n">
-        <v>2.79</v>
+        <v>3.14</v>
       </c>
       <c r="CG7" t="inlineStr">
         <is>
@@ -2780,17 +2780,17 @@
         </is>
       </c>
       <c r="CH7" t="n">
-        <v>623.28</v>
+        <v>621.34</v>
       </c>
       <c r="CI7" t="n">
-        <v>2.95</v>
+        <v>2.63</v>
       </c>
       <c r="CJ7" t="n">
-        <v>1.23</v>
+        <v>-0.36</v>
       </c>
       <c r="CK7" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-21</t>
         </is>
       </c>
     </row>
@@ -3087,13 +3087,13 @@
         </is>
       </c>
       <c r="CD8" t="n">
-        <v>1845.82</v>
+        <v>1845.78</v>
       </c>
       <c r="CE8" t="n">
         <v>4.68</v>
       </c>
       <c r="CF8" t="n">
-        <v>4.55</v>
+        <v>4.54</v>
       </c>
       <c r="CG8" t="inlineStr">
         <is>
@@ -3101,17 +3101,17 @@
         </is>
       </c>
       <c r="CH8" t="n">
-        <v>1852</v>
+        <v>1844.95</v>
       </c>
       <c r="CI8" t="n">
-        <v>3.72</v>
+        <v>3.32</v>
       </c>
       <c r="CJ8" t="n">
-        <v>1.34</v>
+        <v>-0.18</v>
       </c>
       <c r="CK8" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-21</t>
         </is>
       </c>
     </row>
@@ -3408,13 +3408,13 @@
         </is>
       </c>
       <c r="CD9" t="n">
-        <v>2697.47</v>
+        <v>2697.56</v>
       </c>
       <c r="CE9" t="n">
-        <v>1.49</v>
+        <v>1.5</v>
       </c>
       <c r="CF9" t="n">
-        <v>0.34</v>
+        <v>0.35</v>
       </c>
       <c r="CG9" t="inlineStr">
         <is>
@@ -3422,17 +3422,17 @@
         </is>
       </c>
       <c r="CH9" t="n">
-        <v>2695.49</v>
+        <v>2704.54</v>
       </c>
       <c r="CI9" t="n">
-        <v>0.88</v>
+        <v>1.22</v>
       </c>
       <c r="CJ9" t="n">
-        <v>-0.29</v>
+        <v>1.04</v>
       </c>
       <c r="CK9" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-21</t>
         </is>
       </c>
     </row>
@@ -3729,13 +3729,13 @@
         </is>
       </c>
       <c r="CD10" t="n">
-        <v>2406.39</v>
+        <v>2406.48</v>
       </c>
       <c r="CE10" t="n">
         <v>0.93</v>
       </c>
       <c r="CF10" t="n">
-        <v>-0.54</v>
+        <v>-0.53</v>
       </c>
       <c r="CG10" t="inlineStr">
         <is>
@@ -3743,17 +3743,17 @@
         </is>
       </c>
       <c r="CH10" t="n">
-        <v>2404.02</v>
+        <v>2413.01</v>
       </c>
       <c r="CI10" t="n">
-        <v>0.4</v>
+        <v>0.78</v>
       </c>
       <c r="CJ10" t="n">
-        <v>-0.39</v>
+        <v>1.09</v>
       </c>
       <c r="CK10" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-21</t>
         </is>
       </c>
     </row>
@@ -4064,17 +4064,17 @@
         </is>
       </c>
       <c r="CH11" t="n">
-        <v>291.47</v>
+        <v>291.53</v>
       </c>
       <c r="CI11" t="n">
-        <v>5.01</v>
+        <v>5.03</v>
       </c>
       <c r="CJ11" t="n">
-        <v>0.54</v>
+        <v>0.61</v>
       </c>
       <c r="CK11" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-21</t>
         </is>
       </c>
     </row>
@@ -4371,13 +4371,13 @@
         </is>
       </c>
       <c r="CD12" t="n">
-        <v>1927.84</v>
+        <v>1928.39</v>
       </c>
       <c r="CE12" t="n">
-        <v>4.96</v>
+        <v>4.99</v>
       </c>
       <c r="CF12" t="n">
-        <v>5.14</v>
+        <v>5.26</v>
       </c>
       <c r="CG12" t="inlineStr">
         <is>
@@ -4385,17 +4385,17 @@
         </is>
       </c>
       <c r="CH12" t="n">
-        <v>1938.17</v>
+        <v>1932.06</v>
       </c>
       <c r="CI12" t="n">
-        <v>4.29</v>
+        <v>3.96</v>
       </c>
       <c r="CJ12" t="n">
-        <v>2.16</v>
+        <v>0.76</v>
       </c>
       <c r="CK12" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-21</t>
         </is>
       </c>
     </row>
@@ -4692,13 +4692,13 @@
         </is>
       </c>
       <c r="CD13" t="n">
-        <v>1096.41</v>
+        <v>1097.01</v>
       </c>
       <c r="CE13" t="n">
-        <v>4.27</v>
+        <v>4.33</v>
       </c>
       <c r="CF13" t="n">
-        <v>3.2</v>
+        <v>3.43</v>
       </c>
       <c r="CG13" t="inlineStr">
         <is>
@@ -4706,17 +4706,17 @@
         </is>
       </c>
       <c r="CH13" t="n">
-        <v>1105.85</v>
+        <v>1099.87</v>
       </c>
       <c r="CI13" t="n">
-        <v>3.99</v>
+        <v>3.43</v>
       </c>
       <c r="CJ13" t="n">
-        <v>3.49</v>
+        <v>1.05</v>
       </c>
       <c r="CK13" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-21</t>
         </is>
       </c>
     </row>
@@ -5013,13 +5013,13 @@
         </is>
       </c>
       <c r="CD14" t="n">
-        <v>831.42</v>
+        <v>831.38</v>
       </c>
       <c r="CE14" t="n">
-        <v>5.89</v>
+        <v>5.88</v>
       </c>
       <c r="CF14" t="n">
-        <v>7.77</v>
+        <v>7.75</v>
       </c>
       <c r="CG14" t="inlineStr">
         <is>
@@ -5027,17 +5027,17 @@
         </is>
       </c>
       <c r="CH14" t="n">
-        <v>832.3200000000001</v>
+        <v>832.1900000000001</v>
       </c>
       <c r="CI14" t="n">
-        <v>4.7</v>
+        <v>4.68</v>
       </c>
       <c r="CJ14" t="n">
-        <v>0.43</v>
+        <v>0.39</v>
       </c>
       <c r="CK14" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-21</t>
         </is>
       </c>
     </row>
@@ -5348,17 +5348,17 @@
         </is>
       </c>
       <c r="CH15" t="n">
-        <v>524.49</v>
+        <v>524.63</v>
       </c>
       <c r="CI15" t="n">
-        <v>3.83</v>
+        <v>3.86</v>
       </c>
       <c r="CJ15" t="n">
-        <v>0.04</v>
+        <v>0.15</v>
       </c>
       <c r="CK15" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-21</t>
         </is>
       </c>
     </row>
@@ -5669,17 +5669,17 @@
         </is>
       </c>
       <c r="CH16" t="n">
-        <v>2747.61</v>
+        <v>2750.02</v>
       </c>
       <c r="CI16" t="n">
-        <v>13.12</v>
+        <v>13.22</v>
       </c>
       <c r="CJ16" t="n">
-        <v>3.8</v>
+        <v>4.16</v>
       </c>
       <c r="CK16" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-21</t>
         </is>
       </c>
     </row>
@@ -5990,17 +5990,17 @@
         </is>
       </c>
       <c r="CH17" t="n">
-        <v>1566.27</v>
+        <v>1578.51</v>
       </c>
       <c r="CI17" t="n">
-        <v>14.95</v>
+        <v>15.84</v>
       </c>
       <c r="CJ17" t="n">
-        <v>4.92</v>
+        <v>8.24</v>
       </c>
       <c r="CK17" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-21</t>
         </is>
       </c>
     </row>
@@ -6297,7 +6297,7 @@
         </is>
       </c>
       <c r="CD18" t="n">
-        <v>18089.34</v>
+        <v>18089.53</v>
       </c>
       <c r="CE18" t="n">
         <v>6.28</v>
@@ -6311,17 +6311,17 @@
         </is>
       </c>
       <c r="CH18" t="n">
-        <v>18161.6</v>
+        <v>18125.25</v>
       </c>
       <c r="CI18" t="n">
-        <v>5.78</v>
+        <v>5.56</v>
       </c>
       <c r="CJ18" t="n">
-        <v>1.61</v>
+        <v>0.79</v>
       </c>
       <c r="CK18" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-21</t>
         </is>
       </c>
     </row>
@@ -6618,13 +6618,13 @@
         </is>
       </c>
       <c r="CD19" t="n">
-        <v>1654.67</v>
+        <v>1655.46</v>
       </c>
       <c r="CE19" t="n">
-        <v>7.35</v>
+        <v>7.4</v>
       </c>
       <c r="CF19" t="n">
-        <v>9.300000000000001</v>
+        <v>9.5</v>
       </c>
       <c r="CG19" t="inlineStr">
         <is>
@@ -6632,17 +6632,17 @@
         </is>
       </c>
       <c r="CH19" t="n">
-        <v>1675.79</v>
+        <v>1690.36</v>
       </c>
       <c r="CI19" t="n">
-        <v>5.93</v>
+        <v>6.85</v>
       </c>
       <c r="CJ19" t="n">
-        <v>5.2</v>
+        <v>8.699999999999999</v>
       </c>
       <c r="CK19" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-21</t>
         </is>
       </c>
     </row>
@@ -6939,13 +6939,13 @@
         </is>
       </c>
       <c r="CD20" t="n">
-        <v>16434.67</v>
+        <v>16434.07</v>
       </c>
       <c r="CE20" t="n">
         <v>6.17</v>
       </c>
       <c r="CF20" t="n">
-        <v>4.52</v>
+        <v>4.51</v>
       </c>
       <c r="CG20" t="inlineStr">
         <is>
@@ -6953,17 +6953,17 @@
         </is>
       </c>
       <c r="CH20" t="n">
-        <v>16485.81</v>
+        <v>16434.89</v>
       </c>
       <c r="CI20" t="n">
-        <v>5.76</v>
+        <v>5.43</v>
       </c>
       <c r="CJ20" t="n">
-        <v>1.25</v>
+        <v>0.02</v>
       </c>
       <c r="CK20" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-21</t>
         </is>
       </c>
     </row>
@@ -7260,7 +7260,7 @@
         </is>
       </c>
       <c r="CD21" t="n">
-        <v>7954.16</v>
+        <v>7954.17</v>
       </c>
       <c r="CE21" t="n">
         <v>7.78</v>
@@ -7274,17 +7274,17 @@
         </is>
       </c>
       <c r="CH21" t="n">
-        <v>7999.72</v>
+        <v>8005.01</v>
       </c>
       <c r="CI21" t="n">
-        <v>6.71</v>
+        <v>6.78</v>
       </c>
       <c r="CJ21" t="n">
-        <v>2.31</v>
+        <v>2.58</v>
       </c>
       <c r="CK21" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-21</t>
         </is>
       </c>
     </row>
@@ -7595,17 +7595,17 @@
         </is>
       </c>
       <c r="CH22" t="n">
-        <v>1614.97</v>
+        <v>1615.3</v>
       </c>
       <c r="CI22" t="n">
-        <v>10.95</v>
+        <v>10.98</v>
       </c>
       <c r="CJ22" t="n">
-        <v>4.58</v>
+        <v>4.66</v>
       </c>
       <c r="CK22" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-21</t>
         </is>
       </c>
     </row>
@@ -7916,17 +7916,17 @@
         </is>
       </c>
       <c r="CH23" t="n">
-        <v>918.39</v>
+        <v>911.52</v>
       </c>
       <c r="CI23" t="n">
-        <v>3</v>
+        <v>2.23</v>
       </c>
       <c r="CJ23" t="n">
-        <v>2.6</v>
+        <v>-0.43</v>
       </c>
       <c r="CK23" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-21</t>
         </is>
       </c>
     </row>
@@ -8237,17 +8237,17 @@
         </is>
       </c>
       <c r="CH24" t="n">
-        <v>125.46</v>
+        <v>126.16</v>
       </c>
       <c r="CI24" t="n">
-        <v>-1.79</v>
+        <v>-1.25</v>
       </c>
       <c r="CJ24" t="n">
-        <v>1.38</v>
+        <v>3.65</v>
       </c>
       <c r="CK24" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-21</t>
         </is>
       </c>
     </row>
@@ -8558,17 +8558,17 @@
         </is>
       </c>
       <c r="CH25" t="n">
-        <v>6.24</v>
+        <v>6.25</v>
       </c>
       <c r="CI25" t="n">
-        <v>-2.97</v>
+        <v>-2.78</v>
       </c>
       <c r="CJ25" t="n">
-        <v>-7.97</v>
+        <v>-7.25</v>
       </c>
       <c r="CK25" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-21</t>
         </is>
       </c>
     </row>
@@ -8879,17 +8879,17 @@
         </is>
       </c>
       <c r="CH26" t="n">
-        <v>254.71</v>
+        <v>252.49</v>
       </c>
       <c r="CI26" t="n">
-        <v>5.23</v>
+        <v>4.32</v>
       </c>
       <c r="CJ26" t="n">
-        <v>2.52</v>
+        <v>-1.01</v>
       </c>
       <c r="CK26" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-21</t>
         </is>
       </c>
     </row>
@@ -9200,17 +9200,17 @@
         </is>
       </c>
       <c r="CH27" t="n">
-        <v>531.97</v>
+        <v>526.61</v>
       </c>
       <c r="CI27" t="n">
-        <v>3.22</v>
+        <v>2.18</v>
       </c>
       <c r="CJ27" t="n">
-        <v>3.06</v>
+        <v>-1.03</v>
       </c>
       <c r="CK27" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-21</t>
         </is>
       </c>
     </row>
@@ -9521,17 +9521,17 @@
         </is>
       </c>
       <c r="CH28" t="n">
-        <v>1657.24</v>
+        <v>1665.83</v>
       </c>
       <c r="CI28" t="n">
-        <v>-0.07000000000000001</v>
+        <v>0.45</v>
       </c>
       <c r="CJ28" t="n">
-        <v>-0.57</v>
+        <v>1.51</v>
       </c>
       <c r="CK28" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-21</t>
         </is>
       </c>
     </row>
@@ -9842,17 +9842,17 @@
         </is>
       </c>
       <c r="CH29" t="n">
-        <v>1495.64</v>
+        <v>1504.09</v>
       </c>
       <c r="CI29" t="n">
-        <v>-0.33</v>
+        <v>0.24</v>
       </c>
       <c r="CJ29" t="n">
-        <v>-0.71</v>
+        <v>1.56</v>
       </c>
       <c r="CK29" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-21</t>
         </is>
       </c>
     </row>
@@ -10163,17 +10163,17 @@
         </is>
       </c>
       <c r="CH30" t="n">
-        <v>161.6</v>
+        <v>161.73</v>
       </c>
       <c r="CI30" t="n">
-        <v>2.35</v>
+        <v>2.44</v>
       </c>
       <c r="CJ30" t="n">
-        <v>0.72</v>
+        <v>1.05</v>
       </c>
       <c r="CK30" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-21</t>
         </is>
       </c>
     </row>
@@ -10484,17 +10484,17 @@
         </is>
       </c>
       <c r="CH31" t="n">
-        <v>1584.56</v>
+        <v>1584.91</v>
       </c>
       <c r="CI31" t="n">
-        <v>2.96</v>
+        <v>2.98</v>
       </c>
       <c r="CJ31" t="n">
-        <v>-0.42</v>
+        <v>-0.33</v>
       </c>
       <c r="CK31" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-21</t>
         </is>
       </c>
     </row>
@@ -10805,17 +10805,17 @@
         </is>
       </c>
       <c r="CH32" t="n">
-        <v>1002.07</v>
+        <v>1003.46</v>
       </c>
       <c r="CI32" t="n">
-        <v>3.79</v>
+        <v>3.93</v>
       </c>
       <c r="CJ32" t="n">
-        <v>-0.22</v>
+        <v>0.34</v>
       </c>
       <c r="CK32" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-21</t>
         </is>
       </c>
     </row>
@@ -11126,17 +11126,17 @@
         </is>
       </c>
       <c r="CH33" t="n">
-        <v>582.49</v>
+        <v>581.45</v>
       </c>
       <c r="CI33" t="n">
-        <v>1.56</v>
+        <v>1.38</v>
       </c>
       <c r="CJ33" t="n">
-        <v>-0.76</v>
+        <v>-1.47</v>
       </c>
       <c r="CK33" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-21</t>
         </is>
       </c>
     </row>
@@ -11447,17 +11447,17 @@
         </is>
       </c>
       <c r="CH34" t="n">
-        <v>436.15</v>
+        <v>436.03</v>
       </c>
       <c r="CI34" t="n">
-        <v>1.96</v>
+        <v>1.93</v>
       </c>
       <c r="CJ34" t="n">
-        <v>-0.6899999999999999</v>
+        <v>-0.8</v>
       </c>
       <c r="CK34" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-21</t>
         </is>
       </c>
     </row>
@@ -11754,13 +11754,13 @@
         </is>
       </c>
       <c r="CD35" t="n">
-        <v>2198.83</v>
+        <v>2198.84</v>
       </c>
       <c r="CE35" t="n">
         <v>17.89</v>
       </c>
       <c r="CF35" t="n">
-        <v>18.37</v>
+        <v>18.38</v>
       </c>
       <c r="CG35" t="inlineStr">
         <is>
@@ -11768,17 +11768,17 @@
         </is>
       </c>
       <c r="CH35" t="n">
-        <v>2224.56</v>
+        <v>2227.46</v>
       </c>
       <c r="CI35" t="n">
-        <v>13.96</v>
+        <v>14.11</v>
       </c>
       <c r="CJ35" t="n">
-        <v>4.76</v>
+        <v>5.31</v>
       </c>
       <c r="CK35" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-21</t>
         </is>
       </c>
     </row>
@@ -12089,17 +12089,17 @@
         </is>
       </c>
       <c r="CH36" t="n">
-        <v>1363.98</v>
+        <v>1378</v>
       </c>
       <c r="CI36" t="n">
-        <v>15.44</v>
+        <v>16.62</v>
       </c>
       <c r="CJ36" t="n">
-        <v>5.88</v>
+        <v>10.3</v>
       </c>
       <c r="CK36" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-21</t>
         </is>
       </c>
     </row>
@@ -12410,17 +12410,17 @@
         </is>
       </c>
       <c r="CH37" t="n">
-        <v>12466.24</v>
+        <v>12438.83</v>
       </c>
       <c r="CI37" t="n">
-        <v>6.79</v>
+        <v>6.55</v>
       </c>
       <c r="CJ37" t="n">
-        <v>1.67</v>
+        <v>0.78</v>
       </c>
       <c r="CK37" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-21</t>
         </is>
       </c>
     </row>
@@ -12717,13 +12717,13 @@
         </is>
       </c>
       <c r="CD38" t="n">
-        <v>918.71</v>
+        <v>919.28</v>
       </c>
       <c r="CE38" t="n">
-        <v>13.55</v>
+        <v>13.62</v>
       </c>
       <c r="CF38" t="n">
-        <v>17.95</v>
+        <v>18.24</v>
       </c>
       <c r="CG38" t="inlineStr">
         <is>
@@ -12731,17 +12731,17 @@
         </is>
       </c>
       <c r="CH38" t="n">
-        <v>931.27</v>
+        <v>946.9400000000001</v>
       </c>
       <c r="CI38" t="n">
-        <v>11.29</v>
+        <v>13.16</v>
       </c>
       <c r="CJ38" t="n">
-        <v>5.58</v>
+        <v>12.59</v>
       </c>
       <c r="CK38" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-21</t>
         </is>
       </c>
     </row>
@@ -13038,13 +13038,13 @@
         </is>
       </c>
       <c r="CD39" t="n">
-        <v>11496.03</v>
+        <v>11495.47</v>
       </c>
       <c r="CE39" t="n">
-        <v>6.73</v>
+        <v>6.72</v>
       </c>
       <c r="CF39" t="n">
-        <v>5.39</v>
+        <v>5.37</v>
       </c>
       <c r="CG39" t="inlineStr">
         <is>
@@ -13052,17 +13052,17 @@
         </is>
       </c>
       <c r="CH39" t="n">
-        <v>11534.97</v>
+        <v>11491.89</v>
       </c>
       <c r="CI39" t="n">
-        <v>6.44</v>
+        <v>6.04</v>
       </c>
       <c r="CJ39" t="n">
-        <v>1.36</v>
+        <v>-0.12</v>
       </c>
       <c r="CK39" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-21</t>
         </is>
       </c>
     </row>
@@ -13359,13 +13359,13 @@
         </is>
       </c>
       <c r="CD40" t="n">
-        <v>4754.84</v>
+        <v>4755.86</v>
       </c>
       <c r="CE40" t="n">
-        <v>5.56</v>
+        <v>5.58</v>
       </c>
       <c r="CF40" t="n">
-        <v>5.57</v>
+        <v>5.66</v>
       </c>
       <c r="CG40" t="inlineStr">
         <is>
@@ -13373,17 +13373,17 @@
         </is>
       </c>
       <c r="CH40" t="n">
-        <v>4772.62</v>
+        <v>4764.35</v>
       </c>
       <c r="CI40" t="n">
-        <v>4.59</v>
+        <v>4.41</v>
       </c>
       <c r="CJ40" t="n">
-        <v>1.5</v>
+        <v>0.72</v>
       </c>
       <c r="CK40" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-21</t>
         </is>
       </c>
     </row>
@@ -13694,17 +13694,17 @@
         </is>
       </c>
       <c r="CH41" t="n">
-        <v>742.04</v>
+        <v>741.61</v>
       </c>
       <c r="CI41" t="n">
-        <v>5.78</v>
+        <v>5.72</v>
       </c>
       <c r="CJ41" t="n">
-        <v>1.16</v>
+        <v>0.93</v>
       </c>
       <c r="CK41" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-21</t>
         </is>
       </c>
     </row>
@@ -14001,13 +14001,13 @@
         </is>
       </c>
       <c r="CD42" t="n">
-        <v>2112.15</v>
+        <v>2112.55</v>
       </c>
       <c r="CE42" t="n">
-        <v>3.89</v>
+        <v>3.91</v>
       </c>
       <c r="CF42" t="n">
-        <v>4.39</v>
+        <v>4.47</v>
       </c>
       <c r="CG42" t="inlineStr">
         <is>
@@ -14015,17 +14015,17 @@
         </is>
       </c>
       <c r="CH42" t="n">
-        <v>2115.67</v>
+        <v>2114.32</v>
       </c>
       <c r="CI42" t="n">
-        <v>3.11</v>
+        <v>3.04</v>
       </c>
       <c r="CJ42" t="n">
-        <v>0.67</v>
+        <v>0.33</v>
       </c>
       <c r="CK42" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-21</t>
         </is>
       </c>
     </row>
@@ -14322,13 +14322,13 @@
         </is>
       </c>
       <c r="CD43" t="n">
-        <v>309.1</v>
+        <v>308.96</v>
       </c>
       <c r="CE43" t="n">
-        <v>-0.24</v>
+        <v>-0.29</v>
       </c>
       <c r="CF43" t="n">
-        <v>7.42</v>
+        <v>7.22</v>
       </c>
       <c r="CG43" t="inlineStr">
         <is>
@@ -14336,17 +14336,17 @@
         </is>
       </c>
       <c r="CH43" t="n">
-        <v>309.85</v>
+        <v>309.9</v>
       </c>
       <c r="CI43" t="n">
-        <v>1.33</v>
+        <v>1.35</v>
       </c>
       <c r="CJ43" t="n">
-        <v>0.97</v>
+        <v>1.22</v>
       </c>
       <c r="CK43" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-21</t>
         </is>
       </c>
     </row>
@@ -14643,13 +14643,13 @@
         </is>
       </c>
       <c r="CD44" t="n">
-        <v>116.95</v>
+        <v>117.02</v>
       </c>
       <c r="CE44" t="n">
-        <v>5.23</v>
+        <v>5.29</v>
       </c>
       <c r="CF44" t="n">
-        <v>4.97</v>
+        <v>5.2</v>
       </c>
       <c r="CG44" t="inlineStr">
         <is>
@@ -14657,17 +14657,17 @@
         </is>
       </c>
       <c r="CH44" t="n">
-        <v>117.22</v>
+        <v>117.23</v>
       </c>
       <c r="CI44" t="n">
-        <v>4.17</v>
+        <v>4.18</v>
       </c>
       <c r="CJ44" t="n">
-        <v>0.93</v>
+        <v>0.73</v>
       </c>
       <c r="CK44" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-21</t>
         </is>
       </c>
     </row>
@@ -14964,13 +14964,13 @@
         </is>
       </c>
       <c r="CD45" t="n">
-        <v>368.25</v>
+        <v>368.78</v>
       </c>
       <c r="CE45" t="n">
-        <v>2.41</v>
+        <v>2.56</v>
       </c>
       <c r="CF45" t="n">
-        <v>2.11</v>
+        <v>2.7</v>
       </c>
       <c r="CG45" t="inlineStr">
         <is>
@@ -14978,17 +14978,17 @@
         </is>
       </c>
       <c r="CH45" t="n">
-        <v>368.57</v>
+        <v>368.85</v>
       </c>
       <c r="CI45" t="n">
-        <v>1.43</v>
+        <v>1.51</v>
       </c>
       <c r="CJ45" t="n">
-        <v>0.35</v>
+        <v>0.08</v>
       </c>
       <c r="CK45" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-21</t>
         </is>
       </c>
     </row>
@@ -15285,13 +15285,13 @@
         </is>
       </c>
       <c r="CD46" t="n">
-        <v>1317.85</v>
+        <v>1317.8</v>
       </c>
       <c r="CE46" t="n">
-        <v>5.22</v>
+        <v>5.21</v>
       </c>
       <c r="CF46" t="n">
-        <v>4.28</v>
+        <v>4.27</v>
       </c>
       <c r="CG46" t="inlineStr">
         <is>
@@ -15299,17 +15299,17 @@
         </is>
       </c>
       <c r="CH46" t="n">
-        <v>1320.02</v>
+        <v>1318.34</v>
       </c>
       <c r="CI46" t="n">
-        <v>3.92</v>
+        <v>3.79</v>
       </c>
       <c r="CJ46" t="n">
-        <v>0.66</v>
+        <v>0.16</v>
       </c>
       <c r="CK46" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-21</t>
         </is>
       </c>
     </row>
@@ -15606,13 +15606,13 @@
         </is>
       </c>
       <c r="CD47" t="n">
-        <v>1037.87</v>
+        <v>1037.95</v>
       </c>
       <c r="CE47" t="n">
         <v>3.42</v>
       </c>
       <c r="CF47" t="n">
-        <v>2.37</v>
+        <v>2.4</v>
       </c>
       <c r="CG47" t="inlineStr">
         <is>
@@ -15620,17 +15620,17 @@
         </is>
       </c>
       <c r="CH47" t="n">
-        <v>1038.25</v>
+        <v>1038.71</v>
       </c>
       <c r="CI47" t="n">
-        <v>2.44</v>
+        <v>2.48</v>
       </c>
       <c r="CJ47" t="n">
-        <v>0.15</v>
+        <v>0.29</v>
       </c>
       <c r="CK47" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-21</t>
         </is>
       </c>
     </row>
@@ -15927,13 +15927,13 @@
         </is>
       </c>
       <c r="CD48" t="n">
-        <v>908.1</v>
+        <v>908.1799999999999</v>
       </c>
       <c r="CE48" t="n">
-        <v>2.36</v>
+        <v>2.37</v>
       </c>
       <c r="CF48" t="n">
-        <v>0.91</v>
+        <v>0.9399999999999999</v>
       </c>
       <c r="CG48" t="inlineStr">
         <is>
@@ -15941,17 +15941,17 @@
         </is>
       </c>
       <c r="CH48" t="n">
-        <v>908.37</v>
+        <v>908.92</v>
       </c>
       <c r="CI48" t="n">
-        <v>1.62</v>
+        <v>1.68</v>
       </c>
       <c r="CJ48" t="n">
-        <v>0.12</v>
+        <v>0.33</v>
       </c>
       <c r="CK48" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-21</t>
         </is>
       </c>
     </row>
@@ -16254,7 +16254,7 @@
         <v>11.46</v>
       </c>
       <c r="CF49" t="n">
-        <v>13.38</v>
+        <v>13.39</v>
       </c>
       <c r="CG49" t="inlineStr">
         <is>
@@ -16262,17 +16262,17 @@
         </is>
       </c>
       <c r="CH49" t="n">
-        <v>129.88</v>
+        <v>129.79</v>
       </c>
       <c r="CI49" t="n">
-        <v>8.52</v>
+        <v>8.449999999999999</v>
       </c>
       <c r="CJ49" t="n">
-        <v>0.33</v>
+        <v>0.07000000000000001</v>
       </c>
       <c r="CK49" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-21</t>
         </is>
       </c>
     </row>
@@ -16569,13 +16569,13 @@
         </is>
       </c>
       <c r="CD50" t="n">
-        <v>341.62</v>
+        <v>342.17</v>
       </c>
       <c r="CE50" t="n">
-        <v>9.039999999999999</v>
+        <v>9.210000000000001</v>
       </c>
       <c r="CF50" t="n">
-        <v>15.22</v>
+        <v>15.97</v>
       </c>
       <c r="CG50" t="inlineStr">
         <is>
@@ -16583,17 +16583,17 @@
         </is>
       </c>
       <c r="CH50" t="n">
-        <v>353.61</v>
+        <v>347.15</v>
       </c>
       <c r="CI50" t="n">
-        <v>10.72</v>
+        <v>8.699999999999999</v>
       </c>
       <c r="CJ50" t="n">
-        <v>14.8</v>
+        <v>5.95</v>
       </c>
       <c r="CK50" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-21</t>
         </is>
       </c>
     </row>
@@ -16890,13 +16890,13 @@
         </is>
       </c>
       <c r="CD51" t="n">
-        <v>93.8</v>
+        <v>94.40000000000001</v>
       </c>
       <c r="CE51" t="n">
-        <v>-2.36</v>
+        <v>-1.73</v>
       </c>
       <c r="CF51" t="n">
-        <v>-5</v>
+        <v>-2.56</v>
       </c>
       <c r="CG51" t="inlineStr">
         <is>
@@ -16904,17 +16904,17 @@
         </is>
       </c>
       <c r="CH51" t="n">
-        <v>103.78</v>
+        <v>96.41</v>
       </c>
       <c r="CI51" t="n">
-        <v>5.96</v>
+        <v>-1.56</v>
       </c>
       <c r="CJ51" t="n">
-        <v>49.86</v>
+        <v>8.82</v>
       </c>
       <c r="CK51" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-21</t>
         </is>
       </c>
     </row>
@@ -17211,13 +17211,13 @@
         </is>
       </c>
       <c r="CD52" t="n">
-        <v>247.82</v>
+        <v>247.77</v>
       </c>
       <c r="CE52" t="n">
-        <v>14.07</v>
+        <v>14.05</v>
       </c>
       <c r="CF52" t="n">
-        <v>24.27</v>
+        <v>24.18</v>
       </c>
       <c r="CG52" t="inlineStr">
         <is>
@@ -17225,17 +17225,17 @@
         </is>
       </c>
       <c r="CH52" t="n">
-        <v>249.83</v>
+        <v>250.74</v>
       </c>
       <c r="CI52" t="n">
-        <v>12.82</v>
+        <v>13.23</v>
       </c>
       <c r="CJ52" t="n">
-        <v>3.28</v>
+        <v>4.87</v>
       </c>
       <c r="CK52" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-21</t>
         </is>
       </c>
     </row>
@@ -17546,17 +17546,17 @@
         </is>
       </c>
       <c r="CH53" t="n">
-        <v>88.34</v>
+        <v>88.61</v>
       </c>
       <c r="CI53" t="n">
-        <v>14.19</v>
+        <v>14.53</v>
       </c>
       <c r="CJ53" t="n">
-        <v>3.7</v>
+        <v>4.96</v>
       </c>
       <c r="CK53" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-21</t>
         </is>
       </c>
     </row>
@@ -17853,13 +17853,13 @@
         </is>
       </c>
       <c r="CD54" t="n">
-        <v>523.3</v>
+        <v>523.29</v>
       </c>
       <c r="CE54" t="n">
-        <v>16.06</v>
+        <v>16.05</v>
       </c>
       <c r="CF54" t="n">
-        <v>10.81</v>
+        <v>10.79</v>
       </c>
       <c r="CG54" t="inlineStr">
         <is>
@@ -17867,17 +17867,17 @@
         </is>
       </c>
       <c r="CH54" t="n">
-        <v>523.05</v>
+        <v>522.5599999999999</v>
       </c>
       <c r="CI54" t="n">
-        <v>9.67</v>
+        <v>9.56</v>
       </c>
       <c r="CJ54" t="n">
-        <v>-0.19</v>
+        <v>-0.5600000000000001</v>
       </c>
       <c r="CK54" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-21</t>
         </is>
       </c>
     </row>
@@ -18188,17 +18188,17 @@
         </is>
       </c>
       <c r="CH55" t="n">
-        <v>202.29</v>
+        <v>200.51</v>
       </c>
       <c r="CI55" t="n">
-        <v>11.74</v>
+        <v>10.76</v>
       </c>
       <c r="CJ55" t="n">
-        <v>-1.24</v>
+        <v>-4.68</v>
       </c>
       <c r="CK55" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-21</t>
         </is>
       </c>
     </row>
@@ -18495,13 +18495,13 @@
         </is>
       </c>
       <c r="CD56" t="n">
-        <v>5674.6</v>
+        <v>5674.79</v>
       </c>
       <c r="CE56" t="n">
         <v>4.3</v>
       </c>
       <c r="CF56" t="n">
-        <v>2.14</v>
+        <v>2.15</v>
       </c>
       <c r="CG56" t="inlineStr">
         <is>
@@ -18509,17 +18509,17 @@
         </is>
       </c>
       <c r="CH56" t="n">
-        <v>5695.36</v>
+        <v>5686.41</v>
       </c>
       <c r="CI56" t="n">
-        <v>3.63</v>
+        <v>3.47</v>
       </c>
       <c r="CJ56" t="n">
-        <v>1.47</v>
+        <v>0.82</v>
       </c>
       <c r="CK56" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-21</t>
         </is>
       </c>
     </row>
@@ -18816,13 +18816,13 @@
         </is>
       </c>
       <c r="CD57" t="n">
-        <v>735.96</v>
+        <v>736.1799999999999</v>
       </c>
       <c r="CE57" t="n">
-        <v>0.5</v>
+        <v>0.53</v>
       </c>
       <c r="CF57" t="n">
-        <v>-0.42</v>
+        <v>-0.3</v>
       </c>
       <c r="CG57" t="inlineStr">
         <is>
@@ -18830,17 +18830,17 @@
         </is>
       </c>
       <c r="CH57" t="n">
-        <v>744.52</v>
+        <v>743.42</v>
       </c>
       <c r="CI57" t="n">
-        <v>-0.09</v>
+        <v>-0.24</v>
       </c>
       <c r="CJ57" t="n">
-        <v>4.73</v>
+        <v>3.99</v>
       </c>
       <c r="CK57" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-21</t>
         </is>
       </c>
     </row>
@@ -19137,7 +19137,7 @@
         </is>
       </c>
       <c r="CD58" t="n">
-        <v>4938.65</v>
+        <v>4938.6</v>
       </c>
       <c r="CE58" t="n">
         <v>4.89</v>
@@ -19151,17 +19151,17 @@
         </is>
       </c>
       <c r="CH58" t="n">
-        <v>4950.84</v>
+        <v>4943</v>
       </c>
       <c r="CI58" t="n">
-        <v>4.21</v>
+        <v>4.05</v>
       </c>
       <c r="CJ58" t="n">
-        <v>0.99</v>
+        <v>0.36</v>
       </c>
       <c r="CK58" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-21</t>
         </is>
       </c>
     </row>
@@ -19888,28 +19888,28 @@
         <v>13</v>
       </c>
       <c r="CD2" t="n">
-        <v>12594.54</v>
+        <v>12594.75</v>
       </c>
       <c r="CE2" t="n">
         <v>6.67</v>
       </c>
       <c r="CF2" t="n">
-        <v>5.71</v>
+        <v>5.72</v>
       </c>
       <c r="CG2" t="n">
         <v>14</v>
       </c>
       <c r="CH2" t="n">
-        <v>12763.08</v>
+        <v>12759</v>
       </c>
       <c r="CI2" t="n">
-        <v>6.52</v>
+        <v>6.49</v>
       </c>
       <c r="CJ2" t="n">
-        <v>5.46</v>
+        <v>5.32</v>
       </c>
       <c r="CK2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="3">
@@ -20167,7 +20167,7 @@
         <v>13</v>
       </c>
       <c r="CD3" t="n">
-        <v>2307.32</v>
+        <v>2307.33</v>
       </c>
       <c r="CE3" t="n">
         <v>7.58</v>
@@ -20179,16 +20179,16 @@
         <v>14</v>
       </c>
       <c r="CH3" t="n">
-        <v>2358.01</v>
+        <v>2357.39</v>
       </c>
       <c r="CI3" t="n">
-        <v>9.4</v>
+        <v>9.369999999999999</v>
       </c>
       <c r="CJ3" t="n">
-        <v>9.08</v>
+        <v>8.960000000000001</v>
       </c>
       <c r="CK3" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="4">
@@ -20446,28 +20446,28 @@
         <v>13</v>
       </c>
       <c r="CD4" t="n">
-        <v>3004.46</v>
+        <v>3004.52</v>
       </c>
       <c r="CE4" t="n">
         <v>3.32</v>
       </c>
       <c r="CF4" t="n">
-        <v>3.63</v>
+        <v>3.64</v>
       </c>
       <c r="CG4" t="n">
         <v>14</v>
       </c>
       <c r="CH4" t="n">
-        <v>3032.63</v>
+        <v>3029.91</v>
       </c>
       <c r="CI4" t="n">
+        <v>3.32</v>
+      </c>
+      <c r="CJ4" t="n">
         <v>3.42</v>
       </c>
-      <c r="CJ4" t="n">
-        <v>3.8</v>
-      </c>
       <c r="CK4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="5">
@@ -20725,28 +20725,28 @@
         <v>13</v>
       </c>
       <c r="CD5" t="n">
-        <v>431.7</v>
+        <v>431.67</v>
       </c>
       <c r="CE5" t="n">
-        <v>-2.06</v>
+        <v>-2.07</v>
       </c>
       <c r="CF5" t="n">
-        <v>3.4</v>
+        <v>3.38</v>
       </c>
       <c r="CG5" t="n">
         <v>14</v>
       </c>
       <c r="CH5" t="n">
-        <v>435.78</v>
+        <v>435.66</v>
       </c>
       <c r="CI5" t="n">
-        <v>0.15</v>
+        <v>0.12</v>
       </c>
       <c r="CJ5" t="n">
-        <v>3.83</v>
+        <v>3.75</v>
       </c>
       <c r="CK5" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="6">
@@ -21004,13 +21004,13 @@
         <v>13</v>
       </c>
       <c r="CD6" t="n">
-        <v>122.54</v>
+        <v>122.59</v>
       </c>
       <c r="CE6" t="n">
-        <v>4.38</v>
+        <v>4.42</v>
       </c>
       <c r="CF6" t="n">
-        <v>4.59</v>
+        <v>4.74</v>
       </c>
       <c r="CG6" t="n">
         <v>14</v>
@@ -21022,10 +21022,10 @@
         <v>4.31</v>
       </c>
       <c r="CJ6" t="n">
-        <v>2.97</v>
+        <v>2.83</v>
       </c>
       <c r="CK6" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="7">
@@ -21283,28 +21283,28 @@
         <v>13</v>
       </c>
       <c r="CD7" t="n">
-        <v>617.0599999999999</v>
+        <v>617.11</v>
       </c>
       <c r="CE7" t="n">
-        <v>3.9</v>
+        <v>3.91</v>
       </c>
       <c r="CF7" t="n">
-        <v>1.36</v>
+        <v>1.39</v>
       </c>
       <c r="CG7" t="n">
         <v>14</v>
       </c>
       <c r="CH7" t="n">
-        <v>623.5</v>
+        <v>622.9400000000001</v>
       </c>
       <c r="CI7" t="n">
-        <v>3.47</v>
+        <v>3.37</v>
       </c>
       <c r="CJ7" t="n">
-        <v>4.24</v>
+        <v>3.83</v>
       </c>
       <c r="CK7" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="8">
@@ -21562,7 +21562,7 @@
         <v>13</v>
       </c>
       <c r="CD8" t="n">
-        <v>1833.16</v>
+        <v>1833.15</v>
       </c>
       <c r="CE8" t="n">
         <v>4.4</v>
@@ -21574,16 +21574,16 @@
         <v>14</v>
       </c>
       <c r="CH8" t="n">
-        <v>1849.92</v>
+        <v>1847.87</v>
       </c>
       <c r="CI8" t="n">
-        <v>4.14</v>
+        <v>4.02</v>
       </c>
       <c r="CJ8" t="n">
-        <v>3.71</v>
+        <v>3.25</v>
       </c>
       <c r="CK8" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="9">
@@ -21841,28 +21841,28 @@
         <v>13</v>
       </c>
       <c r="CD9" t="n">
-        <v>2696.68</v>
+        <v>2696.72</v>
       </c>
       <c r="CE9" t="n">
         <v>1.64</v>
       </c>
       <c r="CF9" t="n">
-        <v>1.41</v>
+        <v>1.42</v>
       </c>
       <c r="CG9" t="n">
         <v>14</v>
       </c>
       <c r="CH9" t="n">
-        <v>2695.73</v>
+        <v>2698.6</v>
       </c>
       <c r="CI9" t="n">
-        <v>1.08</v>
+        <v>1.19</v>
       </c>
       <c r="CJ9" t="n">
-        <v>-0.14</v>
+        <v>0.28</v>
       </c>
       <c r="CK9" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="10">
@@ -22120,7 +22120,7 @@
         <v>13</v>
       </c>
       <c r="CD10" t="n">
-        <v>2408.06</v>
+        <v>2408.09</v>
       </c>
       <c r="CE10" t="n">
         <v>1.13</v>
@@ -22132,16 +22132,16 @@
         <v>14</v>
       </c>
       <c r="CH10" t="n">
-        <v>2404.28</v>
+        <v>2407.16</v>
       </c>
       <c r="CI10" t="n">
-        <v>0.5600000000000001</v>
+        <v>0.68</v>
       </c>
       <c r="CJ10" t="n">
-        <v>-0.63</v>
+        <v>-0.15</v>
       </c>
       <c r="CK10" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="11">
@@ -22411,16 +22411,16 @@
         <v>14</v>
       </c>
       <c r="CH11" t="n">
-        <v>291.44</v>
+        <v>291.43</v>
       </c>
       <c r="CI11" t="n">
         <v>5.6</v>
       </c>
       <c r="CJ11" t="n">
-        <v>3.97</v>
+        <v>3.95</v>
       </c>
       <c r="CK11" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="12">
@@ -22678,28 +22678,28 @@
         <v>13</v>
       </c>
       <c r="CD12" t="n">
-        <v>1919.39</v>
+        <v>1919.49</v>
       </c>
       <c r="CE12" t="n">
         <v>5.09</v>
       </c>
       <c r="CF12" t="n">
-        <v>5.51</v>
+        <v>5.53</v>
       </c>
       <c r="CG12" t="n">
         <v>14</v>
       </c>
       <c r="CH12" t="n">
-        <v>1937.05</v>
+        <v>1930.03</v>
       </c>
       <c r="CI12" t="n">
-        <v>4.71</v>
+        <v>4.34</v>
       </c>
       <c r="CJ12" t="n">
-        <v>3.73</v>
+        <v>2.21</v>
       </c>
       <c r="CK12" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="13">
@@ -22957,28 +22957,28 @@
         <v>13</v>
       </c>
       <c r="CD13" t="n">
-        <v>1090.16</v>
+        <v>1090.26</v>
       </c>
       <c r="CE13" t="n">
-        <v>4.08</v>
+        <v>4.09</v>
       </c>
       <c r="CF13" t="n">
-        <v>2.71</v>
+        <v>2.75</v>
       </c>
       <c r="CG13" t="n">
         <v>14</v>
       </c>
       <c r="CH13" t="n">
-        <v>1105.01</v>
+        <v>1098.07</v>
       </c>
       <c r="CI13" t="n">
-        <v>4.36</v>
+        <v>3.71</v>
       </c>
       <c r="CJ13" t="n">
-        <v>5.56</v>
+        <v>2.9</v>
       </c>
       <c r="CK13" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="14">
@@ -23236,7 +23236,7 @@
         <v>13</v>
       </c>
       <c r="CD14" t="n">
-        <v>829.24</v>
+        <v>829.23</v>
       </c>
       <c r="CE14" t="n">
         <v>6.43</v>
@@ -23248,16 +23248,16 @@
         <v>14</v>
       </c>
       <c r="CH14" t="n">
-        <v>832.04</v>
+        <v>831.96</v>
       </c>
       <c r="CI14" t="n">
-        <v>5.19</v>
+        <v>5.18</v>
       </c>
       <c r="CJ14" t="n">
-        <v>1.36</v>
+        <v>1.32</v>
       </c>
       <c r="CK14" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="15">
@@ -23527,16 +23527,16 @@
         <v>14</v>
       </c>
       <c r="CH15" t="n">
-        <v>524.46</v>
+        <v>524.4299999999999</v>
       </c>
       <c r="CI15" t="n">
-        <v>4.79</v>
+        <v>4.78</v>
       </c>
       <c r="CJ15" t="n">
-        <v>0.27</v>
+        <v>0.25</v>
       </c>
       <c r="CK15" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="16">
@@ -23794,28 +23794,28 @@
         <v>13</v>
       </c>
       <c r="CD16" t="n">
-        <v>2666.68</v>
+        <v>2666.69</v>
       </c>
       <c r="CE16" t="n">
         <v>17.25</v>
       </c>
       <c r="CF16" t="n">
-        <v>11.43</v>
+        <v>11.44</v>
       </c>
       <c r="CG16" t="n">
         <v>14</v>
       </c>
       <c r="CH16" t="n">
-        <v>2739.66</v>
+        <v>2743.07</v>
       </c>
       <c r="CI16" t="n">
-        <v>15.24</v>
+        <v>15.39</v>
       </c>
       <c r="CJ16" t="n">
-        <v>11.4</v>
+        <v>11.96</v>
       </c>
       <c r="CK16" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="17">
@@ -24085,16 +24085,16 @@
         <v>14</v>
       </c>
       <c r="CH17" t="n">
-        <v>1562.81</v>
+        <v>1567.96</v>
       </c>
       <c r="CI17" t="n">
-        <v>18.97</v>
+        <v>19.36</v>
       </c>
       <c r="CJ17" t="n">
-        <v>14.84</v>
+        <v>16.36</v>
       </c>
       <c r="CK17" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="18">
@@ -24352,7 +24352,7 @@
         <v>13</v>
       </c>
       <c r="CD18" t="n">
-        <v>17938.38</v>
+        <v>17938.39</v>
       </c>
       <c r="CE18" t="n">
         <v>5.98</v>
@@ -24364,16 +24364,16 @@
         <v>14</v>
       </c>
       <c r="CH18" t="n">
-        <v>18145.52</v>
+        <v>18134.15</v>
       </c>
       <c r="CI18" t="n">
-        <v>5.94</v>
+        <v>5.88</v>
       </c>
       <c r="CJ18" t="n">
-        <v>4.7</v>
+        <v>4.44</v>
       </c>
       <c r="CK18" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="19">
@@ -24631,28 +24631,28 @@
         <v>13</v>
       </c>
       <c r="CD19" t="n">
-        <v>1633.32</v>
+        <v>1633.38</v>
       </c>
       <c r="CE19" t="n">
-        <v>5.98</v>
+        <v>5.99</v>
       </c>
       <c r="CF19" t="n">
-        <v>-0.6899999999999999</v>
+        <v>-0.68</v>
       </c>
       <c r="CG19" t="n">
         <v>14</v>
       </c>
       <c r="CH19" t="n">
-        <v>1669.25</v>
+        <v>1674.79</v>
       </c>
       <c r="CI19" t="n">
-        <v>6.2</v>
+        <v>6.56</v>
       </c>
       <c r="CJ19" t="n">
-        <v>9.09</v>
+        <v>10.53</v>
       </c>
       <c r="CK19" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="20">
@@ -24910,7 +24910,7 @@
         <v>13</v>
       </c>
       <c r="CD20" t="n">
-        <v>16305.07</v>
+        <v>16305.01</v>
       </c>
       <c r="CE20" t="n">
         <v>5.98</v>
@@ -24922,16 +24922,16 @@
         <v>14</v>
       </c>
       <c r="CH20" t="n">
-        <v>16476.27</v>
+        <v>16459.36</v>
       </c>
       <c r="CI20" t="n">
-        <v>5.92</v>
+        <v>5.81</v>
       </c>
       <c r="CJ20" t="n">
-        <v>4.27</v>
+        <v>3.84</v>
       </c>
       <c r="CK20" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="21">
@@ -25201,16 +25201,16 @@
         <v>14</v>
       </c>
       <c r="CH21" t="n">
-        <v>7991.58</v>
+        <v>7996.06</v>
       </c>
       <c r="CI21" t="n">
-        <v>7.36</v>
+        <v>7.42</v>
       </c>
       <c r="CJ21" t="n">
-        <v>6.23</v>
+        <v>6.47</v>
       </c>
       <c r="CK21" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="22">
@@ -25480,16 +25480,16 @@
         <v>14</v>
       </c>
       <c r="CH22" t="n">
-        <v>1615.89</v>
+        <v>1615.7</v>
       </c>
       <c r="CI22" t="n">
-        <v>11.16</v>
+        <v>11.15</v>
       </c>
       <c r="CJ22" t="n">
-        <v>11.1</v>
+        <v>11.04</v>
       </c>
       <c r="CK22" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="23">
@@ -25759,16 +25759,16 @@
         <v>14</v>
       </c>
       <c r="CH23" t="n">
-        <v>917.08</v>
+        <v>915.23</v>
       </c>
       <c r="CI23" t="n">
-        <v>3.3</v>
+        <v>3.09</v>
       </c>
       <c r="CJ23" t="n">
-        <v>5.12</v>
+        <v>4.28</v>
       </c>
       <c r="CK23" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="24">
@@ -26038,16 +26038,16 @@
         <v>14</v>
       </c>
       <c r="CH24" t="n">
-        <v>125.61</v>
+        <v>125.79</v>
       </c>
       <c r="CI24" t="n">
-        <v>-1.26</v>
+        <v>-1.12</v>
       </c>
       <c r="CJ24" t="n">
-        <v>4.01</v>
+        <v>4.61</v>
       </c>
       <c r="CK24" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="25">
@@ -26320,13 +26320,13 @@
         <v>6.25</v>
       </c>
       <c r="CI25" t="n">
-        <v>-2.3</v>
+        <v>-2.29</v>
       </c>
       <c r="CJ25" t="n">
-        <v>-1.86</v>
+        <v>-1.85</v>
       </c>
       <c r="CK25" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="26">
@@ -26596,16 +26596,16 @@
         <v>14</v>
       </c>
       <c r="CH26" t="n">
-        <v>254.97</v>
+        <v>254.14</v>
       </c>
       <c r="CI26" t="n">
-        <v>5.79</v>
+        <v>5.45</v>
       </c>
       <c r="CJ26" t="n">
-        <v>6.62</v>
+        <v>5.25</v>
       </c>
       <c r="CK26" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="27">
@@ -26875,16 +26875,16 @@
         <v>14</v>
       </c>
       <c r="CH27" t="n">
-        <v>530.25</v>
+        <v>529.04</v>
       </c>
       <c r="CI27" t="n">
-        <v>3.33</v>
+        <v>3.09</v>
       </c>
       <c r="CJ27" t="n">
-        <v>4.76</v>
+        <v>3.81</v>
       </c>
       <c r="CK27" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="28">
@@ -27154,16 +27154,16 @@
         <v>14</v>
       </c>
       <c r="CH28" t="n">
-        <v>1656.95</v>
+        <v>1659.91</v>
       </c>
       <c r="CI28" t="n">
-        <v>-0.02</v>
+        <v>0.16</v>
       </c>
       <c r="CJ28" t="n">
-        <v>-0.68</v>
+        <v>0.03</v>
       </c>
       <c r="CK28" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="29">
@@ -27433,16 +27433,16 @@
         <v>14</v>
       </c>
       <c r="CH29" t="n">
-        <v>1495.46</v>
+        <v>1498.34</v>
       </c>
       <c r="CI29" t="n">
-        <v>-0.27</v>
+        <v>-0.08</v>
       </c>
       <c r="CJ29" t="n">
-        <v>-0.99</v>
+        <v>-0.22</v>
       </c>
       <c r="CK29" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="30">
@@ -27712,16 +27712,16 @@
         <v>14</v>
       </c>
       <c r="CH30" t="n">
-        <v>161.49</v>
+        <v>161.57</v>
       </c>
       <c r="CI30" t="n">
-        <v>2.44</v>
+        <v>2.49</v>
       </c>
       <c r="CJ30" t="n">
-        <v>2.25</v>
+        <v>2.45</v>
       </c>
       <c r="CK30" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="31">
@@ -27991,16 +27991,16 @@
         <v>14</v>
       </c>
       <c r="CH31" t="n">
-        <v>1583.94</v>
+        <v>1584.26</v>
       </c>
       <c r="CI31" t="n">
-        <v>3.33</v>
+        <v>3.35</v>
       </c>
       <c r="CJ31" t="n">
-        <v>0.71</v>
+        <v>0.79</v>
       </c>
       <c r="CK31" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="32">
@@ -28270,16 +28270,16 @@
         <v>14</v>
       </c>
       <c r="CH32" t="n">
-        <v>1001.35</v>
+        <v>1002.05</v>
       </c>
       <c r="CI32" t="n">
-        <v>4.14</v>
+        <v>4.21</v>
       </c>
       <c r="CJ32" t="n">
-        <v>2.62</v>
+        <v>2.91</v>
       </c>
       <c r="CK32" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="33">
@@ -28549,16 +28549,16 @@
         <v>14</v>
       </c>
       <c r="CH33" t="n">
-        <v>582.59</v>
+        <v>582.21</v>
       </c>
       <c r="CI33" t="n">
-        <v>1.96</v>
+        <v>1.9</v>
       </c>
       <c r="CJ33" t="n">
-        <v>-2.48</v>
+        <v>-2.74</v>
       </c>
       <c r="CK33" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="34">
@@ -28828,16 +28828,16 @@
         <v>14</v>
       </c>
       <c r="CH34" t="n">
-        <v>436.23</v>
+        <v>436.16</v>
       </c>
       <c r="CI34" t="n">
-        <v>2.95</v>
+        <v>2.93</v>
       </c>
       <c r="CJ34" t="n">
-        <v>-2.07</v>
+        <v>-2.13</v>
       </c>
       <c r="CK34" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="35">
@@ -29107,16 +29107,16 @@
         <v>14</v>
       </c>
       <c r="CH35" t="n">
-        <v>2217.72</v>
+        <v>2220.97</v>
       </c>
       <c r="CI35" t="n">
-        <v>16</v>
+        <v>16.17</v>
       </c>
       <c r="CJ35" t="n">
-        <v>12.96</v>
+        <v>13.62</v>
       </c>
       <c r="CK35" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="36">
@@ -29386,16 +29386,16 @@
         <v>14</v>
       </c>
       <c r="CH36" t="n">
-        <v>1361.24</v>
+        <v>1366.83</v>
       </c>
       <c r="CI36" t="n">
-        <v>19.17</v>
+        <v>19.66</v>
       </c>
       <c r="CJ36" t="n">
-        <v>16.15</v>
+        <v>18.06</v>
       </c>
       <c r="CK36" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="37">
@@ -29665,16 +29665,16 @@
         <v>14</v>
       </c>
       <c r="CH37" t="n">
-        <v>12453.63</v>
+        <v>12448.7</v>
       </c>
       <c r="CI37" t="n">
-        <v>6.89</v>
+        <v>6.85</v>
       </c>
       <c r="CJ37" t="n">
-        <v>5.96</v>
+        <v>5.79</v>
       </c>
       <c r="CK37" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="38">
@@ -29932,28 +29932,28 @@
         <v>13</v>
       </c>
       <c r="CD38" t="n">
-        <v>897.17</v>
+        <v>897.21</v>
       </c>
       <c r="CE38" t="n">
         <v>11.23</v>
       </c>
       <c r="CF38" t="n">
-        <v>-1.36</v>
+        <v>-1.35</v>
       </c>
       <c r="CG38" t="n">
         <v>14</v>
       </c>
       <c r="CH38" t="n">
-        <v>922.95</v>
+        <v>930.9400000000001</v>
       </c>
       <c r="CI38" t="n">
-        <v>11.71</v>
+        <v>12.67</v>
       </c>
       <c r="CJ38" t="n">
-        <v>12</v>
+        <v>15.91</v>
       </c>
       <c r="CK38" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="39">
@@ -30211,7 +30211,7 @@
         <v>13</v>
       </c>
       <c r="CD39" t="n">
-        <v>11377.62</v>
+        <v>11377.58</v>
       </c>
       <c r="CE39" t="n">
         <v>6.3</v>
@@ -30223,16 +30223,16 @@
         <v>14</v>
       </c>
       <c r="CH39" t="n">
-        <v>11530.68</v>
+        <v>11517.75</v>
       </c>
       <c r="CI39" t="n">
-        <v>6.52</v>
+        <v>6.4</v>
       </c>
       <c r="CJ39" t="n">
-        <v>5.49</v>
+        <v>5.02</v>
       </c>
       <c r="CK39" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="40">
@@ -30490,28 +30490,28 @@
         <v>13</v>
       </c>
       <c r="CD40" t="n">
-        <v>4722.8</v>
+        <v>4723.01</v>
       </c>
       <c r="CE40" t="n">
         <v>5.39</v>
       </c>
       <c r="CF40" t="n">
-        <v>5.72</v>
+        <v>5.74</v>
       </c>
       <c r="CG40" t="n">
         <v>14</v>
       </c>
       <c r="CH40" t="n">
-        <v>4771.49</v>
+        <v>4762.94</v>
       </c>
       <c r="CI40" t="n">
-        <v>5.14</v>
+        <v>4.95</v>
       </c>
       <c r="CJ40" t="n">
-        <v>4.19</v>
+        <v>3.42</v>
       </c>
       <c r="CK40" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="41">
@@ -30775,22 +30775,22 @@
         <v>5.06</v>
       </c>
       <c r="CF41" t="n">
-        <v>8.07</v>
+        <v>8.08</v>
       </c>
       <c r="CG41" t="n">
         <v>14</v>
       </c>
       <c r="CH41" t="n">
-        <v>742.12</v>
+        <v>741.6900000000001</v>
       </c>
       <c r="CI41" t="n">
-        <v>5.76</v>
+        <v>5.7</v>
       </c>
       <c r="CJ41" t="n">
-        <v>4.85</v>
+        <v>4.6</v>
       </c>
       <c r="CK41" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="42">
@@ -31048,28 +31048,28 @@
         <v>13</v>
       </c>
       <c r="CD42" t="n">
-        <v>2098.77</v>
+        <v>2098.82</v>
       </c>
       <c r="CE42" t="n">
         <v>3.52</v>
       </c>
       <c r="CF42" t="n">
-        <v>3.59</v>
+        <v>3.6</v>
       </c>
       <c r="CG42" t="n">
         <v>14</v>
       </c>
       <c r="CH42" t="n">
-        <v>2115.55</v>
+        <v>2114.69</v>
       </c>
       <c r="CI42" t="n">
-        <v>3.47</v>
+        <v>3.42</v>
       </c>
       <c r="CJ42" t="n">
-        <v>3.24</v>
+        <v>3.06</v>
       </c>
       <c r="CK42" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="43">
@@ -31327,28 +31327,28 @@
         <v>13</v>
       </c>
       <c r="CD43" t="n">
-        <v>307.32</v>
+        <v>307.29</v>
       </c>
       <c r="CE43" t="n">
-        <v>-1.17</v>
+        <v>-1.18</v>
       </c>
       <c r="CF43" t="n">
-        <v>3.77</v>
+        <v>3.73</v>
       </c>
       <c r="CG43" t="n">
         <v>14</v>
       </c>
       <c r="CH43" t="n">
-        <v>310.16</v>
+        <v>309.87</v>
       </c>
       <c r="CI43" t="n">
-        <v>0.73</v>
+        <v>0.64</v>
       </c>
       <c r="CJ43" t="n">
-        <v>3.76</v>
+        <v>3.4</v>
       </c>
       <c r="CK43" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="44">
@@ -31606,13 +31606,13 @@
         <v>13</v>
       </c>
       <c r="CD44" t="n">
-        <v>116.26</v>
+        <v>116.3</v>
       </c>
       <c r="CE44" t="n">
-        <v>4.7</v>
+        <v>4.74</v>
       </c>
       <c r="CF44" t="n">
-        <v>4.8</v>
+        <v>4.95</v>
       </c>
       <c r="CG44" t="n">
         <v>14</v>
@@ -31624,10 +31624,10 @@
         <v>4.69</v>
       </c>
       <c r="CJ44" t="n">
-        <v>3.24</v>
+        <v>3.09</v>
       </c>
       <c r="CK44" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="45">
@@ -31885,28 +31885,28 @@
         <v>13</v>
       </c>
       <c r="CD45" t="n">
-        <v>366.15</v>
+        <v>366.2</v>
       </c>
       <c r="CE45" t="n">
-        <v>2.12</v>
+        <v>2.13</v>
       </c>
       <c r="CF45" t="n">
-        <v>0.5600000000000001</v>
+        <v>0.61</v>
       </c>
       <c r="CG45" t="n">
         <v>14</v>
       </c>
       <c r="CH45" t="n">
-        <v>368.53</v>
+        <v>368.79</v>
       </c>
       <c r="CI45" t="n">
-        <v>1.92</v>
+        <v>1.99</v>
       </c>
       <c r="CJ45" t="n">
-        <v>2.62</v>
+        <v>2.87</v>
       </c>
       <c r="CK45" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="46">
@@ -32176,16 +32176,16 @@
         <v>14</v>
       </c>
       <c r="CH46" t="n">
-        <v>1319.67</v>
+        <v>1318.84</v>
       </c>
       <c r="CI46" t="n">
-        <v>4.47</v>
+        <v>4.4</v>
       </c>
       <c r="CJ46" t="n">
-        <v>3.29</v>
+        <v>3.03</v>
       </c>
       <c r="CK46" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="47">
@@ -32443,28 +32443,28 @@
         <v>13</v>
       </c>
       <c r="CD47" t="n">
-        <v>1036.92</v>
+        <v>1036.95</v>
       </c>
       <c r="CE47" t="n">
         <v>3.72</v>
       </c>
       <c r="CF47" t="n">
-        <v>3.44</v>
+        <v>3.46</v>
       </c>
       <c r="CG47" t="n">
         <v>14</v>
       </c>
       <c r="CH47" t="n">
-        <v>1038.78</v>
+        <v>1038.69</v>
       </c>
       <c r="CI47" t="n">
         <v>2.87</v>
       </c>
       <c r="CJ47" t="n">
-        <v>0.72</v>
+        <v>0.67</v>
       </c>
       <c r="CK47" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="48">
@@ -32722,13 +32722,13 @@
         <v>13</v>
       </c>
       <c r="CD48" t="n">
-        <v>908.89</v>
+        <v>908.92</v>
       </c>
       <c r="CE48" t="n">
-        <v>2.74</v>
+        <v>2.75</v>
       </c>
       <c r="CF48" t="n">
-        <v>2.27</v>
+        <v>2.29</v>
       </c>
       <c r="CG48" t="n">
         <v>14</v>
@@ -32740,10 +32740,10 @@
         <v>1.95</v>
       </c>
       <c r="CJ48" t="n">
-        <v>-0.03</v>
+        <v>-0.04</v>
       </c>
       <c r="CK48" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="49">
@@ -33007,22 +33007,22 @@
         <v>11.2</v>
       </c>
       <c r="CF49" t="n">
-        <v>12.29</v>
+        <v>12.3</v>
       </c>
       <c r="CG49" t="n">
         <v>14</v>
       </c>
       <c r="CH49" t="n">
-        <v>129.95</v>
+        <v>129.86</v>
       </c>
       <c r="CI49" t="n">
-        <v>9.83</v>
+        <v>9.75</v>
       </c>
       <c r="CJ49" t="n">
-        <v>6.15</v>
+        <v>5.85</v>
       </c>
       <c r="CK49" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="50">
@@ -33280,28 +33280,28 @@
         <v>13</v>
       </c>
       <c r="CD50" t="n">
-        <v>338.23</v>
+        <v>338.33</v>
       </c>
       <c r="CE50" t="n">
-        <v>8.83</v>
+        <v>8.859999999999999</v>
       </c>
       <c r="CF50" t="n">
-        <v>14.54</v>
+        <v>14.67</v>
       </c>
       <c r="CG50" t="n">
         <v>14</v>
       </c>
       <c r="CH50" t="n">
-        <v>353.11</v>
+        <v>345.77</v>
       </c>
       <c r="CI50" t="n">
-        <v>11.43</v>
+        <v>9.109999999999999</v>
       </c>
       <c r="CJ50" t="n">
-        <v>18.78</v>
+        <v>9.09</v>
       </c>
       <c r="CK50" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="51">
@@ -33559,28 +33559,28 @@
         <v>13</v>
       </c>
       <c r="CD51" t="n">
-        <v>95.26000000000001</v>
+        <v>95.37</v>
       </c>
       <c r="CE51" t="n">
-        <v>-0.06</v>
+        <v>0.05</v>
       </c>
       <c r="CF51" t="n">
-        <v>-4.56</v>
+        <v>-4.14</v>
       </c>
       <c r="CG51" t="n">
         <v>14</v>
       </c>
       <c r="CH51" t="n">
-        <v>103.66</v>
+        <v>96.02</v>
       </c>
       <c r="CI51" t="n">
-        <v>6.59</v>
+        <v>-1.27</v>
       </c>
       <c r="CJ51" t="n">
-        <v>40.2</v>
+        <v>2.76</v>
       </c>
       <c r="CK51" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="52">
@@ -33838,28 +33838,28 @@
         <v>13</v>
       </c>
       <c r="CD52" t="n">
-        <v>242.97</v>
+        <v>242.96</v>
       </c>
       <c r="CE52" t="n">
         <v>12.77</v>
       </c>
       <c r="CF52" t="n">
-        <v>23.31</v>
+        <v>23.3</v>
       </c>
       <c r="CG52" t="n">
         <v>14</v>
       </c>
       <c r="CH52" t="n">
-        <v>249.45</v>
+        <v>249.75</v>
       </c>
       <c r="CI52" t="n">
-        <v>13.57</v>
+        <v>13.71</v>
       </c>
       <c r="CJ52" t="n">
-        <v>11.09</v>
+        <v>11.65</v>
       </c>
       <c r="CK52" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="53">
@@ -34129,16 +34129,16 @@
         <v>14</v>
       </c>
       <c r="CH53" t="n">
-        <v>88.22</v>
+        <v>88.27</v>
       </c>
       <c r="CI53" t="n">
-        <v>14.93</v>
+        <v>14.98</v>
       </c>
       <c r="CJ53" t="n">
-        <v>12.93</v>
+        <v>13.15</v>
       </c>
       <c r="CK53" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="54">
@@ -34396,28 +34396,28 @@
         <v>13</v>
       </c>
       <c r="CD54" t="n">
-        <v>515.5</v>
+        <v>515.51</v>
       </c>
       <c r="CE54" t="n">
-        <v>15.77</v>
+        <v>15.78</v>
       </c>
       <c r="CF54" t="n">
-        <v>10.46</v>
+        <v>10.47</v>
       </c>
       <c r="CG54" t="n">
         <v>14</v>
       </c>
       <c r="CH54" t="n">
-        <v>521.9400000000001</v>
+        <v>522.1</v>
       </c>
       <c r="CI54" t="n">
-        <v>12.15</v>
+        <v>12.19</v>
       </c>
       <c r="CJ54" t="n">
-        <v>5.09</v>
+        <v>5.22</v>
       </c>
       <c r="CK54" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="55">
@@ -34687,16 +34687,16 @@
         <v>14</v>
       </c>
       <c r="CH55" t="n">
-        <v>201.56</v>
+        <v>201.13</v>
       </c>
       <c r="CI55" t="n">
-        <v>17.63</v>
+        <v>17.38</v>
       </c>
       <c r="CJ55" t="n">
-        <v>6.46</v>
+        <v>5.54</v>
       </c>
       <c r="CK55" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="56">
@@ -34966,16 +34966,16 @@
         <v>14</v>
       </c>
       <c r="CH56" t="n">
-        <v>5691.89</v>
+        <v>5685.45</v>
       </c>
       <c r="CI56" t="n">
-        <v>3.92</v>
+        <v>3.81</v>
       </c>
       <c r="CJ56" t="n">
-        <v>2.01</v>
+        <v>1.55</v>
       </c>
       <c r="CK56" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="57">
@@ -35233,28 +35233,28 @@
         <v>13</v>
       </c>
       <c r="CD57" t="n">
-        <v>736.15</v>
+        <v>736.17</v>
       </c>
       <c r="CE57" t="n">
         <v>0.23</v>
       </c>
       <c r="CF57" t="n">
-        <v>0.13</v>
+        <v>0.14</v>
       </c>
       <c r="CG57" t="n">
         <v>14</v>
       </c>
       <c r="CH57" t="n">
-        <v>746.3</v>
+        <v>743.85</v>
       </c>
       <c r="CI57" t="n">
-        <v>0.11</v>
+        <v>-0.22</v>
       </c>
       <c r="CJ57" t="n">
-        <v>5.63</v>
+        <v>4.23</v>
       </c>
       <c r="CK57" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="58">
@@ -35512,7 +35512,7 @@
         <v>13</v>
       </c>
       <c r="CD58" t="n">
-        <v>4927.44</v>
+        <v>4927.42</v>
       </c>
       <c r="CE58" t="n">
         <v>5.25</v>
@@ -35524,16 +35524,16 @@
         <v>14</v>
       </c>
       <c r="CH58" t="n">
-        <v>4945.59</v>
+        <v>4941.6</v>
       </c>
       <c r="CI58" t="n">
-        <v>4.53</v>
+        <v>4.44</v>
       </c>
       <c r="CJ58" t="n">
-        <v>1.48</v>
+        <v>1.16</v>
       </c>
       <c r="CK58" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="60">

</xml_diff>